<commit_message>
calibração 2026-10-27 10:58 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Propostas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$2</definedName>
@@ -720,7 +720,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27 10:57 UTC</t>
+          <t>2026-10-27 10:58 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-27 11:01 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -708,7 +708,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27 10:49 UTC</t>
+          <t>2026-10-27 10:59 UTC</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27 10:58 UTC</t>
+          <t>2026-10-27 11:00 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
OE 2027: reserva pelo portal desativada e sem ligação à página de detalhe (na nova aplicação da AR os identificadores recomeçam em 1 e coincidem com PA de anos anteriores); retirados 2 registos obtidos por essa via (005C era uma PA de 2005)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012uxwqH5ZwUWosxzcs9nhPb
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Propostas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF70"/>
+  <dimension ref="A1:AF68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -729,11 +729,7 @@
       <c r="Z2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=1</t>
-        </is>
-      </c>
+      <c r="AA2" s="2" t="inlineStr"/>
       <c r="AB2" s="2" t="inlineStr">
         <is>
           <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396859574d325a47526d4d533035596a426c4c54526c595755744f5459314e79316b4e6a49305a57466d4e4451774f446b756347526d&amp;Fich=aac6ddf1-9b0e-4eae-9657-d624eaf44089.pdf&amp;Inline=true</t>
@@ -835,11 +831,7 @@
       <c r="Z3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=2</t>
-        </is>
-      </c>
+      <c r="AA3" s="2" t="inlineStr"/>
       <c r="AB3" s="2" t="inlineStr">
         <is>
           <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c5a6a6c6d596a51785969316a4d4467784c54526d4e4445744f47466b5a43307a4e6a51334f544977596d45354d6a49756347526d&amp;Fich=ef9fb41b-c081-4f41-8add-3647920ba922.pdf&amp;Inline=true</t>
@@ -941,11 +933,7 @@
       <c r="Z4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=3</t>
-        </is>
-      </c>
+      <c r="AA4" s="2" t="inlineStr"/>
       <c r="AB4" s="2" t="inlineStr">
         <is>
           <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4e6a4269595755774d793078593245344c545177596a63744f57526c4e69316d5a544d784d574a6a5a5441794d324d756347526d&amp;Fich=c60bae03-1ca8-40b7-9de6-fe311bce023c.pdf&amp;Inline=true</t>
@@ -1047,11 +1035,7 @@
       <c r="Z5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=4</t>
-        </is>
-      </c>
+      <c r="AA5" s="2" t="inlineStr"/>
       <c r="AB5" s="2" t="inlineStr">
         <is>
           <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338304d7a67324f5455304d53316d4d3252684c5451314d6d4974595455344f53307a4e7a4d784d7a55325a44526a4d6a63756347526d&amp;Fich=43869541-f3da-452b-a589-3731356d4c27.pdf&amp;Inline=true</t>
@@ -1153,11 +1137,7 @@
       <c r="Z6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=5</t>
-        </is>
-      </c>
+      <c r="AA6" s="2" t="inlineStr"/>
       <c r="AB6" s="2" t="inlineStr">
         <is>
           <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314f5445334e446c6c59693035593249334c545133596a55744f4451344f43316b4f474d324d446c6c4d7a45344f5463756347526d&amp;Fich=591749eb-9cb7-47b5-8488-d8c609e31897.pdf&amp;Inline=true</t>
@@ -1183,25 +1163,33 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>005C</t>
+          <t>6C</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>005C</t>
+          <t>6C</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="n">
-        <v>75</v>
+        <v>6</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2005-11-17</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+          <t>2026-10-29 09:00</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Comissão</t>
@@ -1217,15 +1205,19 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Emenda</t>
+          <t>Por Definir</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Aditados os pontos 8A, 19A, 19B e 19C ao Quadro III a que se refere o artigo 6.º</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr"/>
+          <t>Artigo 63.º-A (Aditamento à lista I anexa ao Código do Imposto sobre o Valor Acrescentado)</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Agricultura e Pescas</t>
+        </is>
+      </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
           <t>em apreciação</t>
@@ -1233,7 +1225,7 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Substituído(a) (558C)</t>
+          <t>Entrada (via IPA)</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr"/>
@@ -1244,15 +1236,13 @@
       <c r="W7" s="2" t="inlineStr"/>
       <c r="X7" s="2" t="inlineStr"/>
       <c r="Y7" s="2" t="inlineStr"/>
-      <c r="Z7" s="2" t="inlineStr"/>
-      <c r="AA7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=75</t>
-        </is>
-      </c>
+      <c r="Z7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="2" t="inlineStr"/>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?Path=6iWoOT%2fhIHtXXXxCbqC0pRAngBZYiqkMOb%2bGN1gxBgu4%2fBGY2eBJWPWkXHt8771v3vCu%2bTGSrNzgr7jYkkWXHEaeYjU4VMIvk4UePKhlGWtgYMg8DEMUdmV5uCBRMB4nfZ6PpTdTJj7h%2bUvBTSyKA5%2bVFuHfvPgAWydQWmKT4m1GxcaLbOPNFtjubtcwGWCbHdwgi%2bZCSXS9fFVcAtCI61hsiYhjsltP6Rf4z%2bo6Udq9la6VSlTG57xyh6stfD4Nn78VCfg0YDeuFfWKhMOV%2f8Fk6oI51cGZgNbfQfWdKyR%2fvddAIh%2ffqTvIuihLa40lZ41jLsdb3XISUkBH7ZNWPjKHGtqCz1ASLl5G8qAFVuWM1VO44NTJTZ7di%2baZKKsm&amp;Fich=6815f336-c157-477b-8785-f94071bf0d65.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684d6a52684d7a677a5969316b4d6d52684c545130597a6374596a49784d4330335a5749344e7a45304f5441314d7a41756347526d&amp;Fich=a24a383b-d2da-44c7-b210-7eb871490530.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
@@ -1267,7 +1257,7 @@
       </c>
       <c r="AE7" s="2" t="inlineStr">
         <is>
-          <t>scrape</t>
+          <t>opendata</t>
         </is>
       </c>
       <c r="AF7" s="2" t="inlineStr"/>
@@ -1275,17 +1265,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>6C</t>
+          <t>7C</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>6C</t>
+          <t>7C</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -1322,7 +1312,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Artigo 63.º-A (Aditamento à lista I anexa ao Código do Imposto sobre o Valor Acrescentado)</t>
+          <t>Artigo 104.º (Centros de recolha oficial de animais, apoio à esterilização e à promoção do bem-estar animal)</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1351,14 +1341,10 @@
       <c r="Z8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=6</t>
-        </is>
-      </c>
+      <c r="AA8" s="2" t="inlineStr"/>
       <c r="AB8" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684d6a52684d7a677a5969316b4d6d52684c545130597a6374596a49784d4330335a5749344e7a45304f5441314d7a41756347526d&amp;Fich=a24a383b-d2da-44c7-b210-7eb871490530.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684d324e6d4d4445774e53316a5a6a51354c545134596d51744f57466d4f43307959325a6d5a5449314f475135596a45756347526d&amp;Fich=a3cf0105-cf49-48bd-9af8-2cffe258d9b1.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC8" s="2" t="inlineStr">
@@ -1381,21 +1367,21 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>7C</t>
+          <t>8C</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>7C</t>
+          <t>8C</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:00</t>
+          <t>2026-10-29 09:01</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1428,12 +1414,12 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Artigo 104.º (Centros de recolha oficial de animais, apoio à esterilização e à promoção do bem-estar animal)</t>
+          <t>«Artigo 89.º-A Garantia de apoio psicológico nas escolas</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Agricultura e Pescas</t>
+          <t>Educação e Ciência; Saúde</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1457,14 +1443,10 @@
       <c r="Z9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=7</t>
-        </is>
-      </c>
+      <c r="AA9" s="2" t="inlineStr"/>
       <c r="AB9" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684d324e6d4d4445774e53316a5a6a51354c545134596d51744f57466d4f43307959325a6d5a5449314f475135596a45756347526d&amp;Fich=a3cf0105-cf49-48bd-9af8-2cffe258d9b1.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396b5a6a466c4d6d466d4e4330314d7a59324c545178593255744f44677a4d43316a4d6d51795957526c4f4746685a4463756347526d&amp;Fich=df1e2af4-5366-41ce-8830-c2d2ade8aad7.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC9" s="2" t="inlineStr">
@@ -1487,17 +1469,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>8C</t>
+          <t>9C</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>8C</t>
+          <t>9C</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -1534,12 +1516,12 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 89.º-A Garantia de apoio psicológico nas escolas</t>
+          <t>«Artigo 39.º-C Alteração ao Decreto-Lei n.º 28/2004, de 4 de fevereiro PA - 100% BAIXA ONCOLÓGICA</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Saúde</t>
+          <t>Saúde; Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1563,14 +1545,10 @@
       <c r="Z10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=8</t>
-        </is>
-      </c>
+      <c r="AA10" s="2" t="inlineStr"/>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396b5a6a466c4d6d466d4e4330314d7a59324c545178593255744f44677a4d43316a4d6d51795957526c4f4746685a4463756347526d&amp;Fich=df1e2af4-5366-41ce-8830-c2d2ade8aad7.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339685a5455774f44466b4d4330354e5467794c5452694e5467744f4759304d43307a4f444e6a4d4442695a6a566d597a41756347526d&amp;Fich=ae5081d0-9582-4b58-8f40-383c00bf5fc0.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
@@ -1593,17 +1571,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>9C</t>
+          <t>10C</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>9C</t>
+          <t>10C</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -1640,12 +1618,12 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 39.º-C Alteração ao Decreto-Lei n.º 28/2004, de 4 de fevereiro PA - 100% BAIXA ONCOLÓGICA</t>
+          <t>Artigo 63.º-A (Aditamento à lista I anexa ao Código do Imposto sobre o Valor Acrescentado)</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Saúde; Trabalho, Segurança Social e Inclusão</t>
+          <t>Agricultura e Pescas</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1669,14 +1647,10 @@
       <c r="Z11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=9</t>
-        </is>
-      </c>
+      <c r="AA11" s="2" t="inlineStr"/>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339685a5455774f44466b4d4330354e5467794c5452694e5467744f4759304d43307a4f444e6a4d4442695a6a566d597a41756347526d&amp;Fich=ae5081d0-9582-4b58-8f40-383c00bf5fc0.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338305a475a6959546c6a4e69316b4f4459304c5452694d6a6374596a63305a533169596a457a4e4755774e7a67344e7a67756347526d&amp;Fich=4dfba9c6-d864-4b27-b74e-bb134e078878.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
@@ -1699,17 +1673,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11C</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>10C</t>
+          <t>11C</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -1746,12 +1720,12 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Artigo 63.º-A (Aditamento à lista I anexa ao Código do Imposto sobre o Valor Acrescentado)</t>
+          <t>«Artigo 115.º-A Criação do Plano Nacional para o Alojamento no Ensino Superior 2.0</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Agricultura e Pescas</t>
+          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1775,14 +1749,10 @@
       <c r="Z12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=10</t>
-        </is>
-      </c>
+      <c r="AA12" s="2" t="inlineStr"/>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338305a475a6959546c6a4e69316b4f4459304c5452694d6a6374596a63305a533169596a457a4e4755774e7a67344e7a67756347526d&amp;Fich=4dfba9c6-d864-4b27-b74e-bb134e078878.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338795a6a5134596d466c595330334f5452684c5451774f544d744f54466a4d5330334e6a67354e574d344d3259344f4451756347526d&amp;Fich=2f48baea-794a-4093-91c1-76895c83f884.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
@@ -1805,21 +1775,21 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>11C</t>
+          <t>12C</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>11C</t>
+          <t>12C</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:01</t>
+          <t>2026-10-29 09:02</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1852,12 +1822,12 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 115.º-A Criação do Plano Nacional para o Alojamento no Ensino Superior 2.0</t>
+          <t>«Artigo 120.º-A Rede Nacional de Bancos de Leite Materno</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1881,14 +1851,10 @@
       <c r="Z13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA13" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=11</t>
-        </is>
-      </c>
+      <c r="AA13" s="2" t="inlineStr"/>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338795a6a5134596d466c595330334f5452684c5451774f544d744f54466a4d5330334e6a67354e574d344d3259344f4451756347526d&amp;Fich=2f48baea-794a-4093-91c1-76895c83f884.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a5a6d59794f5749324e7930324e5441344c5451784e7a677459546b314e7931684e54566b4f4455344e7a5a6d596a49756347526d&amp;Fich=cff29b67-6508-4178-a957-a55d85876fb2.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
@@ -1911,17 +1877,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>13C</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>13C</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -1958,12 +1924,12 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 120.º-A Rede Nacional de Bancos de Leite Materno</t>
+          <t>Artigo 63.º-B (Aditamento à lista I anexa ao Código do Imposto sobre o Valor Acrescentado)</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Agricultura e Pescas</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1987,14 +1953,10 @@
       <c r="Z14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=12</t>
-        </is>
-      </c>
+      <c r="AA14" s="2" t="inlineStr"/>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a5a6d59794f5749324e7930324e5441344c5451784e7a677459546b314e7931684e54566b4f4455344e7a5a6d596a49756347526d&amp;Fich=cff29b67-6508-4178-a957-a55d85876fb2.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314d5463304f4749304d4330335a6a63774c54526c4d6d55744f54426d5a6931685a44566a5a5749785a475a685a4745756347526d&amp;Fich=51748b40-7f70-4e2e-90ff-ad5ceb1dfada.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC14" s="2" t="inlineStr">
@@ -2017,17 +1979,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>13C</t>
+          <t>14C</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>13C</t>
+          <t>14C</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -2036,12 +1998,12 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>PAN</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Inês de Sousa Real</t>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -2064,12 +2026,12 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Artigo 63.º-B (Aditamento à lista I anexa ao Código do Imposto sobre o Valor Acrescentado)</t>
+          <t>Alarga o abono de família revendo os escalões de rendimento de referência do agregado familiar, pela alteração ao Decreto-Lei n.º 176/2003, de 2 de agosto</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Agricultura e Pescas</t>
+          <t>Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2093,14 +2055,10 @@
       <c r="Z15" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA15" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=13</t>
-        </is>
-      </c>
+      <c r="AA15" s="2" t="inlineStr"/>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314d5463304f4749304d4330335a6a63774c54526c4d6d55744f54426d5a6931685a44566a5a5749785a475a685a4745756347526d&amp;Fich=51748b40-7f70-4e2e-90ff-ad5ceb1dfada.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533968596a51304d5449784e7930314e6a68684c5451785a5441744f57566b5a69316d4d6a55775a444935593255344d446b756347526d&amp;Fich=ab441217-568a-41e0-9edf-f250d29ce809.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
@@ -2123,17 +2081,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>14C</t>
+          <t>15C</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>14C</t>
+          <t>15C</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -2142,12 +2100,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PAN</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+          <t>Inês de Sousa Real</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -2170,12 +2128,12 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Alarga o abono de família revendo os escalões de rendimento de referência do agregado familiar, pela alteração ao Decreto-Lei n.º 176/2003, de 2 de agosto</t>
+          <t>Artigo 125º-A (Programa Nacional de Conservação e Monitorização do Gato-Bravo)</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>Trabalho, Segurança Social e Inclusão</t>
+          <t>Ambiente e Energia</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2199,14 +2157,10 @@
       <c r="Z16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA16" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=14</t>
-        </is>
-      </c>
+      <c r="AA16" s="2" t="inlineStr"/>
       <c r="AB16" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533968596a51304d5449784e7930314e6a68684c5451785a5441744f57566b5a69316d4d6a55775a444935593255344d446b756347526d&amp;Fich=ab441217-568a-41e0-9edf-f250d29ce809.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c5a6a686d4f544d794d53316d4e324d324c54526d596a51744f544d7a4f4330334e6a51314f444d3059544e6b4e5445756347526d&amp;Fich=ef8f9321-f7c6-4fb4-9338-7645834a3d51.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC16" s="2" t="inlineStr">
@@ -2229,17 +2183,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>15C</t>
+          <t>16C</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>15C</t>
+          <t>16C</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -2276,12 +2230,12 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Artigo 125º-A (Programa Nacional de Conservação e Monitorização do Gato-Bravo)</t>
+          <t>Artigo 104.º-A (Centros de recolha oficial de animais, apoio à esterilização e à promoção do bem estar-animal)</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>Ambiente e Energia</t>
+          <t>Agricultura e Pescas</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2305,14 +2259,10 @@
       <c r="Z17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=15</t>
-        </is>
-      </c>
+      <c r="AA17" s="2" t="inlineStr"/>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c5a6a686d4f544d794d53316d4e324d324c54526d596a51744f544d7a4f4330334e6a51314f444d3059544e6b4e5445756347526d&amp;Fich=ef8f9321-f7c6-4fb4-9338-7645834a3d51.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324d5745775a6d4d344d5330305a4759314c545135596a4574596a6c695a53307a597a4e6b4d575535595755775a4759756347526d&amp;Fich=61a0fc81-4df5-49b1-b9be-3c3d1e9ae0df.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
@@ -2335,17 +2285,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>16C</t>
+          <t>17C</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>16C</t>
+          <t>17C</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -2382,7 +2332,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Artigo 104.º-A (Centros de recolha oficial de animais, apoio à esterilização e à promoção do bem estar-animal)</t>
+          <t>Artigo 104.º-C (Criação da linha telefónica nacional de socorro animal)</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -2411,14 +2361,10 @@
       <c r="Z18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=16</t>
-        </is>
-      </c>
+      <c r="AA18" s="2" t="inlineStr"/>
       <c r="AB18" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324d5745775a6d4d344d5330305a4759314c545135596a4574596a6c695a53307a597a4e6b4d575535595755775a4759756347526d&amp;Fich=61a0fc81-4df5-49b1-b9be-3c3d1e9ae0df.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4f575577597a6c684d79303059324d324c54526b4f5467744f474978596930774e5459305a5455304e4456695a4451756347526d&amp;Fich=c9e0c9a3-4cc6-4d98-8b1b-0564e5445bd4.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC18" s="2" t="inlineStr">
@@ -2441,17 +2387,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>17C</t>
+          <t>18C</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>17C</t>
+          <t>18C</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -2488,12 +2434,12 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Artigo 104.º-C (Criação da linha telefónica nacional de socorro animal)</t>
+          <t>«Artigo 115.º-B Residências modulares em instituições de Ensino Superior</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Agricultura e Pescas</t>
+          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2517,14 +2463,10 @@
       <c r="Z19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=17</t>
-        </is>
-      </c>
+      <c r="AA19" s="2" t="inlineStr"/>
       <c r="AB19" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4f575577597a6c684d79303059324d324c54526b4f5467744f474978596930774e5459305a5455304e4456695a4451756347526d&amp;Fich=c9e0c9a3-4cc6-4d98-8b1b-0564e5445bd4.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338775a5446694e6d4a694f4330334e444a684c5451314d7a4574596a41324f5330784f546b7a4f5759794e4755315a5749756347526d&amp;Fich=0e1b6bb8-742a-4531-b069-19939f24e5eb.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC19" s="2" t="inlineStr">
@@ -2547,17 +2489,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>18C</t>
+          <t>19C</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>18C</t>
+          <t>19C</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -2594,12 +2536,12 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 115.º-B Residências modulares em instituições de Ensino Superior</t>
+          <t>«Artigo 122.º-A Criação do passe ‘’Vai e Vem’'</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
+          <t>Infraestruturas, Mobilidade e Habitação; Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2623,14 +2565,10 @@
       <c r="Z20" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=18</t>
-        </is>
-      </c>
+      <c r="AA20" s="2" t="inlineStr"/>
       <c r="AB20" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338775a5446694e6d4a694f4330334e444a684c5451314d7a4574596a41324f5330784f546b7a4f5759794e4755315a5749756347526d&amp;Fich=0e1b6bb8-742a-4531-b069-19939f24e5eb.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339685a474d33595455324d6930334e44526b4c5451344d446b74596d4e694d5331684d4441354f474e6c5a4755344e4445756347526d&amp;Fich=adc7a562-744d-4809-bcb1-a0098cede841.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC20" s="2" t="inlineStr">
@@ -2653,17 +2591,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>19C</t>
+          <t>20C</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>19C</t>
+          <t>20C</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -2729,14 +2667,10 @@
       <c r="Z21" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=19</t>
-        </is>
-      </c>
+      <c r="AA21" s="2" t="inlineStr"/>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339685a474d33595455324d6930334e44526b4c5451344d446b74596d4e694d5331684d4441354f474e6c5a4755344e4445756347526d&amp;Fich=adc7a562-744d-4809-bcb1-a0098cede841.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338334e474e695a474e68596930774e546b344c545133595441745954497a4f5330775a6d5531596a637a4e7a4d355a4751756347526d&amp;Fich=74cbdcab-0598-47a0-a239-0fe5b73739dd.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
@@ -2759,31 +2693,31 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>20C</t>
+          <t>21C</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>20C</t>
+          <t>21C</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:02</t>
+          <t>2026-10-29 09:04</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>PAN</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Inês de Sousa Real</t>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2806,12 +2740,12 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 122.º-A Criação do passe ‘’Vai e Vem’'</t>
+          <t>[NOVO] Artigo 60.º-A - Imposto Mínimo sobre Grandes Fortunas</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Infraestruturas, Mobilidade e Habitação; Orçamento, Finanças e Administração Pública</t>
+          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2835,14 +2769,10 @@
       <c r="Z22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=20</t>
-        </is>
-      </c>
+      <c r="AA22" s="2" t="inlineStr"/>
       <c r="AB22" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338334e474e695a474e68596930774e546b344c545133595441745954497a4f5330775a6d5531596a637a4e7a4d355a4751756347526d&amp;Fich=74cbdcab-0598-47a0-a239-0fe5b73739dd.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a5a4749324f4755334f4330354d57457a4c5451774d324d744f474d344d53316d4d6a49345a546b794f4455304f5745756347526d&amp;Fich=cdb68e78-91a3-403c-8c81-f228e928549a.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC22" s="2" t="inlineStr">
@@ -2865,17 +2795,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>21C</t>
+          <t>22C</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>21C</t>
+          <t>22C</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
@@ -2884,12 +2814,12 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PAN</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+          <t>Inês de Sousa Real</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2912,12 +2842,12 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 60.º-A - Imposto Mínimo sobre Grandes Fortunas</t>
+          <t>Artigo 64.º (Eliminação gradual das isenções prejudiciais em matéria de produtos petrolíferos e energéticos)</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
+          <t>Ambiente e Energia</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -2941,14 +2871,10 @@
       <c r="Z23" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=21</t>
-        </is>
-      </c>
+      <c r="AA23" s="2" t="inlineStr"/>
       <c r="AB23" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a5a4749324f4755334f4330354d57457a4c5451774d324d744f474d344d53316d4d6a49345a546b794f4455304f5745756347526d&amp;Fich=cdb68e78-91a3-403c-8c81-f228e928549a.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324d5455774f44466d4f5330334e446b344c5452694e7a6b744f54457a4f53307a4d5745335a6a4d31595759774e3255756347526d&amp;Fich=615081f9-7498-4b79-9139-31a7f35af07e.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC23" s="2" t="inlineStr">
@@ -2971,21 +2897,21 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>22C</t>
+          <t>23C</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>22C</t>
+          <t>23C</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:04</t>
+          <t>2026-10-29 09:05</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -3018,12 +2944,12 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Artigo 64.º (Eliminação gradual das isenções prejudiciais em matéria de produtos petrolíferos e energéticos)</t>
+          <t>«Artigo 122.º-A Criação do passe ‘’Vai e Vem’'</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Ambiente e Energia</t>
+          <t>Infraestruturas, Mobilidade e Habitação; Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3047,14 +2973,10 @@
       <c r="Z24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=22</t>
-        </is>
-      </c>
+      <c r="AA24" s="2" t="inlineStr"/>
       <c r="AB24" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324d5455774f44466d4f5330334e446b344c5452694e7a6b744f54457a4f53307a4d5745335a6a4d31595759774e3255756347526d&amp;Fich=615081f9-7498-4b79-9139-31a7f35af07e.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339694d7a6379596d45345953316c593249794c54526d5a6a5574596a67315a69307a4e4459354f5759774d4452684e4755756347526d&amp;Fich=b372ba8a-ecb2-4ff5-b85f-34699f004a4e.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC24" s="2" t="inlineStr">
@@ -3077,17 +2999,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>23C</t>
+          <t>24C</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>23C</t>
+          <t>24C</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -3124,12 +3046,12 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 122.º-A Criação do passe ‘’Vai e Vem’'</t>
+          <t>«Artigo 89.º-A Garantia de apoio psicológico nas escolas</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Infraestruturas, Mobilidade e Habitação; Orçamento, Finanças e Administração Pública</t>
+          <t>Educação e Ciência; Saúde</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3153,14 +3075,10 @@
       <c r="Z25" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=23</t>
-        </is>
-      </c>
+      <c r="AA25" s="2" t="inlineStr"/>
       <c r="AB25" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339694d7a6379596d45345953316c593249794c54526d5a6a5574596a67315a69307a4e4459354f5759774d4452684e4755756347526d&amp;Fich=b372ba8a-ecb2-4ff5-b85f-34699f004a4e.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314f5463355a6d45334d53316b4d7a49794c5451794d6a59744f4451324e5331684d6d45774f5449795a5441324f446b756347526d&amp;Fich=5979fa71-d322-4226-8465-a2a0922e0689.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC25" s="2" t="inlineStr">
@@ -3183,17 +3101,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>24C</t>
+          <t>25C</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>24C</t>
+          <t>25C</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -3230,12 +3148,12 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 89.º-A Garantia de apoio psicológico nas escolas</t>
+          <t>«Artigo 39.º-C Alteração ao Decreto-Lei n.º 28/2004, de 4 de fevereiro PA - 100% BAIXA ONCOLÓGICA</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Saúde</t>
+          <t>Saúde; Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3259,14 +3177,10 @@
       <c r="Z26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=24</t>
-        </is>
-      </c>
+      <c r="AA26" s="2" t="inlineStr"/>
       <c r="AB26" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314f5463355a6d45334d53316b4d7a49794c5451794d6a59744f4451324e5331684d6d45774f5449795a5441324f446b756347526d&amp;Fich=5979fa71-d322-4226-8465-a2a0922e0689.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d595755344d544131595330314f4745774c5451784f4455744f446b33597931694e7a417a4d6a4934596d55794e4759756347526d&amp;Fich=fae8105a-58a0-4185-897c-b703228be24f.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC26" s="2" t="inlineStr">
@@ -3289,21 +3203,21 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>25C</t>
+          <t>26C</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>25C</t>
+          <t>26C</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:05</t>
+          <t>2026-10-29 09:06</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -3336,12 +3250,12 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 39.º-C Alteração ao Decreto-Lei n.º 28/2004, de 4 de fevereiro PA - 100% BAIXA ONCOLÓGICA</t>
+          <t>«Artigo 115.º-B Residências modulares em instituições de Ensino Superior</t>
         </is>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Saúde; Trabalho, Segurança Social e Inclusão</t>
+          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3365,14 +3279,10 @@
       <c r="Z27" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=25</t>
-        </is>
-      </c>
+      <c r="AA27" s="2" t="inlineStr"/>
       <c r="AB27" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d595755344d544131595330314f4745774c5451784f4455744f446b33597931694e7a417a4d6a4934596d55794e4759756347526d&amp;Fich=fae8105a-58a0-4185-897c-b703228be24f.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338774f5456694e7a55775a69316c4e3251794c54526b5a446b7459574e6d4e5330314e7a646a5a546330596a41324e7a63756347526d&amp;Fich=095b750f-e7d2-4dd9-acf5-577ce74b0677.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC27" s="2" t="inlineStr">
@@ -3395,17 +3305,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>26C</t>
+          <t>27C</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>26C</t>
+          <t>27C</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -3442,12 +3352,12 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 115.º-B Residências modulares em instituições de Ensino Superior</t>
+          <t>«Artigo 120.º-A Rede Nacional de Bancos de Leite Materno</t>
         </is>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3471,14 +3381,10 @@
       <c r="Z28" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=26</t>
-        </is>
-      </c>
+      <c r="AA28" s="2" t="inlineStr"/>
       <c r="AB28" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338774f5456694e7a55775a69316c4e3251794c54526b5a446b7459574e6d4e5330314e7a646a5a546330596a41324e7a63756347526d&amp;Fich=095b750f-e7d2-4dd9-acf5-577ce74b0677.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4d7a6378597a457859793078596d51304c54526c4f5451744f57457a5a4330794d446c684e475932596a566c4d4459756347526d&amp;Fich=3371c11c-1bd4-4e94-9a3d-209a4f6b5e06.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC28" s="2" t="inlineStr">
@@ -3501,17 +3407,17 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>27C</t>
+          <t>28C</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>27C</t>
+          <t>28C</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -3520,12 +3426,12 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>PAN</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Inês de Sousa Real</t>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -3548,12 +3454,12 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 120.º-A Rede Nacional de Bancos de Leite Materno</t>
+          <t>Aumento da majoração para as famílias monoparentais do Abono de Família</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3577,14 +3483,10 @@
       <c r="Z29" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=27</t>
-        </is>
-      </c>
+      <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4d7a6378597a457859793078596d51304c54526c4f5451744f57457a5a4330794d446c684e475932596a566c4d4459756347526d&amp;Fich=3371c11c-1bd4-4e94-9a3d-209a4f6b5e06.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d545534597a41344e6930775a6a457a4c545178595745744f57593359533034593249304d4445314d54426d5a4455756347526d&amp;Fich=8158c086-0f13-41aa-9f7a-8cb401510fd5.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC29" s="2" t="inlineStr">
@@ -3607,17 +3509,17 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>28C</t>
+          <t>29C</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>28C</t>
+          <t>29C</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -3626,12 +3528,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PAN</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+          <t>Inês de Sousa Real</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -3654,12 +3556,12 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>Aumento da majoração para as famílias monoparentais do Abono de Família</t>
+          <t>«Artigo 115.º-B Residências modulares em instituições de Ensino Superior</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>Trabalho, Segurança Social e Inclusão</t>
+          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -3683,14 +3585,10 @@
       <c r="Z30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=28</t>
-        </is>
-      </c>
+      <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d545534597a41344e6930775a6a457a4c545178595745744f57593359533034593249304d4445314d54426d5a4455756347526d&amp;Fich=8158c086-0f13-41aa-9f7a-8cb401510fd5.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4e6d45314d6d51304e4330304d7a4a694c5452684e7a6b74596d55774d4331694d4445334d47466b5a54426c4e5759756347526d&amp;Fich=e6a52d44-432b-4a79-be00-b0170ade0e5f.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC30" s="2" t="inlineStr">
@@ -3713,31 +3611,31 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>29C</t>
+          <t>30C</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>29C</t>
+          <t>30C</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:06</t>
+          <t>2026-10-29 09:07</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>PAN</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Inês de Sousa Real</t>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3760,12 +3658,12 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 115.º-B Residências modulares em instituições de Ensino Superior</t>
+          <t>[NOVO] Artigo 19.º-A - Programa “Semana de quatro dias de trabalho na Administração Pública”</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
+          <t>Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -3789,14 +3687,10 @@
       <c r="Z31" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=29</t>
-        </is>
-      </c>
+      <c r="AA31" s="2" t="inlineStr"/>
       <c r="AB31" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4e6d45314d6d51304e4330304d7a4a694c5452684e7a6b74596d55774d4331694d4445334d47466b5a54426c4e5759756347526d&amp;Fich=e6a52d44-432b-4a79-be00-b0170ade0e5f.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4d4452694e6a4a6c4d4331694d32597a4c54526a4e446b74596a517a596930784f5456684d7a55784f5751795a6a59756347526d&amp;Fich=304b62e0-b3f3-4c49-b43b-195a3519d2f6.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC31" s="2" t="inlineStr">
@@ -3819,17 +3713,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>30C</t>
+          <t>31C</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>30C</t>
+          <t>31C</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
@@ -3838,12 +3732,12 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PAN</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+          <t>Inês de Sousa Real</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -3866,12 +3760,12 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 19.º-A - Programa “Semana de quatro dias de trabalho na Administração Pública”</t>
+          <t>«Artigo 115.º-A Criação do Plano Nacional para o Alojamento no Ensino Superior 2.0</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>Orçamento, Finanças e Administração Pública</t>
+          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -3895,14 +3789,10 @@
       <c r="Z32" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=30</t>
-        </is>
-      </c>
+      <c r="AA32" s="2" t="inlineStr"/>
       <c r="AB32" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4d4452694e6a4a6c4d4331694d32597a4c54526a4e446b74596a517a596930784f5456684d7a55784f5751795a6a59756347526d&amp;Fich=304b62e0-b3f3-4c49-b43b-195a3519d2f6.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d44466b4f544d795969316d4f4759314c5452694e4759744f445a6a5a4330774e444133597a526b4d574d335a544d756347526d&amp;Fich=801d932b-f8f5-4b4f-86cd-0407c4d1c7e3.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC32" s="2" t="inlineStr">
@@ -3925,17 +3815,17 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>31C</t>
+          <t>32C</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>31C</t>
+          <t>32C</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr"/>
       <c r="D33" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
@@ -4001,14 +3891,10 @@
       <c r="Z33" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=31</t>
-        </is>
-      </c>
+      <c r="AA33" s="2" t="inlineStr"/>
       <c r="AB33" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d44466b4f544d795969316d4f4759314c5452694e4759744f445a6a5a4330774e444133597a526b4d574d335a544d756347526d&amp;Fich=801d932b-f8f5-4b4f-86cd-0407c4d1c7e3.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338304e6a4e685a4745354d5330774d6d55784c5451774e4759744f575a68596930345a545a6a5a4467305a5455334f4755756347526d&amp;Fich=463ada91-02e1-404f-9fab-8e6cd84e578e.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC33" s="2" t="inlineStr">
@@ -4031,21 +3917,21 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>32C</t>
+          <t>33C</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>32C</t>
+          <t>33C</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:07</t>
+          <t>2026-10-29 09:08</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -4078,12 +3964,12 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 115.º-A Criação do Plano Nacional para o Alojamento no Ensino Superior 2.0</t>
+          <t>«Artigo 89.º-A Garantia de apoio psicológico nas escolas</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Infraestruturas, Mobilidade e Habitação</t>
+          <t>Educação e Ciência; Saúde</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -4107,14 +3993,10 @@
       <c r="Z34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=32</t>
-        </is>
-      </c>
+      <c r="AA34" s="2" t="inlineStr"/>
       <c r="AB34" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338304e6a4e685a4745354d5330774d6d55784c5451774e4759744f575a68596930345a545a6a5a4467305a5455334f4755756347526d&amp;Fich=463ada91-02e1-404f-9fab-8e6cd84e578e.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338335a6a45324e446b784d5331684e3249344c54526b595745744f44646b597930775a4455775a5451344d7a49324e3251756347526d&amp;Fich=7f164911-a7b8-4daa-87dc-0d50e483267d.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC34" s="2" t="inlineStr">
@@ -4137,31 +4019,31 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>33C</t>
+          <t>34C</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>33C</t>
+          <t>34C</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:08</t>
+          <t>2026-10-29 09:09</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>PAN</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Inês de Sousa Real</t>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -4184,12 +4066,12 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 89.º-A Garantia de apoio psicológico nas escolas</t>
+          <t>[NOVO] Artigo 4.º-A - Cria o Serviço Nacional de Habitação</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Saúde</t>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -4213,14 +4095,10 @@
       <c r="Z35" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=33</t>
-        </is>
-      </c>
+      <c r="AA35" s="2" t="inlineStr"/>
       <c r="AB35" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338335a6a45324e446b784d5331684e3249344c54526b595745744f44646b597930775a4455775a5451344d7a49324e3251756347526d&amp;Fich=7f164911-a7b8-4daa-87dc-0d50e483267d.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c59574a6d4e574d774d4330334d6a566c4c54526b4d446b74596a59314e53316b4e325178597a4e694e7a56695a5749756347526d&amp;Fich=eabf5c00-725e-4d09-b655-d7d1c3b75beb.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC35" s="2" t="inlineStr">
@@ -4243,17 +4121,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>34C</t>
+          <t>35C</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>34C</t>
+          <t>35C</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
@@ -4290,12 +4168,12 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 4.º-A - Cria o Serviço Nacional de Habitação</t>
+          <t>[NOVO] Artigo 45.º-A Aumento do valor do Abono de Família em 10%</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>Infraestruturas, Mobilidade e Habitação</t>
+          <t>Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -4319,14 +4197,10 @@
       <c r="Z36" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=34</t>
-        </is>
-      </c>
+      <c r="AA36" s="2" t="inlineStr"/>
       <c r="AB36" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c59574a6d4e574d774d4330334d6a566c4c54526b4d446b74596a59314e53316b4e325178597a4e694e7a56695a5749756347526d&amp;Fich=eabf5c00-725e-4d09-b655-d7d1c3b75beb.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a5a4467784e6a6b784d7930344d6d51784c5451304f4451744f54526a4d4330324e32466b4d6a63314e4459324f5459756347526d&amp;Fich=cd816913-82d1-4484-94c0-67ad27546696.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC36" s="2" t="inlineStr">
@@ -4349,17 +4223,17 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>35C</t>
+          <t>36C</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>35C</t>
+          <t>36C</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr"/>
       <c r="D37" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
@@ -4396,12 +4270,12 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 45.º-A Aumento do valor do Abono de Família em 10%</t>
+          <t>Limitação das propinas no ensino superior público</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>Trabalho, Segurança Social e Inclusão</t>
+          <t>Educação e Ciência</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4425,14 +4299,10 @@
       <c r="Z37" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA37" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=35</t>
-        </is>
-      </c>
+      <c r="AA37" s="2" t="inlineStr"/>
       <c r="AB37" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a5a4467784e6a6b784d7930344d6d51784c5451304f4451744f54526a4d4330324e32466b4d6a63314e4459324f5459756347526d&amp;Fich=cd816913-82d1-4484-94c0-67ad27546696.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396b596a4d354d5459794e5330775a6a4d7a4c54517959546b74595746684d4330345a54646a4d3251334f54426a4d3251756347526d&amp;Fich=db391625-0f33-42a9-aaa0-8e7c3d790c3d.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC37" s="2" t="inlineStr">
@@ -4455,17 +4325,17 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>36C</t>
+          <t>37C</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>36C</t>
+          <t>37C</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
@@ -4502,12 +4372,12 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>Limitação das propinas no ensino superior público</t>
+          <t>[NOVO] Artigo 110.º-A - Retoma e alarga o Projeto-piloto da semana de quatro dias de trabalho no setor privado</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência</t>
+          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -4531,14 +4401,10 @@
       <c r="Z38" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=36</t>
-        </is>
-      </c>
+      <c r="AA38" s="2" t="inlineStr"/>
       <c r="AB38" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396b596a4d354d5459794e5330775a6a4d7a4c54517959546b74595746684d4330345a54646a4d3251334f54426a4d3251756347526d&amp;Fich=db391625-0f33-42a9-aaa0-8e7c3d790c3d.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338304e5441354d7a45775a43307a4f54466d4c54526a596d49744f44597a5a6930794f444e6c5a5459794e7a55304f5459756347526d&amp;Fich=4509310d-391f-4cbb-863f-283ee6275496.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC38" s="2" t="inlineStr">
@@ -4561,21 +4427,21 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>37C</t>
+          <t>38C</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>37C</t>
+          <t>38C</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:09</t>
+          <t>2026-10-29 09:11</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -4608,12 +4474,12 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 110.º-A - Retoma e alarga o Projeto-piloto da semana de quatro dias de trabalho no setor privado</t>
+          <t>Alteração ao Código do Imposto sobre o Valor Acrescentado</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
+          <t>Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -4637,14 +4503,10 @@
       <c r="Z39" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA39" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=37</t>
-        </is>
-      </c>
+      <c r="AA39" s="2" t="inlineStr"/>
       <c r="AB39" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338304e5441354d7a45775a43307a4f54466d4c54526a596d49744f44597a5a6930794f444e6c5a5459794e7a55304f5459756347526d&amp;Fich=4509310d-391f-4cbb-863f-283ee6275496.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4f5759794d47466c5a5330305a5467774c5451794d4751744f4449794e69316b4d444d334e5445335a474d784d6a63756347526d&amp;Fich=39f20aee-4e80-420d-8226-d037517dc127.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC39" s="2" t="inlineStr">
@@ -4667,21 +4529,21 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>38C</t>
+          <t>39C</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>38C</t>
+          <t>39C</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:11</t>
+          <t>2026-10-29 09:12</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -4714,12 +4576,12 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>Alteração ao Código do Imposto sobre o Valor Acrescentado</t>
+          <t>[NOVO] Artigo 64.º-A - Redução faseada da taxa de IVA</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Orçamento, Finanças e Administração Pública</t>
+          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -4743,14 +4605,10 @@
       <c r="Z40" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=38</t>
-        </is>
-      </c>
+      <c r="AA40" s="2" t="inlineStr"/>
       <c r="AB40" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4f5759794d47466c5a5330305a5467774c5451794d4751744f4449794e69316b4d444d334e5445335a474d784d6a63756347526d&amp;Fich=39f20aee-4e80-420d-8226-d037517dc127.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4f574e684f4451335a5331695a6d4e694c5451344d5459744f4455354e4330304d44526c5a545a685954466c4e6d59756347526d&amp;Fich=c9ca847e-bfcb-4816-8594-404ee6aa1e6f.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC40" s="2" t="inlineStr">
@@ -4773,17 +4631,17 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>39C</t>
+          <t>40C</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>39C</t>
+          <t>40C</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
@@ -4820,12 +4678,12 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 64.º-A - Redução faseada da taxa de IVA</t>
+          <t>[NOVO] Artigo 21.º - A Reforça o recrutamento de médicos e enfermeiros especialistas com vista à reabertura das urgências de ginecologia e obstetrícia encerradas</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
+          <t>Saúde; Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
@@ -4849,14 +4707,10 @@
       <c r="Z41" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA41" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=39</t>
-        </is>
-      </c>
+      <c r="AA41" s="2" t="inlineStr"/>
       <c r="AB41" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4f574e684f4451335a5331695a6d4e694c5451344d5459744f4455354e4330304d44526c5a545a685954466c4e6d59756347526d&amp;Fich=c9ca847e-bfcb-4816-8594-404ee6aa1e6f.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4d6d4978596d49795a69307a59544a684c54517a4d545574596a4a6d4e7930334d544d784e7a5a694d5745774e5463756347526d&amp;Fich=f2b1bb2f-3a2a-4315-b2f7-713176b1a057.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC41" s="2" t="inlineStr">
@@ -4879,17 +4733,17 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>40C</t>
+          <t>41C</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>40C</t>
+          <t>41C</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr"/>
       <c r="D42" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
@@ -4926,12 +4780,12 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 21.º - A Reforça o recrutamento de médicos e enfermeiros especialistas com vista à reabertura das urgências de ginecologia e obstetrícia encerradas</t>
+          <t>[NOVO] Artigo 4.º-A - Cria o Fundo para a Habitação Pública</t>
         </is>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>Saúde; Trabalho, Segurança Social e Inclusão</t>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -4955,14 +4809,10 @@
       <c r="Z42" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=40</t>
-        </is>
-      </c>
+      <c r="AA42" s="2" t="inlineStr"/>
       <c r="AB42" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4d6d4978596d49795a69307a59544a684c54517a4d545574596a4a6d4e7930334d544d784e7a5a694d5745774e5463756347526d&amp;Fich=f2b1bb2f-3a2a-4315-b2f7-713176b1a057.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4e6a4a6c4d5755334d69316d4d6d4a684c54526b4e7a4574596a45344e5330794e324d314d6a52694d4463325a4459756347526d&amp;Fich=f62e1e72-f2ba-4d71-b185-27c524b076d6.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC42" s="2" t="inlineStr">
@@ -4985,21 +4835,21 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>41C</t>
+          <t>42C</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>41C</t>
+          <t>42C</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:12</t>
+          <t>2026-10-29 09:13</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -5032,12 +4882,12 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 4.º-A - Cria o Fundo para a Habitação Pública</t>
+          <t>Acompanhamento e fiscalização do IVA</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>Infraestruturas, Mobilidade e Habitação</t>
+          <t>Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -5061,14 +4911,10 @@
       <c r="Z43" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA43" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=41</t>
-        </is>
-      </c>
+      <c r="AA43" s="2" t="inlineStr"/>
       <c r="AB43" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4e6a4a6c4d5755334d69316d4d6d4a684c54526b4e7a4574596a45344e5330794e324d314d6a52694d4463325a4459756347526d&amp;Fich=f62e1e72-f2ba-4d71-b185-27c524b076d6.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338794d3251784d54497a4f5331684d324a6b4c54517a4d7a6b74596a56685a6930305a6a6b794f574d354e6a466b5a5749756347526d&amp;Fich=23d11239-a3bd-4339-b5af-4f929c961deb.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC43" s="2" t="inlineStr">
@@ -5091,31 +4937,31 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>42C</t>
+          <t>43C</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>42C</t>
+          <t>43C</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:13</t>
+          <t>2026-10-29 09:14</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PAN</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+          <t>Inês de Sousa Real</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -5138,12 +4984,12 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>Acompanhamento e fiscalização do IVA</t>
+          <t>«Artigo 21.º-A Contratação de psicólogos para instituições de Ensino Superior</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>Orçamento, Finanças e Administração Pública</t>
+          <t>Educação e Ciência; Saúde</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5167,14 +5013,10 @@
       <c r="Z44" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA44" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=42</t>
-        </is>
-      </c>
+      <c r="AA44" s="2" t="inlineStr"/>
       <c r="AB44" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338794d3251784d54497a4f5331684d324a6b4c54517a4d7a6b74596a56685a6930305a6a6b794f574d354e6a466b5a5749756347526d&amp;Fich=23d11239-a3bd-4339-b5af-4f929c961deb.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684e546b7a4e6a5668597930345932517a4c54517859545574596d49785a693031597a41794e7a4d774e6d45354e444d756347526d&amp;Fich=a59365ac-8cd3-41a5-bb1f-5c027306a943.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC44" s="2" t="inlineStr">
@@ -5197,17 +5039,17 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>43C</t>
+          <t>44C</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>43C</t>
+          <t>44C</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
@@ -5216,12 +5058,12 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>PAN</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Inês de Sousa Real</t>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -5244,12 +5086,12 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 21.º-A Contratação de psicólogos para instituições de Ensino Superior</t>
+          <t>[NOVO] Artigo 118.° - A Reposição do orçamento para a promoção da saúde e prevenção da doença</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Saúde</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -5273,14 +5115,10 @@
       <c r="Z45" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA45" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=43</t>
-        </is>
-      </c>
+      <c r="AA45" s="2" t="inlineStr"/>
       <c r="AB45" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684e546b7a4e6a5668597930345932517a4c54517859545574596d49785a693031597a41794e7a4d774e6d45354e444d756347526d&amp;Fich=a59365ac-8cd3-41a5-bb1f-5c027306a943.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4d6a4930597a49314e6930774f546b324c5451774d4449744f5459335a433078593259345a4745794d4467344e474d756347526d&amp;Fich=3224c256-0996-4002-967d-1cf8da20884c.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC45" s="2" t="inlineStr">
@@ -5303,17 +5141,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>44C</t>
+          <t>45C</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>44C</t>
+          <t>45C</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
@@ -5350,12 +5188,12 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 118.° - A Reposição do orçamento para a promoção da saúde e prevenção da doença</t>
+          <t>[NOVO] Artigo 122.º-A - Passe de Mobilidade Nacional</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -5379,14 +5217,10 @@
       <c r="Z46" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA46" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=44</t>
-        </is>
-      </c>
+      <c r="AA46" s="2" t="inlineStr"/>
       <c r="AB46" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4d6a4930597a49314e6930774f546b324c5451774d4449744f5459335a433078593259345a4745794d4467344e474d756347526d&amp;Fich=3224c256-0996-4002-967d-1cf8da20884c.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314e44426d4d5467334d4331684f54646b4c5451304d7a4574595441344e693034596a6c695a546c6d597a466d4e5445756347526d&amp;Fich=540f1870-a97d-4431-a086-8b9be9fc1f51.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC46" s="2" t="inlineStr">
@@ -5409,21 +5243,21 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>45C</t>
+          <t>46C</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>45C</t>
+          <t>46C</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:14</t>
+          <t>2026-10-29 09:15</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -5456,7 +5290,7 @@
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 122.º-A - Passe de Mobilidade Nacional</t>
+          <t>[NOVO] Artigo 122.º-A - Reforço do Fundo para a Mobilidade e Transportes</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
@@ -5485,14 +5319,10 @@
       <c r="Z47" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA47" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=45</t>
-        </is>
-      </c>
+      <c r="AA47" s="2" t="inlineStr"/>
       <c r="AB47" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314e44426d4d5467334d4331684f54646b4c5451304d7a4574595441344e693034596a6c695a546c6d597a466d4e5445756347526d&amp;Fich=540f1870-a97d-4431-a086-8b9be9fc1f51.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4f54646c4e574a6c596931684e6a41784c5451325a6a45744f574d345a5330324e44686c597a566a4d7a51304d5459756347526d&amp;Fich=c97e5beb-a601-46f1-9c8e-648ec5c34416.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC47" s="2" t="inlineStr">
@@ -5515,17 +5345,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>46C</t>
+          <t>47C</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>46C</t>
+          <t>47C</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
@@ -5562,12 +5392,12 @@
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 122.º-A - Reforço do Fundo para a Mobilidade e Transportes</t>
+          <t>Reforço do Programa Incentiva +TP</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>Infraestruturas, Mobilidade e Habitação</t>
+          <t>Economia e Coesão Territorial; Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -5591,14 +5421,10 @@
       <c r="Z48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA48" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=46</t>
-        </is>
-      </c>
+      <c r="AA48" s="2" t="inlineStr"/>
       <c r="AB48" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4f54646c4e574a6c596931684e6a41784c5451325a6a45744f574d345a5330324e44686c597a566a4d7a51304d5459756347526d&amp;Fich=c97e5beb-a601-46f1-9c8e-648ec5c34416.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338794e3251314e6a51784e69316a595745334c54517a4d7a45744f545a6a5a43303559574d31597a6731596d4d77596d59756347526d&amp;Fich=27d56416-caa7-4331-96cd-9ac5c85bc0bf.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC48" s="2" t="inlineStr">
@@ -5621,21 +5447,21 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>47C</t>
+          <t>48C</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>47C</t>
+          <t>48C</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr"/>
       <c r="D49" s="2" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:15</t>
+          <t>2026-10-29 09:21</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -5668,12 +5494,12 @@
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>Reforço do Programa Incentiva +TP</t>
+          <t>[NOVO] Artigo 117.º-A - Estratégia Nacional para a Recuperação e Reciclagem de Minerais Críticos 2050</t>
         </is>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>Economia e Coesão Territorial; Infraestruturas, Mobilidade e Habitação</t>
+          <t>Ambiente e Energia; Economia e Coesão Territorial</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
@@ -5697,14 +5523,10 @@
       <c r="Z49" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA49" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=47</t>
-        </is>
-      </c>
+      <c r="AA49" s="2" t="inlineStr"/>
       <c r="AB49" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338794e3251314e6a51784e69316a595745334c54517a4d7a45744f545a6a5a43303559574d31597a6731596d4d77596d59756347526d&amp;Fich=27d56416-caa7-4331-96cd-9ac5c85bc0bf.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338354d6d45314e574a6a4e693030595467324c5451774e5745744f54526c5a6931695a6a67354e544d324e6a5133595455756347526d&amp;Fich=92a55bc6-4a86-405a-94ef-bf89536647a5.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC49" s="2" t="inlineStr">
@@ -5727,17 +5549,17 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>48C</t>
+          <t>49C</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>48C</t>
+          <t>49C</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
@@ -5774,12 +5596,12 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 117.º-A - Estratégia Nacional para a Recuperação e Reciclagem de Minerais Críticos 2050</t>
+          <t>Descida de impostos sobre os rendimentos do trabalho para toda a classe trabalhadora - Alteração ao Código do Imposto sobre o Rendimento das Pessoas Singulares - Artigo 60.º</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>Ambiente e Energia; Economia e Coesão Territorial</t>
+          <t>Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -5803,14 +5625,10 @@
       <c r="Z50" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA50" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=48</t>
-        </is>
-      </c>
+      <c r="AA50" s="2" t="inlineStr"/>
       <c r="AB50" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338354d6d45314e574a6a4e693030595467324c5451774e5745744f54526c5a6931695a6a67354e544d324e6a5133595455756347526d&amp;Fich=92a55bc6-4a86-405a-94ef-bf89536647a5.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533879595751344e6a457a4e69316c59574d784c545178595455744f444d334e69307a4e44526b4d324a6959545a6c595467756347526d&amp;Fich=2ad86136-eac1-41a5-8376-344d3bba6ea8.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC50" s="2" t="inlineStr">
@@ -5833,21 +5651,21 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>49C</t>
+          <t>50C</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>49C</t>
+          <t>50C</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:21</t>
+          <t>2026-10-29 09:25</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -5880,12 +5698,12 @@
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>Descida de impostos sobre os rendimentos do trabalho para toda a classe trabalhadora - Alteração ao Código do Imposto sobre o Rendimento das Pessoas Singulares - Artigo 60.º</t>
+          <t>[NOVO] Artigo 45.º-A Clarifica o conceito de agregado familiar monoparental para atribuição da majoração do abono de família, alterando o Decreto-Lei n.º 176/2003, de 2 de agosto</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>Orçamento, Finanças e Administração Pública</t>
+          <t>Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr">
@@ -5909,14 +5727,10 @@
       <c r="Z51" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA51" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=49</t>
-        </is>
-      </c>
+      <c r="AA51" s="2" t="inlineStr"/>
       <c r="AB51" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533879595751344e6a457a4e69316c59574d784c545178595455744f444d334e69307a4e44526b4d324a6959545a6c595467756347526d&amp;Fich=2ad86136-eac1-41a5-8376-344d3bba6ea8.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d5a5468694d324d314d7930344e6d46684c54526b4e6d45744f44426b5a53307a4f5463334d7a686b4e5456694d4455756347526d&amp;Fich=fe8b3c53-86aa-4d6a-80de-397738d55b05.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC51" s="2" t="inlineStr">
@@ -5939,17 +5753,17 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>50C</t>
+          <t>51C</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>50C</t>
+          <t>51C</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
@@ -5986,12 +5800,12 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 45.º-A Clarifica o conceito de agregado familiar monoparental para atribuição da majoração do abono de família, alterando o Decreto-Lei n.º 176/2003, de 2 de agosto</t>
+          <t>Majora a dedução das despesas gerais familiares para as famílias monoparentais - Artigo 45.º - A</t>
         </is>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>Trabalho, Segurança Social e Inclusão</t>
+          <t>Orçamento, Finanças e Administração Pública; Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -6015,14 +5829,10 @@
       <c r="Z52" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA52" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=50</t>
-        </is>
-      </c>
+      <c r="AA52" s="2" t="inlineStr"/>
       <c r="AB52" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d5a5468694d324d314d7930344e6d46684c54526b4e6d45744f44426b5a53307a4f5463334d7a686b4e5456694d4455756347526d&amp;Fich=fe8b3c53-86aa-4d6a-80de-397738d55b05.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314e5451774d6a6b334e4330305a6a45324c5452684d7a55744f574d334d793031593255335a6a513359545a6d5a4441756347526d&amp;Fich=55402974-4f16-4a35-9c73-5ce7f47a6fd0.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC52" s="2" t="inlineStr">
@@ -6045,17 +5855,17 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>51C</t>
+          <t>52C</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>51C</t>
+          <t>52C</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
@@ -6092,12 +5902,12 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>Majora a dedução das despesas gerais familiares para as famílias monoparentais - Artigo 45.º - A</t>
+          <t>[NOVO] Artigo 125.º-A - Rede de refúgios climáticos</t>
         </is>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>Orçamento, Finanças e Administração Pública; Trabalho, Segurança Social e Inclusão</t>
+          <t>Ambiente e Energia</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -6121,14 +5931,10 @@
       <c r="Z53" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA53" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=51</t>
-        </is>
-      </c>
+      <c r="AA53" s="2" t="inlineStr"/>
       <c r="AB53" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314e5451774d6a6b334e4330305a6a45324c5452684d7a55744f574d334d793031593255335a6a513359545a6d5a4441756347526d&amp;Fich=55402974-4f16-4a35-9c73-5ce7f47a6fd0.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339695a6a51314e7a51324d6930784f446c6c4c54517a4e5441744f57466c4d533168596a686d5a6d59774e4751794d3249756347526d&amp;Fich=bf457462-189e-4350-9ae1-ab8fff04d23b.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC53" s="2" t="inlineStr">
@@ -6151,21 +5957,21 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>52C</t>
+          <t>53C</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>52C</t>
+          <t>53C</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:25</t>
+          <t>2026-10-29 09:29</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -6198,12 +6004,12 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 125.º-A - Rede de refúgios climáticos</t>
+          <t>[NOVO] Artigo 125º-A - Rede Nacional de Cafés Reparação</t>
         </is>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>Ambiente e Energia</t>
+          <t>Ambiente e Energia; Economia e Coesão Territorial</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -6227,14 +6033,10 @@
       <c r="Z54" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=52</t>
-        </is>
-      </c>
+      <c r="AA54" s="2" t="inlineStr"/>
       <c r="AB54" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339695a6a51314e7a51324d6930784f446c6c4c54517a4e5441744f57466c4d533168596a686d5a6d59774e4751794d3249756347526d&amp;Fich=bf457462-189e-4350-9ae1-ab8fff04d23b.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338775a6d59775a44566c4e43316d5a6d4e6b4c5452694d544d744f5467345a4330334e4449344d6d4534595463304d3255756347526d&amp;Fich=0ff0d5e4-ffcd-4b13-988d-74282a8a743e.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC54" s="2" t="inlineStr">
@@ -6257,21 +6059,21 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>53C</t>
+          <t>54C</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>53C</t>
+          <t>54C</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:29</t>
+          <t>2026-10-29 09:37</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -6304,12 +6106,12 @@
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 125º-A - Rede Nacional de Cafés Reparação</t>
+          <t>[NOVO] Artigo 110.º-A - Retoma e alargamento do Programa 3C - Casa, Conforto e Clima</t>
         </is>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>Ambiente e Energia; Economia e Coesão Territorial</t>
+          <t>Ambiente e Energia; Economia e Coesão Territorial; Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -6333,14 +6135,10 @@
       <c r="Z55" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA55" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=53</t>
-        </is>
-      </c>
+      <c r="AA55" s="2" t="inlineStr"/>
       <c r="AB55" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338775a6d59775a44566c4e43316d5a6d4e6b4c5452694d544d744f5467345a4330334e4449344d6d4534595463304d3255756347526d&amp;Fich=0ff0d5e4-ffcd-4b13-988d-74282a8a743e.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338784f4451324f444e6a4d79316b5a57517a4c54526b4f5455744f446333596930325a446b78593246685a6a55324e4455756347526d&amp;Fich=184683c3-ded3-4d95-877b-6d91caaf5645.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC55" s="2" t="inlineStr">
@@ -6363,17 +6161,17 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>54C</t>
+          <t>55C</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>54C</t>
+          <t>55C</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr"/>
       <c r="D56" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
@@ -6410,12 +6208,12 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 110.º-A - Retoma e alargamento do Programa 3C - Casa, Conforto e Clima</t>
+          <t>Aumento da remuneração base do salário base dos quatro primeiros escalões dos Docentes da educação pré-escolar e dos ensinos básico e secundário - Artigo 21.º A</t>
         </is>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>Ambiente e Energia; Economia e Coesão Territorial; Infraestruturas, Mobilidade e Habitação</t>
+          <t>Educação e Ciência; Orçamento, Finanças e Administração Pública; Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P56" s="2" t="inlineStr">
@@ -6439,14 +6237,10 @@
       <c r="Z56" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA56" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=54</t>
-        </is>
-      </c>
+      <c r="AA56" s="2" t="inlineStr"/>
       <c r="AB56" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338784f4451324f444e6a4d79316b5a57517a4c54526b4f5455744f446333596930325a446b78593246685a6a55324e4455756347526d&amp;Fich=184683c3-ded3-4d95-877b-6d91caaf5645.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4e4755324d4445314d4330344e44417a4c5451324e54517459544a6a4f433032596d4d314e7a417a4e544e6b4f5463756347526d&amp;Fich=c4e60150-8403-4654-a2c8-6bc570353d97.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC56" s="2" t="inlineStr">
@@ -6469,21 +6263,21 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>55C</t>
+          <t>56C</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>55C</t>
+          <t>56C</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr"/>
       <c r="D57" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:37</t>
+          <t>2026-10-29 09:38</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -6516,12 +6310,12 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>Aumento da remuneração base do salário base dos quatro primeiros escalões dos Docentes da educação pré-escolar e dos ensinos básico e secundário - Artigo 21.º A</t>
+          <t>[NOVO] Artigo 62º-A - Alteração ao Código do Imposto sobre o Rendimento das Pessoas Coletivas - Elimina a redução de IRC para as grandes empresas</t>
         </is>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>Educação e Ciência; Orçamento, Finanças e Administração Pública; Trabalho, Segurança Social e Inclusão</t>
+          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P57" s="2" t="inlineStr">
@@ -6545,14 +6339,10 @@
       <c r="Z57" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=55</t>
-        </is>
-      </c>
+      <c r="AA57" s="2" t="inlineStr"/>
       <c r="AB57" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4e4755324d4445314d4330344e44417a4c5451324e54517459544a6a4f433032596d4d314e7a417a4e544e6b4f5463756347526d&amp;Fich=c4e60150-8403-4654-a2c8-6bc570353d97.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396b4d6a686b4e7a5930597930794d5759794c5451314d5459744f4445794e43303159545a6d5a57517759574e685a4467756347526d&amp;Fich=d28d764c-21f2-4516-8124-5a6fed0acad8.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC57" s="2" t="inlineStr">
@@ -6575,31 +6365,31 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>56C</t>
+          <t>57C</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>56C</t>
+          <t>57C</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:38</t>
+          <t>2026-10-29 09:39</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>PAN</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+          <t>Inês de Sousa Real</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -6609,7 +6399,7 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Articulado</t>
+          <t>Mapas</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
@@ -6622,12 +6412,12 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 62º-A - Alteração ao Código do Imposto sobre o Rendimento das Pessoas Coletivas - Elimina a redução de IRC para as grandes empresas</t>
+          <t>Artigo 39.º-C (Alteração ao Decreto-Lei n.º 28/2004, de 4 de fevereiro)</t>
         </is>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
+          <t>Saúde; Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P58" s="2" t="inlineStr">
@@ -6651,14 +6441,10 @@
       <c r="Z58" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA58" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=56</t>
-        </is>
-      </c>
+      <c r="AA58" s="2" t="inlineStr"/>
       <c r="AB58" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396b4d6a686b4e7a5930597930794d5759794c5451314d5459744f4445794e43303159545a6d5a57517759574e685a4467756347526d&amp;Fich=d28d764c-21f2-4516-8124-5a6fed0acad8.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533830596d51324e54426d595330354e7a63784c5451774d7a49744f574a6c5a693078596a6b344e444d314d7a63305a6a59756347526d&amp;Fich=4bd650fa-9771-4032-9bef-1b98435374f6.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC58" s="2" t="inlineStr">
@@ -6681,21 +6467,21 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>57C</t>
+          <t>58C</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>57C</t>
+          <t>58C</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:39</t>
+          <t>2026-10-29 09:41</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -6728,12 +6514,12 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>Artigo 39.º-C (Alteração ao Decreto-Lei n.º 28/2004, de 4 de fevereiro)</t>
+          <t>Anexo I Mapa de alterações e transferências orçamentais (a que se refere o artigo 7.º) Diversas alterações e transferências 130</t>
         </is>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>Saúde; Trabalho, Segurança Social e Inclusão</t>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
         </is>
       </c>
       <c r="P59" s="2" t="inlineStr">
@@ -6757,14 +6543,10 @@
       <c r="Z59" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA59" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=57</t>
-        </is>
-      </c>
+      <c r="AA59" s="2" t="inlineStr"/>
       <c r="AB59" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533830596d51324e54426d595330354e7a63784c5451774d7a49744f574a6c5a693078596a6b344e444d314d7a63305a6a59756347526d&amp;Fich=4bd650fa-9771-4032-9bef-1b98435374f6.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314f575978596a51314e4331685a574a684c545177595449744f57497a4d6930354d6a557a596d59795954497a5a4455756347526d&amp;Fich=59f1b454-aeba-40a2-9b32-9253bf2a23d5.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC59" s="2" t="inlineStr">
@@ -6787,21 +6569,21 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>58C</t>
+          <t>59C</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>58C</t>
+          <t>59C</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:41</t>
+          <t>2026-10-29 09:43</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -6821,7 +6603,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Mapas</t>
+          <t>Articulado</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
@@ -6834,12 +6616,12 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>Anexo I Mapa de alterações e transferências orçamentais (a que se refere o artigo 7.º) Diversas alterações e transferências 130</t>
+          <t>Artigo 60.º</t>
         </is>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P60" s="2" t="inlineStr">
@@ -6863,14 +6645,10 @@
       <c r="Z60" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA60" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=58</t>
-        </is>
-      </c>
+      <c r="AA60" s="2" t="inlineStr"/>
       <c r="AB60" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314f575978596a51314e4331685a574a684c545177595449744f57497a4d6930354d6a557a596d59795954497a5a4455756347526d&amp;Fich=59f1b454-aeba-40a2-9b32-9253bf2a23d5.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4d6d51344f54466d4e5331694e546b344c545130595445744f475131595330324e7a55344e3245324e4445315a444d756347526d&amp;Fich=f2d891f5-b598-44a1-8d5a-67587a6415d3.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC60" s="2" t="inlineStr">
@@ -6893,31 +6671,31 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>59C</t>
+          <t>60C</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>59C</t>
+          <t>60C</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="2" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:43</t>
+          <t>2026-10-29 09:46</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>PAN</t>
+          <t>L</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Inês de Sousa Real</t>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -6940,12 +6718,12 @@
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>Artigo 60.º</t>
+          <t>[NOVO] Artigo 125.º-A - Plano de Ação para a Conservação da Natureza e Biodiversidade 2030</t>
         </is>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>Infraestruturas, Mobilidade e Habitação</t>
+          <t>Ambiente e Energia</t>
         </is>
       </c>
       <c r="P61" s="2" t="inlineStr">
@@ -6969,14 +6747,10 @@
       <c r="Z61" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA61" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=59</t>
-        </is>
-      </c>
+      <c r="AA61" s="2" t="inlineStr"/>
       <c r="AB61" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4d6d51344f54466d4e5331694e546b344c545130595445744f475131595330324e7a55344e3245324e4445315a444d756347526d&amp;Fich=f2d891f5-b598-44a1-8d5a-67587a6415d3.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533834595749354f4441344e433032595755314c5451774e546374596a426b4e7930785954417a5a4755344d324d315a4455756347526d&amp;Fich=8ab98084-6ae5-4057-b0d7-1a03de83c5d5.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC61" s="2" t="inlineStr">
@@ -6999,21 +6773,21 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>60C</t>
+          <t>61C</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>60C</t>
+          <t>61C</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="2" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:46</t>
+          <t>2026-10-29 09:48</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -7046,12 +6820,12 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 125.º-A - Plano de Ação para a Conservação da Natureza e Biodiversidade 2030</t>
+          <t>Tributa em sede de IRS o saldo líquido obtido em jogos e apostas online - Artigo 60.º</t>
         </is>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>Ambiente e Energia</t>
+          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
@@ -7075,14 +6849,10 @@
       <c r="Z62" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA62" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=60</t>
-        </is>
-      </c>
+      <c r="AA62" s="2" t="inlineStr"/>
       <c r="AB62" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533834595749354f4441344e433032595755314c5451774e546374596a426b4e7930785954417a5a4755344d324d315a4455756347526d&amp;Fich=8ab98084-6ae5-4057-b0d7-1a03de83c5d5.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314e5441335a6a6c6d4e7930315954526d4c5451324d474d74596d5130597930304d324d7a4e7a41774e3245774f5751756347526d&amp;Fich=5507f9f7-5a4f-460c-bd4c-43c37007a09d.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC62" s="2" t="inlineStr">
@@ -7105,21 +6875,21 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>61C</t>
+          <t>62C</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>61C</t>
+          <t>62C</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:48</t>
+          <t>2026-10-29 09:49</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -7152,12 +6922,12 @@
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>Tributa em sede de IRS o saldo líquido obtido em jogos e apostas online - Artigo 60.º</t>
+          <t>[NOVO] Artigo 19.º - A - Aditamento ao Decreto-Lei n.º 89/2009, de 9 de abril - Permite que ambos os pais acompanhem a criança com doença oncológica, sem perda financeira, sempre que medicamente recomendado</t>
         </is>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>Economia e Coesão Territorial; Orçamento, Finanças e Administração Pública</t>
+          <t>Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P63" s="2" t="inlineStr">
@@ -7181,14 +6951,10 @@
       <c r="Z63" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA63" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=61</t>
-        </is>
-      </c>
+      <c r="AA63" s="2" t="inlineStr"/>
       <c r="AB63" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314e5441335a6a6c6d4e7930315954526d4c5451324d474d74596d5130597930304d324d7a4e7a41774e3245774f5751756347526d&amp;Fich=5507f9f7-5a4f-460c-bd4c-43c37007a09d.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4e474d774d7a59784d5330344d5464694c54526a4d6d59744f4755314f53316b4f446b344e325132596d4a6d4e4451756347526d&amp;Fich=c4c03611-817b-4c2f-8e59-d8987d6bbf44.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC63" s="2" t="inlineStr">
@@ -7211,21 +6977,21 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>62C</t>
+          <t>63C</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>62C</t>
+          <t>63C</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:49</t>
+          <t>2026-10-29 09:54</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -7258,12 +7024,12 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 19.º - A - Aditamento ao Decreto-Lei n.º 89/2009, de 9 de abril - Permite que ambos os pais acompanhem a criança com doença oncológica, sem perda financeira, sempre que medicamente recomendado</t>
+          <t>Continuidade e Financiamento das Equipas Comunitárias de Saúde Mental - Artigo 22.º - A</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>Trabalho, Segurança Social e Inclusão</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="P64" s="2" t="inlineStr">
@@ -7287,14 +7053,10 @@
       <c r="Z64" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA64" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=62</t>
-        </is>
-      </c>
+      <c r="AA64" s="2" t="inlineStr"/>
       <c r="AB64" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4e474d774d7a59784d5330344d5464694c54526a4d6d59744f4755314f53316b4f446b344e325132596d4a6d4e4451756347526d&amp;Fich=c4c03611-817b-4c2f-8e59-d8987d6bbf44.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4d324e6d596a55774f5330314d6a46684c5451334d325974595759354f4331695a6a42685a6a4e69596a557a5a6d49756347526d&amp;Fich=c3cfb509-521a-473f-af98-bf0af3bb53fb.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC64" s="2" t="inlineStr">
@@ -7317,17 +7079,17 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>63C</t>
+          <t>64C</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>63C</t>
+          <t>64C</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
@@ -7364,12 +7126,12 @@
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>Continuidade e Financiamento das Equipas Comunitárias de Saúde Mental - Artigo 22.º - A</t>
+          <t>[NOVO] Artigo 62.º - A - Alteração ao Código do Imposto sobre o Valor Acrescentado (Retira a isenção do IVA aos artistas tauromáquicos)</t>
         </is>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Agricultura e Pescas; Orçamento, Finanças e Administração Pública</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">
@@ -7393,14 +7155,10 @@
       <c r="Z65" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA65" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=63</t>
-        </is>
-      </c>
+      <c r="AA65" s="2" t="inlineStr"/>
       <c r="AB65" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a4d324e6d596a55774f5330314d6a46684c5451334d325974595759354f4331695a6a42685a6a4e69596a557a5a6d49756347526d&amp;Fich=c3cfb509-521a-473f-af98-bf0af3bb53fb.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4f545a6d4f474e6d4f433034596d4d334c545177597a49744f446c69595330785a5745794e47457a4e6d4d784d3245756347526d&amp;Fich=f96f8cf8-8bc7-40c2-89ba-1ea24a36c13a.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC65" s="2" t="inlineStr">
@@ -7423,21 +7181,21 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>64C</t>
+          <t>65C</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>64C</t>
+          <t>65C</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:54</t>
+          <t>2026-10-29 09:57</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -7470,12 +7228,12 @@
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 62.º - A - Alteração ao Código do Imposto sobre o Valor Acrescentado (Retira a isenção do IVA aos artistas tauromáquicos)</t>
+          <t>[NOVO] Artigo 6.º-A - Proteção das pessoas em vulnerabilidade habitacional e risco de despejo</t>
         </is>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>Agricultura e Pescas; Orçamento, Finanças e Administração Pública</t>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
         </is>
       </c>
       <c r="P66" s="2" t="inlineStr">
@@ -7499,14 +7257,10 @@
       <c r="Z66" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA66" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=64</t>
-        </is>
-      </c>
+      <c r="AA66" s="2" t="inlineStr"/>
       <c r="AB66" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4f545a6d4f474e6d4f433034596d4d334c545177597a49744f446c69595330785a5745794e47457a4e6d4d784d3245756347526d&amp;Fich=f96f8cf8-8bc7-40c2-89ba-1ea24a36c13a.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338354e544931595451345a69316c4e324d774c5452694d5467744f5459305979316c4d6d557a5a6a41334d474e6d4e7a45756347526d&amp;Fich=9525a48f-e7c0-4b18-964c-e2e3f070cf71.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC66" s="2" t="inlineStr">
@@ -7529,21 +7283,21 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>65C</t>
+          <t>66C</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>65C</t>
+          <t>66C</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="2" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 09:57</t>
+          <t>2026-10-29 09:59</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -7576,7 +7330,7 @@
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 6.º-A - Proteção das pessoas em vulnerabilidade habitacional e risco de despejo</t>
+          <t>[NOVO] Artigo 110.º-A - Aumenta o período de apoio do Porta 65 - jovem</t>
         </is>
       </c>
       <c r="O67" s="2" t="inlineStr">
@@ -7605,14 +7359,10 @@
       <c r="Z67" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA67" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=65</t>
-        </is>
-      </c>
+      <c r="AA67" s="2" t="inlineStr"/>
       <c r="AB67" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338354e544931595451345a69316c4e324d774c5452694d5467744f5459305979316c4d6d557a5a6a41334d474e6d4e7a45756347526d&amp;Fich=9525a48f-e7c0-4b18-964c-e2e3f070cf71.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338774e44677a4f5451355a6930784e6d517a4c54526d4e544574595749304e433077595455325a57517a596a4a6a5a6d45756347526d&amp;Fich=0483949f-16d3-4f51-ab44-0a56ed3b2cfa.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC67" s="2" t="inlineStr">
@@ -7635,17 +7385,17 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>66C</t>
+          <t>67C</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>66C</t>
+          <t>67C</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
@@ -7682,12 +7432,12 @@
       </c>
       <c r="N68" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 110.º-A - Aumenta o período de apoio do Porta 65 - jovem</t>
+          <t>[NOVO] Artigo 19.º - A - Aditamento ao Decreto-Lei n.º 89/2009, de 9 de abril - Alarga os direitos parentais em caso de doença ou acidente da criança</t>
         </is>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>Infraestruturas, Mobilidade e Habitação</t>
+          <t>Orçamento, Finanças e Administração Pública; Trabalho, Segurança Social e Inclusão</t>
         </is>
       </c>
       <c r="P68" s="2" t="inlineStr">
@@ -7711,14 +7461,10 @@
       <c r="Z68" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA68" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=66</t>
-        </is>
-      </c>
+      <c r="AA68" s="2" t="inlineStr"/>
       <c r="AB68" s="2" t="inlineStr">
         <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338774e44677a4f5451355a6930784e6d517a4c54526d4e544574595749304e433077595455325a57517a596a4a6a5a6d45756347526d&amp;Fich=0483949f-16d3-4f51-ab44-0a56ed3b2cfa.pdf&amp;Inline=true</t>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533834596d5a6b5a6a67774f5330314e6a5a694c545133596d5574596a67334d53316c4f4746694e5455775a6a55354e3259756347526d&amp;Fich=8bfdf809-566b-47be-b871-e8ab550f597f.pdf&amp;Inline=true</t>
         </is>
       </c>
       <c r="AC68" s="2" t="inlineStr">
@@ -7738,222 +7484,8 @@
       </c>
       <c r="AF68" s="2" t="inlineStr"/>
     </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>67C</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>67C</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr"/>
-      <c r="D69" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-29 09:59</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>Comissão</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>Articulado</t>
-        </is>
-      </c>
-      <c r="J69" s="2" t="inlineStr"/>
-      <c r="K69" s="2" t="inlineStr"/>
-      <c r="L69" s="2" t="inlineStr"/>
-      <c r="M69" s="2" t="inlineStr">
-        <is>
-          <t>Por Definir</t>
-        </is>
-      </c>
-      <c r="N69" s="2" t="inlineStr">
-        <is>
-          <t>[NOVO] Artigo 19.º - A - Aditamento ao Decreto-Lei n.º 89/2009, de 9 de abril - Alarga os direitos parentais em caso de doença ou acidente da criança</t>
-        </is>
-      </c>
-      <c r="O69" s="2" t="inlineStr">
-        <is>
-          <t>Orçamento, Finanças e Administração Pública; Trabalho, Segurança Social e Inclusão</t>
-        </is>
-      </c>
-      <c r="P69" s="2" t="inlineStr">
-        <is>
-          <t>em apreciação</t>
-        </is>
-      </c>
-      <c r="Q69" s="2" t="inlineStr">
-        <is>
-          <t>Entrada (via IPA)</t>
-        </is>
-      </c>
-      <c r="R69" s="2" t="inlineStr"/>
-      <c r="S69" s="2" t="inlineStr"/>
-      <c r="T69" s="2" t="inlineStr"/>
-      <c r="U69" s="2" t="inlineStr"/>
-      <c r="V69" s="2" t="inlineStr"/>
-      <c r="W69" s="2" t="inlineStr"/>
-      <c r="X69" s="2" t="inlineStr"/>
-      <c r="Y69" s="2" t="inlineStr"/>
-      <c r="Z69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA69" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=67</t>
-        </is>
-      </c>
-      <c r="AB69" s="2" t="inlineStr">
-        <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533834596d5a6b5a6a67774f5330314e6a5a694c545133596d5574596a67334d53316c4f4746694e5455775a6a55354e3259756347526d&amp;Fich=8bfdf809-566b-47be-b871-e8ab550f597f.pdf&amp;Inline=true</t>
-        </is>
-      </c>
-      <c r="AC69" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-29 10:04</t>
-        </is>
-      </c>
-      <c r="AD69" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-29 10:04</t>
-        </is>
-      </c>
-      <c r="AE69" s="2" t="inlineStr">
-        <is>
-          <t>opendata</t>
-        </is>
-      </c>
-      <c r="AF69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>68C</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>68C</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr"/>
-      <c r="D70" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-29</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>Comissão</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>Articulado</t>
-        </is>
-      </c>
-      <c r="J70" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 21.º</t>
-        </is>
-      </c>
-      <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr"/>
-      <c r="M70" s="2" t="inlineStr">
-        <is>
-          <t>Por Definir</t>
-        </is>
-      </c>
-      <c r="N70" s="2" t="inlineStr">
-        <is>
-          <t>Profissionalização de Docentes em Serviço - Artigo 21.º - A</t>
-        </is>
-      </c>
-      <c r="O70" s="2" t="inlineStr">
-        <is>
-          <t>Educação e Ciência; Trabalho, Segurança Social e Inclusão</t>
-        </is>
-      </c>
-      <c r="P70" s="2" t="inlineStr">
-        <is>
-          <t>em apreciação</t>
-        </is>
-      </c>
-      <c r="Q70" s="2" t="inlineStr">
-        <is>
-          <t>Entrada (via IPA)</t>
-        </is>
-      </c>
-      <c r="R70" s="2" t="inlineStr"/>
-      <c r="S70" s="2" t="inlineStr"/>
-      <c r="T70" s="2" t="inlineStr"/>
-      <c r="U70" s="2" t="inlineStr"/>
-      <c r="V70" s="2" t="inlineStr"/>
-      <c r="W70" s="2" t="inlineStr"/>
-      <c r="X70" s="2" t="inlineStr"/>
-      <c r="Y70" s="2" t="inlineStr"/>
-      <c r="Z70" s="2" t="inlineStr"/>
-      <c r="AA70" s="2" t="inlineStr">
-        <is>
-          <t>https://www.parlamento.pt/OrcamentoEstado/Paginas/DetalhePropostaAlteracao.aspx?BID=68</t>
-        </is>
-      </c>
-      <c r="AB70" s="2" t="inlineStr">
-        <is>
-          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?Path=dotxco%2fpx15BG%2fpAeZ6fyjol4qnhm4j%2bMj%2boSXIVSCxCjdBEoF6k%2fQejo%2bDQ3OcgOAXuKz37Nu53KyC%2fxAkBqAf7XjFeIcc6VIH1Xjmw%2fhFp8s9ug%2fhiWg0PL2uxbGUi9Ws2la7ZJ3c7te%2fBVWXOlzybF4HQAdIGZi4gOYHICm%2bE%2bKZ9eCTphWGMcPJB1TjLogsw0qe36LdU2C7q%2fujd1YiTvHj8vgwA0MSbF6PPN472nUxv7N5ilUr%2buNtzmdI09kKIGZ%2fOX4qAnm7CUrrNo%2bQXOWGaBChTTDX6s8TaXGIn44%2f0wy0XnDub4VFkCbAjUD8CehpKwsDBEmKIrprewruPUoMveS6hS93y9e0nfzc%3d&amp;Fich=104accf0-0cad-4f8e-8757-537cded9dcc2.pdf&amp;Inline=true</t>
-        </is>
-      </c>
-      <c r="AC70" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-29 10:04</t>
-        </is>
-      </c>
-      <c r="AD70" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-29 10:04</t>
-        </is>
-      </c>
-      <c r="AE70" s="2" t="inlineStr">
-        <is>
-          <t>scrape</t>
-        </is>
-      </c>
-      <c r="AF70" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AF70"/>
+  <autoFilter ref="A1:AF68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8023,7 +7555,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 10:05 UTC</t>
+          <t>2026-10-29 10:07 UTC</t>
         </is>
       </c>
     </row>
@@ -8034,7 +7566,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7">
@@ -8044,7 +7576,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-29 10:08 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Propostas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Propostas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$68</definedName>
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04</t>
+          <t>2026-10-29 10:08</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7543,7 +7543,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 10:04 UTC</t>
+          <t>2026-10-29 10:08 UTC</t>
         </is>
       </c>
     </row>
@@ -7555,7 +7555,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 10:07 UTC</t>
+          <t>2026-10-29 10:08 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 12:19 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF68"/>
+  <dimension ref="A1:AF91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -715,7 +715,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr"/>
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr"/>
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr"/>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr"/>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr"/>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr"/>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr"/>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr"/>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08</t>
+          <t>2026-10-29 12:19</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7484,8 +7484,2578 @@
       </c>
       <c r="AF68" s="2" t="inlineStr"/>
     </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>68C</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>68C</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr"/>
+      <c r="D69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:02</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>Profissionalização de Docentes em Serviço - Artigo 21.º - A</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>Educação e Ciência; Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="inlineStr"/>
+      <c r="S69" s="2" t="inlineStr"/>
+      <c r="T69" s="2" t="inlineStr"/>
+      <c r="U69" s="2" t="inlineStr"/>
+      <c r="V69" s="2" t="inlineStr"/>
+      <c r="W69" s="2" t="inlineStr"/>
+      <c r="X69" s="2" t="inlineStr"/>
+      <c r="Y69" s="2" t="inlineStr"/>
+      <c r="Z69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="2" t="inlineStr"/>
+      <c r="AB69" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338784d44526859324e6d4d4330775932466b4c54526d4f4755744f4463314e7930314d7a646a5a47566b4f57526a597a49756347526d&amp;Fich=104accf0-0cad-4f8e-8757-537cded9dcc2.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE69" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>69C</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>69C</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr"/>
+      <c r="D70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:04</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 113.º-A - Cheque-livro</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>Cultura, Comunicação, Juventude e Desporto</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr"/>
+      <c r="S70" s="2" t="inlineStr"/>
+      <c r="T70" s="2" t="inlineStr"/>
+      <c r="U70" s="2" t="inlineStr"/>
+      <c r="V70" s="2" t="inlineStr"/>
+      <c r="W70" s="2" t="inlineStr"/>
+      <c r="X70" s="2" t="inlineStr"/>
+      <c r="Y70" s="2" t="inlineStr"/>
+      <c r="Z70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="2" t="inlineStr"/>
+      <c r="AB70" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c597a41314e44426d596930324e6d4e6c4c54526d4e575174596d4a6b4e69316c4e5759305a6a6b7a5a444934596a63756347526d&amp;Fich=ec0540fb-66ce-4f5d-bbd6-e5f4f93d28b7.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE70" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>70C</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>70C</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr"/>
+      <c r="D71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:06</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>Levantamento exaustivo das famílias em situação de vulnerabilidade habitacional - 6.º - A</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P71" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="inlineStr"/>
+      <c r="S71" s="2" t="inlineStr"/>
+      <c r="T71" s="2" t="inlineStr"/>
+      <c r="U71" s="2" t="inlineStr"/>
+      <c r="V71" s="2" t="inlineStr"/>
+      <c r="W71" s="2" t="inlineStr"/>
+      <c r="X71" s="2" t="inlineStr"/>
+      <c r="Y71" s="2" t="inlineStr"/>
+      <c r="Z71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA71" s="2" t="inlineStr"/>
+      <c r="AB71" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4e6d5a6c4d7a41314e4330354d7a6b774c54526c4d474974595756685a5330794d4467314d6d566a5954686d4e5751756347526d&amp;Fich=36fe3054-9390-4e0b-aeae-20852eca8f5d.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE71" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>71C</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>71C</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:08</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>Cria o Programa de Alargamento da Rede de Equipamentos Sociais - Quarta Geração - Artigo 45.º-A</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="inlineStr"/>
+      <c r="S72" s="2" t="inlineStr"/>
+      <c r="T72" s="2" t="inlineStr"/>
+      <c r="U72" s="2" t="inlineStr"/>
+      <c r="V72" s="2" t="inlineStr"/>
+      <c r="W72" s="2" t="inlineStr"/>
+      <c r="X72" s="2" t="inlineStr"/>
+      <c r="Y72" s="2" t="inlineStr">
+        <is>
+          <t>01 - Encargos Gerais do Estado</t>
+        </is>
+      </c>
+      <c r="Z72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="2" t="inlineStr"/>
+      <c r="AB72" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338774f5451304d445a685a53316d4e4467314c54526a595449744f544e6a5a5330794e7a417a4f5445324f4756685a6a4d756347526d&amp;Fich=094406ae-f485-4ca2-93ce-27039168eaf3.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE72" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>72C</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>72C</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr"/>
+      <c r="D73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:08</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr"/>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 117.º-A - Apoio à gestão e residência na Rede de Teatros e Cineteatros Portugueses e na Rede Portuguesa de Arte Contemporânea</t>
+        </is>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>Cultura, Comunicação, Juventude e Desporto</t>
+        </is>
+      </c>
+      <c r="P73" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q73" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R73" s="2" t="inlineStr"/>
+      <c r="S73" s="2" t="inlineStr"/>
+      <c r="T73" s="2" t="inlineStr"/>
+      <c r="U73" s="2" t="inlineStr"/>
+      <c r="V73" s="2" t="inlineStr"/>
+      <c r="W73" s="2" t="inlineStr"/>
+      <c r="X73" s="2" t="inlineStr"/>
+      <c r="Y73" s="2" t="inlineStr">
+        <is>
+          <t>07 - Ambiente, do Ordenamento do Território e do Desenvolvimento Regional</t>
+        </is>
+      </c>
+      <c r="Z73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA73" s="2" t="inlineStr"/>
+      <c r="AB73" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338354e3251794e474e68595331684e445a6b4c54526b4e4459744f444e6d4d6931694d4467774d6a45304d5755794e3249756347526d&amp;Fich=97d24caa-a46d-4d46-83f2-b0802141e27b.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE73" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>73C</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>73C</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr"/>
+      <c r="D74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:10</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 6.º</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>Transferências orçamentais</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>Programa Casas de Função - Artigo 110.º - A</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q74" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="inlineStr"/>
+      <c r="S74" s="2" t="inlineStr"/>
+      <c r="T74" s="2" t="inlineStr"/>
+      <c r="U74" s="2" t="inlineStr"/>
+      <c r="V74" s="2" t="inlineStr"/>
+      <c r="W74" s="2" t="inlineStr"/>
+      <c r="X74" s="2" t="inlineStr"/>
+      <c r="Y74" s="2" t="inlineStr"/>
+      <c r="Z74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA74" s="2" t="inlineStr"/>
+      <c r="AB74" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153383059574e6b4f575a6d5a69316c4d7a41354c545179596a55744f444e6d4e6930794e5446684f54686a4f4442684d574d756347526d&amp;Fich=4acd9fff-e309-42b5-83f6-251a98c80a1c.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE74" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>74C</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>74C</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr"/>
+      <c r="D75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:10</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 104.º-B (Programa Nacional de financiamento da rede de centros de recuperação de fauna selvagem)</t>
+        </is>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>Agricultura e Pescas</t>
+        </is>
+      </c>
+      <c r="P75" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q75" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R75" s="2" t="inlineStr"/>
+      <c r="S75" s="2" t="inlineStr"/>
+      <c r="T75" s="2" t="inlineStr"/>
+      <c r="U75" s="2" t="inlineStr"/>
+      <c r="V75" s="2" t="inlineStr"/>
+      <c r="W75" s="2" t="inlineStr"/>
+      <c r="X75" s="2" t="inlineStr"/>
+      <c r="Y75" s="2" t="inlineStr">
+        <is>
+          <t>07 - Ambiente, do Ordenamento do Território e do Desenvolvimento Regional</t>
+        </is>
+      </c>
+      <c r="Z75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA75" s="2" t="inlineStr"/>
+      <c r="AB75" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c596a677a4f4455305a43316c4e574e684c5451775a5441744f4759794f43316c4e474a6d597a566c4e6a4d774f5759756347526d&amp;Fich=eb83854d-e5ca-40e0-8f28-e4bfc5e6309f.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD75" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE75" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>75C</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>75C</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr"/>
+      <c r="D76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:11</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 6.º</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>Transferências orçamentais</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 115.º-A - Língua Gestual Portuguesa nas Escolas</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>Educação e Ciência</t>
+        </is>
+      </c>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q76" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R76" s="2" t="inlineStr"/>
+      <c r="S76" s="2" t="inlineStr"/>
+      <c r="T76" s="2" t="inlineStr"/>
+      <c r="U76" s="2" t="inlineStr"/>
+      <c r="V76" s="2" t="inlineStr"/>
+      <c r="W76" s="2" t="inlineStr"/>
+      <c r="X76" s="2" t="inlineStr"/>
+      <c r="Y76" s="2" t="inlineStr"/>
+      <c r="Z76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="2" t="inlineStr"/>
+      <c r="AB76" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684e3259784e6a466c4e4331694d4745794c54517a5a474574596a5977595330344d4759344d4459794f54466c4f446b756347526d&amp;Fich=a7f161e4-b0a2-43da-b60a-80f806291e89.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE76" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>76C</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>76C</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr"/>
+      <c r="D77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:11</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 38.º - A - Alteração ao Código do Trabalho - Alarga o direito dos trabalhadores a faltar nos casos de hospitalização domiciliária da criança</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P77" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q77" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R77" s="2" t="inlineStr"/>
+      <c r="S77" s="2" t="inlineStr"/>
+      <c r="T77" s="2" t="inlineStr"/>
+      <c r="U77" s="2" t="inlineStr"/>
+      <c r="V77" s="2" t="inlineStr"/>
+      <c r="W77" s="2" t="inlineStr"/>
+      <c r="X77" s="2" t="inlineStr"/>
+      <c r="Y77" s="2" t="inlineStr">
+        <is>
+          <t>10 - Obras Públicas, Transportes e Comunicações</t>
+        </is>
+      </c>
+      <c r="Z77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="2" t="inlineStr"/>
+      <c r="AB77" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d54457a4d7a56694d6930344d44526b4c5451344f44597459574e694e6930335a6a51775a545179597a566b4d6a55756347526d&amp;Fich=811335b2-804d-4886-acb6-7f40e42c5d25.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE77" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>77C</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>77C</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr"/>
+      <c r="D78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:12</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 63.º-D (Alteração ao Código do Imposto sobre o Valor Acrescentado)</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P78" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q78" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R78" s="2" t="inlineStr"/>
+      <c r="S78" s="2" t="inlineStr"/>
+      <c r="T78" s="2" t="inlineStr"/>
+      <c r="U78" s="2" t="inlineStr"/>
+      <c r="V78" s="2" t="inlineStr"/>
+      <c r="W78" s="2" t="inlineStr"/>
+      <c r="X78" s="2" t="inlineStr"/>
+      <c r="Y78" s="2" t="inlineStr">
+        <is>
+          <t>10 - Obras Públicas, Transportes e Comunicações</t>
+        </is>
+      </c>
+      <c r="Z78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="2" t="inlineStr"/>
+      <c r="AB78" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4e7a49304e6d49795953316a4e574d344c5451324e545574595755314e7931694f574a6859575a6c5a44597a5a6a51756347526d&amp;Fich=f7246b2a-c5c8-4655-ae57-b9baafed63f4.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE78" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>78C</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>78C</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr"/>
+      <c r="D79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:13</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 65.º-A (Alteração ao Código do Imposto Municipal sobre Imóveis)</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P79" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q79" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R79" s="2" t="inlineStr"/>
+      <c r="S79" s="2" t="inlineStr"/>
+      <c r="T79" s="2" t="inlineStr"/>
+      <c r="U79" s="2" t="inlineStr"/>
+      <c r="V79" s="2" t="inlineStr"/>
+      <c r="W79" s="2" t="inlineStr"/>
+      <c r="X79" s="2" t="inlineStr"/>
+      <c r="Y79" s="2" t="inlineStr">
+        <is>
+          <t>11 - Trabalho e Solidariedade Social</t>
+        </is>
+      </c>
+      <c r="Z79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="2" t="inlineStr"/>
+      <c r="AB79" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324e6a5a6b597a466b597930794d6d4d334c5451324d445574595445344e53316d4d574530597a686b593255355a444d756347526d&amp;Fich=666dc1dc-22c7-4605-a185-f1a4c8dce9d3.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE79" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>79C</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>79C</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr"/>
+      <c r="D80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:14</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 6.º</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>Transferências orçamentais</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 63.º-C (Alteração à lista I anexa ao Código do Imposto sobre o Valor Acrescentado)</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q80" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R80" s="2" t="inlineStr"/>
+      <c r="S80" s="2" t="inlineStr"/>
+      <c r="T80" s="2" t="inlineStr"/>
+      <c r="U80" s="2" t="inlineStr"/>
+      <c r="V80" s="2" t="inlineStr"/>
+      <c r="W80" s="2" t="inlineStr"/>
+      <c r="X80" s="2" t="inlineStr"/>
+      <c r="Y80" s="2" t="inlineStr"/>
+      <c r="Z80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="2" t="inlineStr"/>
+      <c r="AB80" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338784d6a55794d5755774e6931694e324d344c545135597a4974596d46694e4331694d574d30596d45344d6d45775a4451756347526d&amp;Fich=12521e06-b7c8-49c2-bab4-b1c4ba82a0d4.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE80" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>80C</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>80C</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr"/>
+      <c r="D81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:17</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr"/>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 22.º - A - Abertura de concursos em Medicina Geral e Familiar</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="P81" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q81" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R81" s="2" t="inlineStr"/>
+      <c r="S81" s="2" t="inlineStr"/>
+      <c r="T81" s="2" t="inlineStr"/>
+      <c r="U81" s="2" t="inlineStr"/>
+      <c r="V81" s="2" t="inlineStr"/>
+      <c r="W81" s="2" t="inlineStr"/>
+      <c r="X81" s="2" t="inlineStr"/>
+      <c r="Y81" s="2" t="inlineStr">
+        <is>
+          <t>13 - Educação</t>
+        </is>
+      </c>
+      <c r="Z81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="2" t="inlineStr"/>
+      <c r="AB81" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396b59574d3459574d77596931684e7a63354c54517a4d444974596a4535595330334f5459344e6a4933595441354e6a51756347526d&amp;Fich=dac8ac0b-a779-4302-b19a-7968627a0964.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE81" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>81C</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>81C</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr"/>
+      <c r="D82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:21</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 127.º-A (Apoios à transição tecnológica no setor avícola e revisão da legislação relativa ao bem-estar animal)</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>Agricultura e Pescas</t>
+        </is>
+      </c>
+      <c r="P82" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q82" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R82" s="2" t="inlineStr"/>
+      <c r="S82" s="2" t="inlineStr"/>
+      <c r="T82" s="2" t="inlineStr"/>
+      <c r="U82" s="2" t="inlineStr"/>
+      <c r="V82" s="2" t="inlineStr"/>
+      <c r="W82" s="2" t="inlineStr"/>
+      <c r="X82" s="2" t="inlineStr"/>
+      <c r="Y82" s="2" t="inlineStr">
+        <is>
+          <t>10 - Obras Públicas, Transportes e Comunicações</t>
+        </is>
+      </c>
+      <c r="Z82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA82" s="2" t="inlineStr"/>
+      <c r="AB82" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4d7a4578596d5668595331685a5467314c54526b597a41744f54557a4d79316a4f4759334e57526b4d546c6c597a45756347526d&amp;Fich=f311beaa-ae85-4dc0-9533-c8f75dd19ec1.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE82" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>82C</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>82C</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr"/>
+      <c r="D83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:21</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 6.º</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>Transferências orçamentais</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr"/>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>NOVO] Artigo 38.º - A - Aditamento ao Decreto-Lei n.º 91/2009, de 9 de abril - Permite que ambos os pais acompanhem a criança com doença oncológica, sem perda financeira, sempre que medicamente recomendado</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P83" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q83" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R83" s="2" t="inlineStr"/>
+      <c r="S83" s="2" t="inlineStr"/>
+      <c r="T83" s="2" t="inlineStr"/>
+      <c r="U83" s="2" t="inlineStr"/>
+      <c r="V83" s="2" t="inlineStr"/>
+      <c r="W83" s="2" t="inlineStr"/>
+      <c r="X83" s="2" t="inlineStr"/>
+      <c r="Y83" s="2" t="inlineStr"/>
+      <c r="Z83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA83" s="2" t="inlineStr"/>
+      <c r="AB83" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4d7a6c6a597a526c5969307a5a4751324c5451355a6d59744f54457959793035597a4a6a59575a6b5a6a4e684d6d49756347526d&amp;Fich=e39cc4eb-3dd6-49ff-912c-9c2cafdf3a2b.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE83" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>83C</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>83C</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr"/>
+      <c r="D84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:22</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="inlineStr"/>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 21.º-B (Integração de investigadores bolseiros na Carreira de Investigação Científica)</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>Educação e Ciência</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q84" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R84" s="2" t="inlineStr"/>
+      <c r="S84" s="2" t="inlineStr"/>
+      <c r="T84" s="2" t="inlineStr"/>
+      <c r="U84" s="2" t="inlineStr"/>
+      <c r="V84" s="2" t="inlineStr"/>
+      <c r="W84" s="2" t="inlineStr"/>
+      <c r="X84" s="2" t="inlineStr"/>
+      <c r="Y84" s="2" t="inlineStr">
+        <is>
+          <t>10 - Obras Públicas, Transportes e Comunicações</t>
+        </is>
+      </c>
+      <c r="Z84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA84" s="2" t="inlineStr"/>
+      <c r="AB84" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4d6d526b597a4932596930354d6d52684c54526b4e5449744f574e6d4e43316d5a5759344f444e6d59545a684e546b756347526d&amp;Fich=32ddc26b-92da-4d52-9cf4-fef883fa6a59.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE84" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>84C</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>84C</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr"/>
+      <c r="D85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:22</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>Mapas</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="inlineStr"/>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>Anexo I - Mapa de alterações e transferências orçamentais (Majoração dos projetos de reflorestação nativa)</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>Ambiente e Energia</t>
+        </is>
+      </c>
+      <c r="P85" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q85" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R85" s="2" t="inlineStr"/>
+      <c r="S85" s="2" t="inlineStr"/>
+      <c r="T85" s="2" t="inlineStr"/>
+      <c r="U85" s="2" t="inlineStr"/>
+      <c r="V85" s="2" t="inlineStr"/>
+      <c r="W85" s="2" t="inlineStr"/>
+      <c r="X85" s="2" t="inlineStr"/>
+      <c r="Y85" s="2" t="inlineStr">
+        <is>
+          <t>09 - Agricultura, Desenvolvimento Rural e Pescas</t>
+        </is>
+      </c>
+      <c r="Z85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA85" s="2" t="inlineStr"/>
+      <c r="AB85" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533832593245334d6d55775a6931685a4449774c5451314d446b744f474d354d433031596a426b5a4463354d4451334e7a45756347526d&amp;Fich=6ca72e0f-ad20-4509-8c90-5b0dd7904771.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE85" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>85C</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>85C</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr"/>
+      <c r="D86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:23</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 116.º-A (Eliminação de taxas e emolumentos referentes à entrega de dissertações e emissão de diplomas no Ensino Superior)</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>Educação e Ciência</t>
+        </is>
+      </c>
+      <c r="P86" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q86" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R86" s="2" t="inlineStr"/>
+      <c r="S86" s="2" t="inlineStr"/>
+      <c r="T86" s="2" t="inlineStr"/>
+      <c r="U86" s="2" t="inlineStr"/>
+      <c r="V86" s="2" t="inlineStr"/>
+      <c r="W86" s="2" t="inlineStr"/>
+      <c r="X86" s="2" t="inlineStr"/>
+      <c r="Y86" s="2" t="inlineStr">
+        <is>
+          <t>01 - Encargos Gerais do Estado</t>
+        </is>
+      </c>
+      <c r="Z86" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA86" s="2" t="inlineStr"/>
+      <c r="AB86" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4e7a4d344f4755794d43307a5a4445784c54526859545974595441335969303559574a6d4e7a637a5a54566b4e5755756347526d&amp;Fich=f7388e20-3d11-4aa6-a07b-9abf773e5d5e.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD86" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE86" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>86C</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>86C</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr"/>
+      <c r="D87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:58</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr"/>
+      <c r="M87" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 62.º - A - Alteração ao Código do Imposto sobre o Valor Acrescentado (IVA Atos Veterinários)</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>Agricultura e Pescas; Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P87" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q87" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R87" s="2" t="inlineStr"/>
+      <c r="S87" s="2" t="inlineStr"/>
+      <c r="T87" s="2" t="inlineStr"/>
+      <c r="U87" s="2" t="inlineStr"/>
+      <c r="V87" s="2" t="inlineStr"/>
+      <c r="W87" s="2" t="inlineStr"/>
+      <c r="X87" s="2" t="inlineStr"/>
+      <c r="Y87" s="2" t="inlineStr">
+        <is>
+          <t>07 - Ambiente, do Ordenamento do Território e do Desenvolvimento Regional</t>
+        </is>
+      </c>
+      <c r="Z87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA87" s="2" t="inlineStr"/>
+      <c r="AB87" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684d545a6b4d4464685a5331695a444e6d4c54526d59545574595456685969307759544930597a646b5a6a646d4e7a4d756347526d&amp;Fich=a16d07ae-bd3f-4fa5-a5ab-0a24c7df7f73.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD87" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE87" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>87C</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>87C</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr"/>
+      <c r="D88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:00</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 122.º-A - Apoio para instalação de hangares de bicicletas em parques de estacionamento</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q88" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R88" s="2" t="inlineStr"/>
+      <c r="S88" s="2" t="inlineStr"/>
+      <c r="T88" s="2" t="inlineStr"/>
+      <c r="U88" s="2" t="inlineStr"/>
+      <c r="V88" s="2" t="inlineStr"/>
+      <c r="W88" s="2" t="inlineStr"/>
+      <c r="X88" s="2" t="inlineStr"/>
+      <c r="Y88" s="2" t="inlineStr">
+        <is>
+          <t>12 - Saúde</t>
+        </is>
+      </c>
+      <c r="Z88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA88" s="2" t="inlineStr"/>
+      <c r="AB88" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a5a474d334d7a41785979316d59574a6d4c545134595745744f474e6c4e79316a5a6a6b314e6a5a6b4f474d7a5a5467756347526d&amp;Fich=3dc7301c-fabf-48aa-8ce7-cf9566d8c3e8.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD88" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE88" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>88C</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>88C</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr"/>
+      <c r="D89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:01</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr"/>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>PA - Aditamento - Redução da taxa normal do IVA de 23% para 22,5% - Artigo 64.º-A</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P89" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q89" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R89" s="2" t="inlineStr"/>
+      <c r="S89" s="2" t="inlineStr"/>
+      <c r="T89" s="2" t="inlineStr"/>
+      <c r="U89" s="2" t="inlineStr"/>
+      <c r="V89" s="2" t="inlineStr"/>
+      <c r="W89" s="2" t="inlineStr"/>
+      <c r="X89" s="2" t="inlineStr"/>
+      <c r="Y89" s="2" t="inlineStr">
+        <is>
+          <t>15 - Cultura</t>
+        </is>
+      </c>
+      <c r="Z89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA89" s="2" t="inlineStr"/>
+      <c r="AB89" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4e5449345a546c6a5a433031596d4e6c4c54526a4e4441744f44686b5a693168597a526d4f574a685954466a4d4745756347526d&amp;Fich=e528e9cd-5bce-4c40-88df-ac4f9baa1c0a.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD89" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE89" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>89C</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>89C</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr"/>
+      <c r="D90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:02</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr"/>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 122.º-A - Projetos-piloto de logística urbana sustentável</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q90" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R90" s="2" t="inlineStr"/>
+      <c r="S90" s="2" t="inlineStr"/>
+      <c r="T90" s="2" t="inlineStr"/>
+      <c r="U90" s="2" t="inlineStr"/>
+      <c r="V90" s="2" t="inlineStr"/>
+      <c r="W90" s="2" t="inlineStr"/>
+      <c r="X90" s="2" t="inlineStr"/>
+      <c r="Y90" s="2" t="inlineStr">
+        <is>
+          <t>15 - Cultura</t>
+        </is>
+      </c>
+      <c r="Z90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA90" s="2" t="inlineStr"/>
+      <c r="AB90" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396b5a6d466d4d546334596930774e6a55324c5451314e7a6b744f5441325979316a5a6d4d355a47566b4d5467345a6d51756347526d&amp;Fich=dfaf178b-0656-4579-906c-cfc9ded188fd.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE90" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>90C</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>90C</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr"/>
+      <c r="D91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 11:07</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 1.º</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>Aprovação</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="inlineStr"/>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>Valorização dos assistentes operacionais e assistentes técnicos nas escolas públicas - Artigo 85.º - A</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>Educação e Ciência; Reforma do Estado e Poder Local; Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P91" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q91" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R91" s="2" t="inlineStr"/>
+      <c r="S91" s="2" t="inlineStr"/>
+      <c r="T91" s="2" t="inlineStr"/>
+      <c r="U91" s="2" t="inlineStr"/>
+      <c r="V91" s="2" t="inlineStr"/>
+      <c r="W91" s="2" t="inlineStr"/>
+      <c r="X91" s="2" t="inlineStr"/>
+      <c r="Y91" s="2" t="inlineStr">
+        <is>
+          <t>12 - Saúde</t>
+        </is>
+      </c>
+      <c r="Z91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA91" s="2" t="inlineStr"/>
+      <c r="AB91" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324e446c6c5a4745344e7930315a546b344c5451775a6a5174595441354d6931694e54637a4f4445344e54457759574d756347526d&amp;Fich=649eda87-5e98-40f4-a092-b573818510ac.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AD91" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 12:19</t>
+        </is>
+      </c>
+      <c r="AE91" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF91" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF68"/>
+  <autoFilter ref="A1:AF91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7543,7 +10113,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08 UTC</t>
+          <t>2026-10-29 12:19 UTC</t>
         </is>
       </c>
     </row>
@@ -7555,7 +10125,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 10:08 UTC</t>
+          <t>2026-10-29 12:19 UTC</t>
         </is>
       </c>
     </row>
@@ -7566,7 +10136,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>67</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7">
@@ -7576,7 +10146,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>67</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-29 12:33 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8232,7 +8232,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8456,7 +8456,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8570,7 +8570,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8684,7 +8684,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8794,7 +8794,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9132,7 +9132,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9246,7 +9246,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9702,7 +9702,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19</t>
+          <t>2026-10-29 12:32</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10113,7 +10113,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19 UTC</t>
+          <t>2026-10-29 12:32 UTC</t>
         </is>
       </c>
     </row>
@@ -10125,7 +10125,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 12:19 UTC</t>
+          <t>2026-10-29 12:33 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 12:34 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7830,16 +7830,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr"/>
       <c r="M72" s="2" t="inlineStr">
         <is>
@@ -7894,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7944,16 +7936,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K73" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr"/>
       <c r="L73" s="2" t="inlineStr"/>
       <c r="M73" s="2" t="inlineStr">
         <is>
@@ -8008,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8058,16 +8042,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 6.º</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr">
-        <is>
-          <t>Transferências orçamentais</t>
-        </is>
-      </c>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr"/>
       <c r="M74" s="2" t="inlineStr">
         <is>
@@ -8118,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8168,16 +8144,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K75" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr"/>
       <c r="M75" s="2" t="inlineStr">
         <is>
@@ -8232,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8282,16 +8250,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 6.º</t>
-        </is>
-      </c>
-      <c r="K76" s="2" t="inlineStr">
-        <is>
-          <t>Transferências orçamentais</t>
-        </is>
-      </c>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr">
         <is>
@@ -8342,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8392,16 +8352,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K77" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr"/>
       <c r="M77" s="2" t="inlineStr">
         <is>
@@ -8456,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8506,16 +8458,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K78" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr">
         <is>
@@ -8570,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,16 +8564,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J79" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K79" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr"/>
       <c r="L79" s="2" t="inlineStr"/>
       <c r="M79" s="2" t="inlineStr">
         <is>
@@ -8684,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8734,16 +8670,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J80" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 6.º</t>
-        </is>
-      </c>
-      <c r="K80" s="2" t="inlineStr">
-        <is>
-          <t>Transferências orçamentais</t>
-        </is>
-      </c>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr"/>
       <c r="M80" s="2" t="inlineStr">
         <is>
@@ -8794,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8844,16 +8772,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J81" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K81" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J81" s="2" t="inlineStr"/>
+      <c r="K81" s="2" t="inlineStr"/>
       <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="2" t="inlineStr">
         <is>
@@ -8908,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8958,16 +8878,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K82" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr"/>
       <c r="M82" s="2" t="inlineStr">
         <is>
@@ -9022,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9072,16 +8984,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J83" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 6.º</t>
-        </is>
-      </c>
-      <c r="K83" s="2" t="inlineStr">
-        <is>
-          <t>Transferências orçamentais</t>
-        </is>
-      </c>
+      <c r="J83" s="2" t="inlineStr"/>
+      <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr"/>
       <c r="M83" s="2" t="inlineStr">
         <is>
@@ -9132,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9182,16 +9086,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J84" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K84" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr"/>
       <c r="M84" s="2" t="inlineStr">
         <is>
@@ -9246,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9296,16 +9192,8 @@
           <t>Mapas</t>
         </is>
       </c>
-      <c r="J85" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K85" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J85" s="2" t="inlineStr"/>
+      <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr"/>
       <c r="M85" s="2" t="inlineStr">
         <is>
@@ -9360,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9410,16 +9298,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J86" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K86" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr"/>
       <c r="M86" s="2" t="inlineStr">
         <is>
@@ -9474,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9524,16 +9404,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J87" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K87" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J87" s="2" t="inlineStr"/>
+      <c r="K87" s="2" t="inlineStr"/>
       <c r="L87" s="2" t="inlineStr"/>
       <c r="M87" s="2" t="inlineStr">
         <is>
@@ -9588,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9638,16 +9510,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J88" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K88" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr"/>
       <c r="M88" s="2" t="inlineStr">
         <is>
@@ -9702,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9752,16 +9616,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J89" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K89" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J89" s="2" t="inlineStr"/>
+      <c r="K89" s="2" t="inlineStr"/>
       <c r="L89" s="2" t="inlineStr"/>
       <c r="M89" s="2" t="inlineStr">
         <is>
@@ -9816,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9866,16 +9722,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J90" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K90" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J90" s="2" t="inlineStr"/>
+      <c r="K90" s="2" t="inlineStr"/>
       <c r="L90" s="2" t="inlineStr"/>
       <c r="M90" s="2" t="inlineStr">
         <is>
@@ -9930,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9980,16 +9828,8 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J91" s="2" t="inlineStr">
-        <is>
-          <t>Artigo 1.º</t>
-        </is>
-      </c>
-      <c r="K91" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
+      <c r="J91" s="2" t="inlineStr"/>
+      <c r="K91" s="2" t="inlineStr"/>
       <c r="L91" s="2" t="inlineStr"/>
       <c r="M91" s="2" t="inlineStr">
         <is>
@@ -10044,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32</t>
+          <t>2026-10-29 12:34</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10113,7 +9953,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 12:32 UTC</t>
+          <t>2026-10-29 12:34 UTC</t>
         </is>
       </c>
     </row>
@@ -10125,7 +9965,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 12:33 UTC</t>
+          <t>2026-10-29 12:34 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 12:45 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34</t>
+          <t>2026-10-29 12:44</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9953,7 +9953,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34 UTC</t>
+          <t>2026-10-29 12:44 UTC</t>
         </is>
       </c>
     </row>
@@ -9965,7 +9965,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 12:34 UTC</t>
+          <t>2026-10-29 12:45 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 13:50 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr"/>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr"/>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr"/>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr"/>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr"/>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr"/>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44</t>
+          <t>2026-10-29 13:50</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9953,7 +9953,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 12:44 UTC</t>
+          <t>2026-10-29 13:50 UTC</t>
         </is>
       </c>
     </row>
@@ -9965,7 +9965,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 12:45 UTC</t>
+          <t>2026-10-29 13:50 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 14:15 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50</t>
+          <t>2026-10-29 14:14</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9953,7 +9953,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50 UTC</t>
+          <t>2026-10-29 14:14 UTC</t>
         </is>
       </c>
     </row>
@@ -9965,7 +9965,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 13:50 UTC</t>
+          <t>2026-10-29 14:15 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 14:27 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14</t>
+          <t>2026-10-29 14:26</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9953,7 +9953,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 14:14 UTC</t>
+          <t>2026-10-29 14:26 UTC</t>
         </is>
       </c>
     </row>
@@ -9965,7 +9965,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 14:15 UTC</t>
+          <t>2026-10-29 14:27 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 14:29 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26</t>
+          <t>2026-10-29 14:28</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9953,7 +9953,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 14:26 UTC</t>
+          <t>2026-10-29 14:28 UTC</t>
         </is>
       </c>
     </row>
@@ -9965,7 +9965,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 14:27 UTC</t>
+          <t>2026-10-29 14:29 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 15:26 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr"/>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr"/>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr"/>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2648,12 +2648,12 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr"/>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr"/>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R23" s="2" t="inlineStr"/>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R24" s="2" t="inlineStr"/>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R25" s="2" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3158,12 +3158,12 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R26" s="2" t="inlineStr"/>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3362,12 +3362,12 @@
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr"/>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr"/>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3566,12 +3566,12 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr"/>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28</t>
+          <t>2026-10-29 15:26</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9953,7 +9953,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 14:28 UTC</t>
+          <t>2026-10-29 15:26 UTC</t>
         </is>
       </c>
     </row>
@@ -9965,7 +9965,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 14:29 UTC</t>
+          <t>2026-10-29 15:26 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 16:25 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF91"/>
+  <dimension ref="A1:AF94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr"/>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3877,7 +3877,7 @@
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr"/>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -3974,12 +3974,12 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R34" s="2" t="inlineStr"/>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr"/>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R36" s="2" t="inlineStr"/>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26</t>
+          <t>2026-10-29 16:25</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9894,8 +9894,326 @@
       </c>
       <c r="AF91" s="2" t="inlineStr"/>
     </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>91C</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>91C</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr"/>
+      <c r="D92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 15:31</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr"/>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 62.º-A Alteração ao Código do Imposto sobre o Rendimento das Pessoas Coletivas (Alarga a taxa reduzida de IRC das PME aos primeiros 100.000 € de lucro)</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q92" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R92" s="2" t="inlineStr"/>
+      <c r="S92" s="2" t="inlineStr"/>
+      <c r="T92" s="2" t="inlineStr"/>
+      <c r="U92" s="2" t="inlineStr"/>
+      <c r="V92" s="2" t="inlineStr"/>
+      <c r="W92" s="2" t="inlineStr"/>
+      <c r="X92" s="2" t="inlineStr"/>
+      <c r="Y92" s="2" t="inlineStr">
+        <is>
+          <t>14 - Ciência, Tecnologia e Ensino Superior</t>
+        </is>
+      </c>
+      <c r="Z92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA92" s="2" t="inlineStr"/>
+      <c r="AB92" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324f44646a596d5669596930784d544d794c5452694f445574596d497a5a4331684e574d774e3259354d4745324e5751756347526d&amp;Fich=687cbebb-1132-4b85-bb3d-a5c07f90a65d.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:25</t>
+        </is>
+      </c>
+      <c r="AD92" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:25</t>
+        </is>
+      </c>
+      <c r="AE92" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>92C</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>92C</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr"/>
+      <c r="D93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 15:34</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr"/>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr"/>
+      <c r="M93" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 62.º-A Aditamento ao Código do Imposto sobre o Rendimento das Pessoas Coletivas (Condiciona a taxa reduzida de IRC à capitalização das empresas)</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>Reforma do Estado e Poder Local</t>
+        </is>
+      </c>
+      <c r="P93" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q93" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R93" s="2" t="inlineStr"/>
+      <c r="S93" s="2" t="inlineStr"/>
+      <c r="T93" s="2" t="inlineStr"/>
+      <c r="U93" s="2" t="inlineStr"/>
+      <c r="V93" s="2" t="inlineStr"/>
+      <c r="W93" s="2" t="inlineStr"/>
+      <c r="X93" s="2" t="inlineStr"/>
+      <c r="Y93" s="2" t="inlineStr">
+        <is>
+          <t>12 - Saúde</t>
+        </is>
+      </c>
+      <c r="Z93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA93" s="2" t="inlineStr"/>
+      <c r="AB93" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338335a6d51774e6a457a596930354d7a49314c5451334d4449744f54597959793033596d526a4f4455354f474e6c596d59756347526d&amp;Fich=7fd0613b-9325-4702-962c-7bdc8598cebf.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:25</t>
+        </is>
+      </c>
+      <c r="AD93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:25</t>
+        </is>
+      </c>
+      <c r="AE93" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>93C</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>93C</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr"/>
+      <c r="D94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 15:39</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr"/>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>NOVO] Artigo 79.º-A Revogação do regime de autorização de residência para atividade de investimento</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q94" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R94" s="2" t="inlineStr"/>
+      <c r="S94" s="2" t="inlineStr"/>
+      <c r="T94" s="2" t="inlineStr"/>
+      <c r="U94" s="2" t="inlineStr"/>
+      <c r="V94" s="2" t="inlineStr"/>
+      <c r="W94" s="2" t="inlineStr"/>
+      <c r="X94" s="2" t="inlineStr"/>
+      <c r="Y94" s="2" t="inlineStr">
+        <is>
+          <t>12 - Saúde</t>
+        </is>
+      </c>
+      <c r="Z94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA94" s="2" t="inlineStr"/>
+      <c r="AB94" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533832595752684f5455324e7930775a6d55334c545131596a67744f445a6c5a43316b59324931597a5a6a4e44466c4f4449756347526d&amp;Fich=6ada9567-0fe7-45b8-86ed-dcb5c6c41e82.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:25</t>
+        </is>
+      </c>
+      <c r="AD94" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 16:25</t>
+        </is>
+      </c>
+      <c r="AE94" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF94" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF91"/>
+  <autoFilter ref="A1:AF94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9953,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26 UTC</t>
+          <t>2026-10-29 16:25 UTC</t>
         </is>
       </c>
     </row>
@@ -9965,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 15:26 UTC</t>
+          <t>2026-10-29 16:25 UTC</t>
         </is>
       </c>
     </row>
@@ -9976,7 +10294,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7">
@@ -9986,7 +10304,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-29 16:56 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4285,7 +4285,7 @@
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr"/>
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr"/>
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R39" s="2" t="inlineStr"/>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4591,7 +4591,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr"/>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R41" s="2" t="inlineStr"/>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4795,7 +4795,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr"/>
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R43" s="2" t="inlineStr"/>
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -4999,7 +4999,7 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr"/>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr"/>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5203,7 +5203,7 @@
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R46" s="2" t="inlineStr"/>
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25</t>
+          <t>2026-10-29 16:55</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25 UTC</t>
+          <t>2026-10-29 16:55 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 16:25 UTC</t>
+          <t>2026-10-29 16:56 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 17:24 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R47" s="2" t="inlineStr"/>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R48" s="2" t="inlineStr"/>
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R49" s="2" t="inlineStr"/>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R50" s="2" t="inlineStr"/>
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R51" s="2" t="inlineStr"/>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5917,7 +5917,7 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr"/>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R54" s="2" t="inlineStr"/>
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6121,7 +6121,7 @@
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R55" s="2" t="inlineStr"/>
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6223,7 +6223,7 @@
       </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R56" s="2" t="inlineStr"/>
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9429,7 +9429,7 @@
       </c>
       <c r="Q87" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R87" s="2" t="inlineStr"/>
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9535,7 +9535,7 @@
       </c>
       <c r="Q88" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R88" s="2" t="inlineStr"/>
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9641,7 +9641,7 @@
       </c>
       <c r="Q89" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R89" s="2" t="inlineStr"/>
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9747,7 +9747,7 @@
       </c>
       <c r="Q90" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R90" s="2" t="inlineStr"/>
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9853,7 +9853,7 @@
       </c>
       <c r="Q91" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R91" s="2" t="inlineStr"/>
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9959,7 +9959,7 @@
       </c>
       <c r="Q92" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R92" s="2" t="inlineStr"/>
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10065,7 +10065,7 @@
       </c>
       <c r="Q93" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R93" s="2" t="inlineStr"/>
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10171,7 +10171,7 @@
       </c>
       <c r="Q94" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R94" s="2" t="inlineStr"/>
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55</t>
+          <t>2026-10-29 17:23</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 16:55 UTC</t>
+          <t>2026-10-29 17:23 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 16:56 UTC</t>
+          <t>2026-10-29 17:24 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 18:23 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3260,12 +3260,12 @@
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R27" s="2" t="inlineStr"/>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3770,12 +3770,12 @@
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R32" s="2" t="inlineStr"/>
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5810,12 +5810,12 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>em apreciação</t>
+          <t>não admitida</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Não Admitida</t>
         </is>
       </c>
       <c r="R52" s="2" t="inlineStr"/>
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7447,7 +7447,7 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R68" s="2" t="inlineStr"/>
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7549,7 +7549,7 @@
       </c>
       <c r="Q69" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R69" s="2" t="inlineStr"/>
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7651,7 +7651,7 @@
       </c>
       <c r="Q70" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R70" s="2" t="inlineStr"/>
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="Q71" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R71" s="2" t="inlineStr"/>
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="Q72" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R72" s="2" t="inlineStr"/>
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7961,7 +7961,7 @@
       </c>
       <c r="Q73" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R73" s="2" t="inlineStr"/>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R74" s="2" t="inlineStr"/>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8169,7 +8169,7 @@
       </c>
       <c r="Q75" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R75" s="2" t="inlineStr"/>
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8275,7 +8275,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R76" s="2" t="inlineStr"/>
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8377,7 +8377,7 @@
       </c>
       <c r="Q77" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R77" s="2" t="inlineStr"/>
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8483,7 +8483,7 @@
       </c>
       <c r="Q78" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R78" s="2" t="inlineStr"/>
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8589,7 +8589,7 @@
       </c>
       <c r="Q79" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R79" s="2" t="inlineStr"/>
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8695,7 +8695,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R80" s="2" t="inlineStr"/>
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8797,7 +8797,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R81" s="2" t="inlineStr"/>
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8903,7 +8903,7 @@
       </c>
       <c r="Q82" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R82" s="2" t="inlineStr"/>
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9009,7 +9009,7 @@
       </c>
       <c r="Q83" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R83" s="2" t="inlineStr"/>
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="Q84" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R84" s="2" t="inlineStr"/>
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9217,7 +9217,7 @@
       </c>
       <c r="Q85" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R85" s="2" t="inlineStr"/>
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9323,7 +9323,7 @@
       </c>
       <c r="Q86" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R86" s="2" t="inlineStr"/>
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23</t>
+          <t>2026-10-29 18:23</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 17:23 UTC</t>
+          <t>2026-10-29 18:23 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 17:24 UTC</t>
+          <t>2026-10-29 18:23 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 19:23 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23</t>
+          <t>2026-10-29 19:23</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23 UTC</t>
+          <t>2026-10-29 19:23 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 18:23 UTC</t>
+          <t>2026-10-29 19:23 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 21:49 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6325,7 +6325,7 @@
       </c>
       <c r="Q57" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R57" s="2" t="inlineStr"/>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="Q58" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R58" s="2" t="inlineStr"/>
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6529,7 +6529,7 @@
       </c>
       <c r="Q59" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R59" s="2" t="inlineStr"/>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6631,7 +6631,7 @@
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R60" s="2" t="inlineStr"/>
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R61" s="2" t="inlineStr"/>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6835,7 +6835,7 @@
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr"/>
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6937,7 +6937,7 @@
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr"/>
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7039,7 +7039,7 @@
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R64" s="2" t="inlineStr"/>
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7141,7 +7141,7 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr"/>
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7243,7 +7243,7 @@
       </c>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R66" s="2" t="inlineStr"/>
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr"/>
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23</t>
+          <t>2026-10-29 21:49</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23 UTC</t>
+          <t>2026-10-29 21:49 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 19:23 UTC</t>
+          <t>2026-10-29 21:49 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 23:18 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49</t>
+          <t>2026-10-29 23:16</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49 UTC</t>
+          <t>2026-10-29 23:16 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 21:49 UTC</t>
+          <t>2026-10-29 23:18 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-29 23:45 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16</t>
+          <t>2026-10-29 23:43</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 23:16 UTC</t>
+          <t>2026-10-29 23:43 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 23:18 UTC</t>
+          <t>2026-10-29 23:45 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-30 00:07 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43</t>
+          <t>2026-10-30 00:07</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 23:43 UTC</t>
+          <t>2026-10-30 00:07 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29 23:45 UTC</t>
+          <t>2026-10-30 00:07 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-30 00:11 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07</t>
+          <t>2026-10-30 00:10</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07 UTC</t>
+          <t>2026-10-30 00:10 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 00:07 UTC</t>
+          <t>2026-10-30 00:11 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-30 00:15 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10</t>
+          <t>2026-10-30 00:15</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 00:10 UTC</t>
+          <t>2026-10-30 00:15 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 00:11 UTC</t>
+          <t>2026-10-30 00:15 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-30 07:31 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4210,7 +4210,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4618,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5230,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6148,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6454,7 +6454,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7270,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7372,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7886,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8408,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8828,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9354,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9566,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9672,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9778,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15</t>
+          <t>2026-10-30 07:31</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15 UTC</t>
+          <t>2026-10-30 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 00:15 UTC</t>
+          <t>2026-10-30 07:31 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
captura 2026-10-30 12:24 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF94"/>
+  <dimension ref="A1:AF95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -663,7 +663,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="n">
-        <v>1</v>
+        <v>25391</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="n">
-        <v>2</v>
+        <v>25392</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="n">
-        <v>3</v>
+        <v>25393</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -894,17 +894,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 63.º-A</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>IVA alimentação animal 63.º-A</t>
+          <t>Artigo 63.º-A (Aditamento à lista I anexa ao Código do Imposto sobre o Valor Acrescentado)</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -919,7 +923,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr"/>
@@ -946,7 +950,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -969,7 +973,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="n">
-        <v>4</v>
+        <v>25394</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -996,12 +1000,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 122.º-A</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1021,7 +1029,7 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr"/>
@@ -1048,7 +1056,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1071,7 +1079,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="n">
-        <v>5</v>
+        <v>25395</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -1150,7 +1158,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1173,7 +1181,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="n">
-        <v>6</v>
+        <v>25396</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -1252,7 +1260,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1275,7 +1283,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="n">
-        <v>7</v>
+        <v>25397</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -1354,7 +1362,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1377,7 +1385,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="n">
-        <v>8</v>
+        <v>25398</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -1456,7 +1464,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1479,7 +1487,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="n">
-        <v>9</v>
+        <v>25399</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -1558,7 +1566,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1581,7 +1589,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="n">
-        <v>10</v>
+        <v>25400</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -1660,7 +1668,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1683,7 +1691,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="n">
-        <v>11</v>
+        <v>25401</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -1762,7 +1770,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1785,7 +1793,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="n">
-        <v>12</v>
+        <v>25402</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -1864,7 +1872,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1887,7 +1895,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="n">
-        <v>13</v>
+        <v>25403</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -1966,7 +1974,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -1989,7 +1997,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="n">
-        <v>14</v>
+        <v>25404</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -2016,17 +2024,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 45.º-A</t>
+        </is>
+      </c>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Alarga o abono de família revendo os escalões de rendimento de referência do agregado familiar, pela alteração ao Decreto-Lei n.º 176/2003, de 2 de agosto</t>
+          <t>Artigo 45.º-A (Alarga o abono de família revendo os escalões de rendimento de referência do agregado familiar, pela alteração ao Decreto-Lei n.º 176/2003, de 2 de agosto)</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -2041,7 +2053,7 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr"/>
@@ -2068,7 +2080,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2091,7 +2103,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="n">
-        <v>15</v>
+        <v>25405</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -2170,7 +2182,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2193,7 +2205,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="n">
-        <v>16</v>
+        <v>25406</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -2272,7 +2284,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2295,7 +2307,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="n">
-        <v>17</v>
+        <v>25407</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -2374,7 +2386,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2397,7 +2409,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="n">
-        <v>18</v>
+        <v>25408</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -2424,17 +2436,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 115.º-B</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 115.º-B Residências modulares em instituições de Ensino Superior</t>
+          <t>Artigo 115.º-B (Residências modulares em instituições de Ensino Superior)</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
@@ -2449,7 +2465,7 @@
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr"/>
@@ -2476,7 +2492,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2499,7 +2515,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="n">
-        <v>19</v>
+        <v>25409</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -2526,17 +2542,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 122.º-A</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 122.º-A Criação do passe ‘’Vai e Vem’'</t>
+          <t>Artigo 122.º-A (Criação do passe ‘’Vai e Vem’')</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -2578,7 +2598,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2601,7 +2621,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="n">
-        <v>20</v>
+        <v>25410</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -2680,7 +2700,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2703,7 +2723,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="n">
-        <v>21</v>
+        <v>25411</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
@@ -2730,17 +2750,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 60.º-A</t>
+        </is>
+      </c>
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 60.º-A - Imposto Mínimo sobre Grandes Fortunas</t>
+          <t>Artigo 60.º-A (Imposto Mínimo sobre Grandes Fortunas)</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -2755,7 +2779,7 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R22" s="2" t="inlineStr"/>
@@ -2782,7 +2806,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2805,7 +2829,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="n">
-        <v>22</v>
+        <v>25412</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
@@ -2884,7 +2908,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -2907,7 +2931,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="n">
-        <v>23</v>
+        <v>25413</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
@@ -2986,7 +3010,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3009,7 +3033,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="2" t="n">
-        <v>24</v>
+        <v>25414</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -3088,7 +3112,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3111,7 +3135,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="n">
-        <v>25</v>
+        <v>25415</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -3190,7 +3214,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3213,7 +3237,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="n">
-        <v>26</v>
+        <v>25416</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
@@ -3292,7 +3316,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3315,7 +3339,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="n">
-        <v>27</v>
+        <v>25417</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -3394,7 +3418,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3417,7 +3441,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="2" t="n">
-        <v>28</v>
+        <v>25418</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -3444,17 +3468,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 45.º-A</t>
+        </is>
+      </c>
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Aumento da majoração para as famílias monoparentais do Abono de Família</t>
+          <t>Artigo 45.º-A (Aumento da majoração para as famílias monoparentais do Abono de Família)</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr">
@@ -3469,7 +3497,7 @@
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R29" s="2" t="inlineStr"/>
@@ -3496,7 +3524,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3519,7 +3547,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="2" t="n">
-        <v>29</v>
+        <v>25419</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -3598,7 +3626,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3621,7 +3649,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="2" t="n">
-        <v>30</v>
+        <v>25420</v>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
@@ -3648,17 +3676,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 19.º-A</t>
+        </is>
+      </c>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 19.º-A - Programa “Semana de quatro dias de trabalho na Administração Pública”</t>
+          <t>Artigo 19.º-A (Programa “Semana de quatro dias de trabalho na Administração Pública”)</t>
         </is>
       </c>
       <c r="O31" s="2" t="inlineStr">
@@ -3673,7 +3705,7 @@
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr"/>
@@ -3700,7 +3732,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3723,7 +3755,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="n">
-        <v>31</v>
+        <v>25421</v>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
@@ -3802,7 +3834,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3825,7 +3857,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr"/>
       <c r="D33" s="2" t="n">
-        <v>32</v>
+        <v>25422</v>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
@@ -3904,7 +3936,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -3927,7 +3959,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="2" t="n">
-        <v>33</v>
+        <v>25423</v>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
@@ -4006,7 +4038,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4041,11 +4073,7 @@
           <t>L</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
-        </is>
-      </c>
+      <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Comissão</t>
@@ -4056,24 +4084,24 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 4.º-A</t>
+        </is>
+      </c>
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 4.º-A - Cria o Serviço Nacional de Habitação</t>
-        </is>
-      </c>
-      <c r="O35" s="2" t="inlineStr">
-        <is>
-          <t>Infraestruturas, Mobilidade e Habitação</t>
-        </is>
-      </c>
+          <t>Artigo 4.º-A (Cria o Serviço Nacional de Habitação)</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr"/>
       <c r="P35" s="2" t="inlineStr">
         <is>
           <t>em apreciação</t>
@@ -4081,7 +4109,7 @@
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R35" s="2" t="inlineStr"/>
@@ -4108,7 +4136,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4143,11 +4171,7 @@
           <t>L</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
-        </is>
-      </c>
+      <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Comissão</t>
@@ -4158,24 +4182,24 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 45.º-A</t>
+        </is>
+      </c>
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 45.º-A Aumento do valor do Abono de Família em 10%</t>
-        </is>
-      </c>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>Trabalho, Segurança Social e Inclusão</t>
-        </is>
-      </c>
+          <t>Artigo 45.º-A (Aumento do valor do Abono de Família em 10%)</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr"/>
       <c r="P36" s="2" t="inlineStr">
         <is>
           <t>em apreciação</t>
@@ -4183,7 +4207,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R36" s="2" t="inlineStr"/>
@@ -4210,7 +4234,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4312,7 +4336,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4414,7 +4438,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4516,7 +4540,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4618,7 +4642,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4668,17 +4692,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 21.º-A</t>
+        </is>
+      </c>
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 21.º - A Reforça o recrutamento de médicos e enfermeiros especialistas com vista à reabertura das urgências de ginecologia e obstetrícia encerradas</t>
+          <t>Artigo 21.º-A (Reforça o recrutamento de médicos e enfermeiros especialistas com vista à reabertura das urgências de ginecologia e obstetrícia encerradas)</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
@@ -4693,7 +4721,7 @@
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R41" s="2" t="inlineStr"/>
@@ -4720,7 +4748,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4770,17 +4798,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 4.º-A</t>
+        </is>
+      </c>
       <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 4.º-A - Cria o Fundo para a Habitação Pública</t>
+          <t>Artigo 4.º-A (Cria o Fundo para a Habitação Pública)</t>
         </is>
       </c>
       <c r="O42" s="2" t="inlineStr">
@@ -4795,7 +4827,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr"/>
@@ -4822,7 +4854,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,7 +4956,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -4974,17 +5006,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 21.º-A</t>
+        </is>
+      </c>
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 21.º-A Contratação de psicólogos para instituições de Ensino Superior</t>
+          <t>Artigo 21.º-A (Contratação de psicólogos para instituições de Ensino Superior)</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
@@ -4999,7 +5035,7 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr"/>
@@ -5026,7 +5062,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5128,7 +5164,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5230,7 +5266,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5332,7 +5368,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5434,7 +5470,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5536,7 +5572,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5638,7 +5674,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5688,17 +5724,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 45.º-A</t>
+        </is>
+      </c>
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 45.º-A Clarifica o conceito de agregado familiar monoparental para atribuição da majoração do abono de família, alterando o Decreto-Lei n.º 176/2003, de 2 de agosto</t>
+          <t>Artigo 45.º-A (Clarifica o conceito de agregado familiar monoparental para atribuição da majoração do abono de família, alterando o Decreto-Lei n.º 176/2003, de 2 de agosto)</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr">
@@ -5713,7 +5753,7 @@
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R51" s="2" t="inlineStr"/>
@@ -5740,7 +5780,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5842,7 +5882,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5944,7 +5984,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6046,7 +6086,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6148,7 +6188,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6198,17 +6238,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 21.º-A</t>
+        </is>
+      </c>
       <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>Aumento da remuneração base do salário base dos quatro primeiros escalões dos Docentes da educação pré-escolar e dos ensinos básico e secundário - Artigo 21.º A</t>
+          <t>Artigo 21.º-A (Docentes da educação pré-escolar e dos ensinos básico e secundário)</t>
         </is>
       </c>
       <c r="O56" s="2" t="inlineStr">
@@ -6223,7 +6267,7 @@
       </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R56" s="2" t="inlineStr"/>
@@ -6250,7 +6294,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6352,7 +6396,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6402,12 +6446,16 @@
           <t>Mapas</t>
         </is>
       </c>
-      <c r="J58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 39.º-C</t>
+        </is>
+      </c>
       <c r="K58" s="2" t="inlineStr"/>
       <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -6427,7 +6475,7 @@
       </c>
       <c r="Q58" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R58" s="2" t="inlineStr"/>
@@ -6454,7 +6502,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6556,7 +6604,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6606,17 +6654,29 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 60.º</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Alteração ao Código do Imposto sobre o Rendimento das Pessoas Singulares</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Aprova o Código do Imposto sobre o Rendimento das Pessoas Singulares (IRS)</t>
+        </is>
+      </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Substituição</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>Artigo 60.º</t>
+          <t>N.º 1, Artigo 78.º do Código do IRS, constante do Artigo 60.º da PPL</t>
         </is>
       </c>
       <c r="O60" s="2" t="inlineStr">
@@ -6631,7 +6691,7 @@
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R60" s="2" t="inlineStr"/>
@@ -6658,7 +6718,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6760,7 +6820,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6862,7 +6922,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6937,7 +6997,7 @@
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Substituído(a)</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr"/>
@@ -6964,7 +7024,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7066,7 +7126,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7168,7 +7228,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7270,7 +7330,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7372,7 +7432,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7447,7 +7507,7 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Substituído(a)</t>
         </is>
       </c>
       <c r="R68" s="2" t="inlineStr"/>
@@ -7474,7 +7534,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7576,7 +7636,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7678,7 +7738,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7780,7 +7840,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7886,7 +7946,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7992,7 +8052,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8094,7 +8154,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8200,7 +8260,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8302,7 +8362,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8408,7 +8468,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8514,7 +8574,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8620,7 +8680,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,7 +8782,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8828,7 +8888,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8934,7 +8994,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9036,7 +9096,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9142,7 +9202,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9248,7 +9308,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9354,7 +9414,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9460,7 +9520,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9566,7 +9626,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9672,7 +9732,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9778,7 +9838,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9884,7 +9944,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9990,7 +10050,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10096,7 +10156,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10262,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31</t>
+          <t>2026-10-30 12:23</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10212,8 +10272,110 @@
       </c>
       <c r="AF94" s="2" t="inlineStr"/>
     </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>94C</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>94C</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr"/>
+      <c r="D95" s="2" t="n">
+        <v>25501</v>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 10:22</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr"/>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 43.º-A Programa-piloto do Rendimento Básico de Coesão</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>Economia e Coesão Territorial</t>
+        </is>
+      </c>
+      <c r="P95" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q95" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R95" s="2" t="inlineStr"/>
+      <c r="S95" s="2" t="inlineStr"/>
+      <c r="T95" s="2" t="inlineStr"/>
+      <c r="U95" s="2" t="inlineStr"/>
+      <c r="V95" s="2" t="inlineStr"/>
+      <c r="W95" s="2" t="inlineStr"/>
+      <c r="X95" s="2" t="inlineStr"/>
+      <c r="Y95" s="2" t="inlineStr"/>
+      <c r="Z95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA95" s="2" t="inlineStr"/>
+      <c r="AB95" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338355954686a4e6a63354d53303359574e694c5451344d6d59744f54686a4d4330775a5755304e446c6d4f574932597a4d756347526d&amp;Fich=9a8c6791-7acb-482f-98c0-0ee449f9b6c3.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 12:23</t>
+        </is>
+      </c>
+      <c r="AD95" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 12:23</t>
+        </is>
+      </c>
+      <c r="AE95" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF95" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF94"/>
+  <autoFilter ref="A1:AF95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10271,7 +10433,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31 UTC</t>
+          <t>2026-10-30 12:23 UTC</t>
         </is>
       </c>
     </row>
@@ -10283,7 +10445,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 07:31 UTC</t>
+          <t>2026-10-30 12:24 UTC</t>
         </is>
       </c>
     </row>
@@ -10294,7 +10456,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7">
@@ -10304,7 +10466,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-30 14:06 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF95"/>
+  <dimension ref="A1:AF97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3834,7 +3834,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="2" t="n">
-        <v>34</v>
+        <v>25424</v>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
@@ -4073,7 +4073,11 @@
           <t>L</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Comissão</t>
@@ -4101,7 +4105,11 @@
           <t>Artigo 4.º-A (Cria o Serviço Nacional de Habitação)</t>
         </is>
       </c>
-      <c r="O35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
           <t>em apreciação</t>
@@ -4136,7 +4144,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4159,7 +4167,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="2" t="n">
-        <v>35</v>
+        <v>25425</v>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
@@ -4171,7 +4179,11 @@
           <t>L</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Comissão</t>
@@ -4199,7 +4211,11 @@
           <t>Artigo 45.º-A (Aumento do valor do Abono de Família em 10%)</t>
         </is>
       </c>
-      <c r="O36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
           <t>em apreciação</t>
@@ -4234,7 +4250,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4257,7 +4273,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr"/>
       <c r="D37" s="2" t="n">
-        <v>36</v>
+        <v>25426</v>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
@@ -4336,7 +4352,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4359,7 +4375,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="n">
-        <v>37</v>
+        <v>25427</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
@@ -4438,7 +4454,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4461,7 +4477,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="2" t="n">
-        <v>38</v>
+        <v>25428</v>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
@@ -4540,7 +4556,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4563,7 +4579,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="n">
-        <v>39</v>
+        <v>25429</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
@@ -4642,7 +4658,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4665,7 +4681,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="2" t="n">
-        <v>40</v>
+        <v>25430</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
@@ -4748,7 +4764,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4771,7 +4787,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr"/>
       <c r="D42" s="2" t="n">
-        <v>41</v>
+        <v>25431</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
@@ -4854,7 +4870,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4877,7 +4893,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="2" t="n">
-        <v>42</v>
+        <v>25432</v>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
@@ -4956,7 +4972,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -4979,7 +4995,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="2" t="n">
-        <v>43</v>
+        <v>25433</v>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
@@ -5062,7 +5078,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5085,7 +5101,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="2" t="n">
-        <v>44</v>
+        <v>25434</v>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
@@ -5164,7 +5180,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5187,7 +5203,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="2" t="n">
-        <v>45</v>
+        <v>25435</v>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
@@ -5266,7 +5282,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5289,7 +5305,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="2" t="n">
-        <v>46</v>
+        <v>25436</v>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
@@ -5368,7 +5384,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5391,7 +5407,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="n">
-        <v>47</v>
+        <v>25437</v>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
@@ -5470,7 +5486,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5493,7 +5509,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr"/>
       <c r="D49" s="2" t="n">
-        <v>48</v>
+        <v>25438</v>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
@@ -5572,7 +5588,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5595,7 +5611,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="2" t="n">
-        <v>49</v>
+        <v>25439</v>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
@@ -5674,7 +5690,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5697,7 +5713,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="2" t="n">
-        <v>50</v>
+        <v>25440</v>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
@@ -5780,7 +5796,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5803,7 +5819,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="n">
-        <v>51</v>
+        <v>25441</v>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
@@ -5882,7 +5898,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -5905,7 +5921,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="2" t="n">
-        <v>52</v>
+        <v>25442</v>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
@@ -5984,7 +6000,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6007,7 +6023,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="2" t="n">
-        <v>53</v>
+        <v>25443</v>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
@@ -6086,7 +6102,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6109,7 +6125,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="2" t="n">
-        <v>54</v>
+        <v>25444</v>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
@@ -6188,7 +6204,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6211,7 +6227,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr"/>
       <c r="D56" s="2" t="n">
-        <v>55</v>
+        <v>25445</v>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
@@ -6294,7 +6310,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6317,7 +6333,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr"/>
       <c r="D57" s="2" t="n">
-        <v>56</v>
+        <v>25446</v>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
@@ -6396,7 +6412,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6419,7 +6435,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="2" t="n">
-        <v>57</v>
+        <v>25447</v>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
@@ -6502,7 +6518,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6525,7 +6541,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="2" t="n">
-        <v>58</v>
+        <v>25448</v>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
@@ -6604,7 +6620,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6627,7 +6643,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="2" t="n">
-        <v>59</v>
+        <v>25449</v>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
@@ -6718,7 +6734,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6741,7 +6757,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="2" t="n">
-        <v>60</v>
+        <v>25450</v>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
@@ -6820,7 +6836,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6843,7 +6859,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="2" t="n">
-        <v>61</v>
+        <v>25451</v>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
@@ -6922,7 +6938,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6945,7 +6961,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="2" t="n">
-        <v>62</v>
+        <v>25452</v>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
@@ -7024,7 +7040,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7047,7 +7063,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="n">
-        <v>63</v>
+        <v>25453</v>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
@@ -7126,7 +7142,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7149,7 +7165,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="2" t="n">
-        <v>64</v>
+        <v>25454</v>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
@@ -7228,7 +7244,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7251,7 +7267,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="2" t="n">
-        <v>65</v>
+        <v>25455</v>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
@@ -7330,7 +7346,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7353,7 +7369,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="2" t="n">
-        <v>66</v>
+        <v>25456</v>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
@@ -7432,7 +7448,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7455,7 +7471,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="2" t="n">
-        <v>67</v>
+        <v>25457</v>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
@@ -7534,7 +7550,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7557,7 +7573,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr"/>
       <c r="D69" s="2" t="n">
-        <v>68</v>
+        <v>25458</v>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
@@ -7636,7 +7652,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7659,7 +7675,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="2" t="n">
-        <v>69</v>
+        <v>25459</v>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
@@ -7738,7 +7754,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7761,7 +7777,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="2" t="n">
-        <v>70</v>
+        <v>25460</v>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
@@ -7840,7 +7856,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7863,7 +7879,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr"/>
       <c r="D72" s="2" t="n">
-        <v>71</v>
+        <v>25461</v>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
@@ -7925,11 +7941,7 @@
       <c r="V72" s="2" t="inlineStr"/>
       <c r="W72" s="2" t="inlineStr"/>
       <c r="X72" s="2" t="inlineStr"/>
-      <c r="Y72" s="2" t="inlineStr">
-        <is>
-          <t>01 - Encargos Gerais do Estado</t>
-        </is>
-      </c>
+      <c r="Y72" s="2" t="inlineStr"/>
       <c r="Z72" s="2" t="n">
         <v>0</v>
       </c>
@@ -7946,7 +7958,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -7969,7 +7981,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="2" t="n">
-        <v>72</v>
+        <v>25462</v>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
@@ -8031,11 +8043,7 @@
       <c r="V73" s="2" t="inlineStr"/>
       <c r="W73" s="2" t="inlineStr"/>
       <c r="X73" s="2" t="inlineStr"/>
-      <c r="Y73" s="2" t="inlineStr">
-        <is>
-          <t>07 - Ambiente, do Ordenamento do Território e do Desenvolvimento Regional</t>
-        </is>
-      </c>
+      <c r="Y73" s="2" t="inlineStr"/>
       <c r="Z73" s="2" t="n">
         <v>0</v>
       </c>
@@ -8052,7 +8060,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8075,7 +8083,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="2" t="n">
-        <v>73</v>
+        <v>25463</v>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
@@ -8154,7 +8162,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8177,7 +8185,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr"/>
       <c r="D75" s="2" t="n">
-        <v>74</v>
+        <v>25464</v>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
@@ -8239,11 +8247,7 @@
       <c r="V75" s="2" t="inlineStr"/>
       <c r="W75" s="2" t="inlineStr"/>
       <c r="X75" s="2" t="inlineStr"/>
-      <c r="Y75" s="2" t="inlineStr">
-        <is>
-          <t>07 - Ambiente, do Ordenamento do Território e do Desenvolvimento Regional</t>
-        </is>
-      </c>
+      <c r="Y75" s="2" t="inlineStr"/>
       <c r="Z75" s="2" t="n">
         <v>0</v>
       </c>
@@ -8260,7 +8264,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8283,7 +8287,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="2" t="n">
-        <v>75</v>
+        <v>25465</v>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
@@ -8362,7 +8366,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8385,7 +8389,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr"/>
       <c r="D77" s="2" t="n">
-        <v>76</v>
+        <v>25466</v>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
@@ -8447,11 +8451,7 @@
       <c r="V77" s="2" t="inlineStr"/>
       <c r="W77" s="2" t="inlineStr"/>
       <c r="X77" s="2" t="inlineStr"/>
-      <c r="Y77" s="2" t="inlineStr">
-        <is>
-          <t>10 - Obras Públicas, Transportes e Comunicações</t>
-        </is>
-      </c>
+      <c r="Y77" s="2" t="inlineStr"/>
       <c r="Z77" s="2" t="n">
         <v>0</v>
       </c>
@@ -8468,7 +8468,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8491,7 +8491,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr"/>
       <c r="D78" s="2" t="n">
-        <v>77</v>
+        <v>25467</v>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
@@ -8553,11 +8553,7 @@
       <c r="V78" s="2" t="inlineStr"/>
       <c r="W78" s="2" t="inlineStr"/>
       <c r="X78" s="2" t="inlineStr"/>
-      <c r="Y78" s="2" t="inlineStr">
-        <is>
-          <t>10 - Obras Públicas, Transportes e Comunicações</t>
-        </is>
-      </c>
+      <c r="Y78" s="2" t="inlineStr"/>
       <c r="Z78" s="2" t="n">
         <v>0</v>
       </c>
@@ -8574,7 +8570,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8597,7 +8593,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr"/>
       <c r="D79" s="2" t="n">
-        <v>78</v>
+        <v>25468</v>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
@@ -8659,11 +8655,7 @@
       <c r="V79" s="2" t="inlineStr"/>
       <c r="W79" s="2" t="inlineStr"/>
       <c r="X79" s="2" t="inlineStr"/>
-      <c r="Y79" s="2" t="inlineStr">
-        <is>
-          <t>11 - Trabalho e Solidariedade Social</t>
-        </is>
-      </c>
+      <c r="Y79" s="2" t="inlineStr"/>
       <c r="Z79" s="2" t="n">
         <v>0</v>
       </c>
@@ -8680,7 +8672,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8703,7 +8695,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr"/>
       <c r="D80" s="2" t="n">
-        <v>79</v>
+        <v>25469</v>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
@@ -8782,7 +8774,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8805,7 +8797,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr"/>
       <c r="D81" s="2" t="n">
-        <v>80</v>
+        <v>25470</v>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
@@ -8867,11 +8859,7 @@
       <c r="V81" s="2" t="inlineStr"/>
       <c r="W81" s="2" t="inlineStr"/>
       <c r="X81" s="2" t="inlineStr"/>
-      <c r="Y81" s="2" t="inlineStr">
-        <is>
-          <t>13 - Educação</t>
-        </is>
-      </c>
+      <c r="Y81" s="2" t="inlineStr"/>
       <c r="Z81" s="2" t="n">
         <v>0</v>
       </c>
@@ -8888,7 +8876,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8911,7 +8899,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr"/>
       <c r="D82" s="2" t="n">
-        <v>81</v>
+        <v>25471</v>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
@@ -8973,11 +8961,7 @@
       <c r="V82" s="2" t="inlineStr"/>
       <c r="W82" s="2" t="inlineStr"/>
       <c r="X82" s="2" t="inlineStr"/>
-      <c r="Y82" s="2" t="inlineStr">
-        <is>
-          <t>10 - Obras Públicas, Transportes e Comunicações</t>
-        </is>
-      </c>
+      <c r="Y82" s="2" t="inlineStr"/>
       <c r="Z82" s="2" t="n">
         <v>0</v>
       </c>
@@ -8994,7 +8978,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9017,7 +9001,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr"/>
       <c r="D83" s="2" t="n">
-        <v>82</v>
+        <v>25472</v>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
@@ -9096,7 +9080,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9119,7 +9103,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr"/>
       <c r="D84" s="2" t="n">
-        <v>83</v>
+        <v>25473</v>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
@@ -9181,11 +9165,7 @@
       <c r="V84" s="2" t="inlineStr"/>
       <c r="W84" s="2" t="inlineStr"/>
       <c r="X84" s="2" t="inlineStr"/>
-      <c r="Y84" s="2" t="inlineStr">
-        <is>
-          <t>10 - Obras Públicas, Transportes e Comunicações</t>
-        </is>
-      </c>
+      <c r="Y84" s="2" t="inlineStr"/>
       <c r="Z84" s="2" t="n">
         <v>0</v>
       </c>
@@ -9202,7 +9182,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9225,7 +9205,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr"/>
       <c r="D85" s="2" t="n">
-        <v>84</v>
+        <v>25474</v>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
@@ -9287,11 +9267,7 @@
       <c r="V85" s="2" t="inlineStr"/>
       <c r="W85" s="2" t="inlineStr"/>
       <c r="X85" s="2" t="inlineStr"/>
-      <c r="Y85" s="2" t="inlineStr">
-        <is>
-          <t>09 - Agricultura, Desenvolvimento Rural e Pescas</t>
-        </is>
-      </c>
+      <c r="Y85" s="2" t="inlineStr"/>
       <c r="Z85" s="2" t="n">
         <v>0</v>
       </c>
@@ -9308,7 +9284,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9331,7 +9307,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr"/>
       <c r="D86" s="2" t="n">
-        <v>85</v>
+        <v>25475</v>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
@@ -9393,11 +9369,7 @@
       <c r="V86" s="2" t="inlineStr"/>
       <c r="W86" s="2" t="inlineStr"/>
       <c r="X86" s="2" t="inlineStr"/>
-      <c r="Y86" s="2" t="inlineStr">
-        <is>
-          <t>01 - Encargos Gerais do Estado</t>
-        </is>
-      </c>
+      <c r="Y86" s="2" t="inlineStr"/>
       <c r="Z86" s="2" t="n">
         <v>0</v>
       </c>
@@ -9414,7 +9386,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9437,7 +9409,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr"/>
       <c r="D87" s="2" t="n">
-        <v>86</v>
+        <v>25476</v>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
@@ -9499,11 +9471,7 @@
       <c r="V87" s="2" t="inlineStr"/>
       <c r="W87" s="2" t="inlineStr"/>
       <c r="X87" s="2" t="inlineStr"/>
-      <c r="Y87" s="2" t="inlineStr">
-        <is>
-          <t>07 - Ambiente, do Ordenamento do Território e do Desenvolvimento Regional</t>
-        </is>
-      </c>
+      <c r="Y87" s="2" t="inlineStr"/>
       <c r="Z87" s="2" t="n">
         <v>0</v>
       </c>
@@ -9520,7 +9488,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9543,7 +9511,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr"/>
       <c r="D88" s="2" t="n">
-        <v>87</v>
+        <v>25477</v>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
@@ -9605,11 +9573,7 @@
       <c r="V88" s="2" t="inlineStr"/>
       <c r="W88" s="2" t="inlineStr"/>
       <c r="X88" s="2" t="inlineStr"/>
-      <c r="Y88" s="2" t="inlineStr">
-        <is>
-          <t>12 - Saúde</t>
-        </is>
-      </c>
+      <c r="Y88" s="2" t="inlineStr"/>
       <c r="Z88" s="2" t="n">
         <v>0</v>
       </c>
@@ -9626,7 +9590,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9649,7 +9613,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr"/>
       <c r="D89" s="2" t="n">
-        <v>88</v>
+        <v>25478</v>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
@@ -9711,11 +9675,7 @@
       <c r="V89" s="2" t="inlineStr"/>
       <c r="W89" s="2" t="inlineStr"/>
       <c r="X89" s="2" t="inlineStr"/>
-      <c r="Y89" s="2" t="inlineStr">
-        <is>
-          <t>15 - Cultura</t>
-        </is>
-      </c>
+      <c r="Y89" s="2" t="inlineStr"/>
       <c r="Z89" s="2" t="n">
         <v>0</v>
       </c>
@@ -9732,7 +9692,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9755,7 +9715,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr"/>
       <c r="D90" s="2" t="n">
-        <v>89</v>
+        <v>25479</v>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
@@ -9817,11 +9777,7 @@
       <c r="V90" s="2" t="inlineStr"/>
       <c r="W90" s="2" t="inlineStr"/>
       <c r="X90" s="2" t="inlineStr"/>
-      <c r="Y90" s="2" t="inlineStr">
-        <is>
-          <t>15 - Cultura</t>
-        </is>
-      </c>
+      <c r="Y90" s="2" t="inlineStr"/>
       <c r="Z90" s="2" t="n">
         <v>0</v>
       </c>
@@ -9838,7 +9794,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9861,7 +9817,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr"/>
       <c r="D91" s="2" t="n">
-        <v>90</v>
+        <v>25480</v>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
@@ -9923,11 +9879,7 @@
       <c r="V91" s="2" t="inlineStr"/>
       <c r="W91" s="2" t="inlineStr"/>
       <c r="X91" s="2" t="inlineStr"/>
-      <c r="Y91" s="2" t="inlineStr">
-        <is>
-          <t>12 - Saúde</t>
-        </is>
-      </c>
+      <c r="Y91" s="2" t="inlineStr"/>
       <c r="Z91" s="2" t="n">
         <v>0</v>
       </c>
@@ -9944,7 +9896,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9967,7 +9919,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr"/>
       <c r="D92" s="2" t="n">
-        <v>91</v>
+        <v>25481</v>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
@@ -10029,11 +9981,7 @@
       <c r="V92" s="2" t="inlineStr"/>
       <c r="W92" s="2" t="inlineStr"/>
       <c r="X92" s="2" t="inlineStr"/>
-      <c r="Y92" s="2" t="inlineStr">
-        <is>
-          <t>14 - Ciência, Tecnologia e Ensino Superior</t>
-        </is>
-      </c>
+      <c r="Y92" s="2" t="inlineStr"/>
       <c r="Z92" s="2" t="n">
         <v>0</v>
       </c>
@@ -10050,7 +9998,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10073,7 +10021,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr"/>
       <c r="D93" s="2" t="n">
-        <v>92</v>
+        <v>25482</v>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
@@ -10135,11 +10083,7 @@
       <c r="V93" s="2" t="inlineStr"/>
       <c r="W93" s="2" t="inlineStr"/>
       <c r="X93" s="2" t="inlineStr"/>
-      <c r="Y93" s="2" t="inlineStr">
-        <is>
-          <t>12 - Saúde</t>
-        </is>
-      </c>
+      <c r="Y93" s="2" t="inlineStr"/>
       <c r="Z93" s="2" t="n">
         <v>0</v>
       </c>
@@ -10156,7 +10100,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10179,7 +10123,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr"/>
       <c r="D94" s="2" t="n">
-        <v>93</v>
+        <v>25483</v>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
@@ -10241,11 +10185,7 @@
       <c r="V94" s="2" t="inlineStr"/>
       <c r="W94" s="2" t="inlineStr"/>
       <c r="X94" s="2" t="inlineStr"/>
-      <c r="Y94" s="2" t="inlineStr">
-        <is>
-          <t>12 - Saúde</t>
-        </is>
-      </c>
+      <c r="Y94" s="2" t="inlineStr"/>
       <c r="Z94" s="2" t="n">
         <v>0</v>
       </c>
@@ -10262,7 +10202,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10364,7 +10304,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23</t>
+          <t>2026-10-30 14:05</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10374,8 +10314,212 @@
       </c>
       <c r="AF95" s="2" t="inlineStr"/>
     </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>95C</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>95C</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr"/>
+      <c r="D96" s="2" t="n">
+        <v>25502</v>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 12:43</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 63.º-E - Reembolso de 100% do IVA na aquisição de bens alimentares essenciais por famílias em situação de pobreza</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q96" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R96" s="2" t="inlineStr"/>
+      <c r="S96" s="2" t="inlineStr"/>
+      <c r="T96" s="2" t="inlineStr"/>
+      <c r="U96" s="2" t="inlineStr"/>
+      <c r="V96" s="2" t="inlineStr"/>
+      <c r="W96" s="2" t="inlineStr"/>
+      <c r="X96" s="2" t="inlineStr"/>
+      <c r="Y96" s="2" t="inlineStr"/>
+      <c r="Z96" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA96" s="2" t="inlineStr"/>
+      <c r="AB96" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338774e4467355a474532595331685a5456684c5451305a5449744f54637a597931684e7a51314d546b325a6a4d794e4467756347526d&amp;Fich=0489da6a-ae5a-44e2-973c-a745196f3248.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 14:05</t>
+        </is>
+      </c>
+      <c r="AD96" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 14:05</t>
+        </is>
+      </c>
+      <c r="AE96" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>96C</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>96C</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr"/>
+      <c r="D97" s="2" t="n">
+        <v>25503</v>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 13:19</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr"/>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>104.º D - Comparticipação dos encargos com seguros de acidentes pessoais e responsabilidade civil para voluntários de Associações Zoófilas e Centros de Recolha Oficial de Animais (CROA)</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>Agricultura e Pescas</t>
+        </is>
+      </c>
+      <c r="P97" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q97" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R97" s="2" t="inlineStr"/>
+      <c r="S97" s="2" t="inlineStr"/>
+      <c r="T97" s="2" t="inlineStr"/>
+      <c r="U97" s="2" t="inlineStr"/>
+      <c r="V97" s="2" t="inlineStr"/>
+      <c r="W97" s="2" t="inlineStr"/>
+      <c r="X97" s="2" t="inlineStr"/>
+      <c r="Y97" s="2" t="inlineStr"/>
+      <c r="Z97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA97" s="2" t="inlineStr"/>
+      <c r="AB97" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533833597a466c5a5752684f43316d4d6a6b774c5451355a444974596a51314e43316c4e5745324e5455344e6a55324d5459756347526d&amp;Fich=7c1eeda8-f290-49d2-b454-e5a655865616.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 14:05</t>
+        </is>
+      </c>
+      <c r="AD97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 14:05</t>
+        </is>
+      </c>
+      <c r="AE97" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF97" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF95"/>
+  <autoFilter ref="A1:AF97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10433,7 +10577,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 12:23 UTC</t>
+          <t>2026-10-30 14:05 UTC</t>
         </is>
       </c>
     </row>
@@ -10445,7 +10589,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 12:24 UTC</t>
+          <t>2026-10-30 14:06 UTC</t>
         </is>
       </c>
     </row>
@@ -10456,7 +10600,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7">
@@ -10466,7 +10610,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-30 16:36 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF97"/>
+  <dimension ref="A1:AF101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Alberto Fonseca; António Rodrigues; Eva Brás Pinho; Francisco Pimentel; Hugo Carneiro; Hugo Soares; Nuno Jorge Gonçalves; Paulo Marcelo; João Pinho de Almeida; Paulo Núncio</t>
+          <t>Alberto Fonseca; António Rodrigues; Eva Brás Pinho; Francisco Pimentel; Hugo Carneiro; Hugo Soares; Nuno Jorge Gonçalves; Paulo Lopes Marcelo; João Pinho de Almeida; Paulo Núncio</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1922,12 +1922,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 63.º-B</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1947,7 +1951,7 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr"/>
@@ -1974,7 +1978,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2080,7 +2084,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2182,7 +2186,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2284,7 +2288,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2386,7 +2390,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2492,7 +2496,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2598,7 +2602,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2700,7 +2704,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2806,7 +2810,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2908,7 +2912,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3010,7 +3014,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3112,7 +3116,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3214,7 +3218,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3316,7 +3320,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3418,7 +3422,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3524,7 +3528,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3626,7 +3630,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3732,7 +3736,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3834,7 +3838,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3936,7 +3940,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4038,7 +4042,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4144,7 +4148,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4250,7 +4254,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4352,7 +4356,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4454,7 +4458,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4556,7 +4560,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4658,7 +4662,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4764,7 +4768,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4870,7 +4874,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4972,7 +4976,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5078,7 +5082,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5180,7 +5184,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5282,7 +5286,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5384,7 +5388,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5486,7 +5490,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5588,7 +5592,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5690,7 +5694,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5796,7 +5800,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5898,7 +5902,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -6000,7 +6004,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6102,7 +6106,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6204,7 +6208,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6310,7 +6314,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6360,17 +6364,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 62.º-A</t>
+        </is>
+      </c>
       <c r="K57" s="2" t="inlineStr"/>
       <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 62º-A - Alteração ao Código do Imposto sobre o Rendimento das Pessoas Coletivas - Elimina a redução de IRC para as grandes empresas</t>
+          <t>Artigo 62.º-A (Alteração ao Código do Imposto sobre o Rendimento das Pessoas Coletivas)</t>
         </is>
       </c>
       <c r="O57" s="2" t="inlineStr">
@@ -6385,7 +6393,7 @@
       </c>
       <c r="Q57" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R57" s="2" t="inlineStr"/>
@@ -6412,7 +6420,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6518,7 +6526,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6620,7 +6628,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6734,7 +6742,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6836,7 +6844,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6938,7 +6946,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -6988,17 +6996,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 19.º-A</t>
+        </is>
+      </c>
       <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 19.º - A - Aditamento ao Decreto-Lei n.º 89/2009, de 9 de abril - Permite que ambos os pais acompanhem a criança com doença oncológica, sem perda financeira, sempre que medicamente recomendado</t>
+          <t>Artigo 19.ª-A (Aditamento ao Decreto-Lei n.º 89/2009, de 9 de abril)</t>
         </is>
       </c>
       <c r="O63" s="2" t="inlineStr">
@@ -7013,7 +7025,7 @@
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>Substituído(a)</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr"/>
@@ -7040,7 +7052,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7090,17 +7102,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 22.º-A</t>
+        </is>
+      </c>
       <c r="K64" s="2" t="inlineStr"/>
       <c r="L64" s="2" t="inlineStr"/>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>Continuidade e Financiamento das Equipas Comunitárias de Saúde Mental - Artigo 22.º - A</t>
+          <t>Artigo 22.º-A (Continuidade e financiamento das Equipas Comunitárias de Saúde Mental)</t>
         </is>
       </c>
       <c r="O64" s="2" t="inlineStr">
@@ -7115,7 +7131,7 @@
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R64" s="2" t="inlineStr"/>
@@ -7142,7 +7158,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7192,17 +7208,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 62.º-A</t>
+        </is>
+      </c>
       <c r="K65" s="2" t="inlineStr"/>
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 62.º - A - Alteração ao Código do Imposto sobre o Valor Acrescentado (Retira a isenção do IVA aos artistas tauromáquicos)</t>
+          <t>Artigo 62.º-A (Alteração ao Código do Imposto sobre o Valor Acrescentado)</t>
         </is>
       </c>
       <c r="O65" s="2" t="inlineStr">
@@ -7217,7 +7237,7 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr"/>
@@ -7244,7 +7264,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7294,17 +7314,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 6.º-A</t>
+        </is>
+      </c>
       <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 6.º-A - Proteção das pessoas em vulnerabilidade habitacional e risco de despejo</t>
+          <t>Artigo 6.º-A (Proteção das pessoas em vulnerabilidade habitacional e risco de despejo)</t>
         </is>
       </c>
       <c r="O66" s="2" t="inlineStr">
@@ -7319,7 +7343,7 @@
       </c>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R66" s="2" t="inlineStr"/>
@@ -7346,7 +7370,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7448,7 +7472,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7550,7 +7574,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7652,7 +7676,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7754,7 +7778,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7856,7 +7880,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7958,7 +7982,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8060,7 +8084,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8162,7 +8186,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8264,7 +8288,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8366,7 +8390,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8416,17 +8440,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 38.º-A</t>
+        </is>
+      </c>
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr"/>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 38.º - A - Alteração ao Código do Trabalho - Alarga o direito dos trabalhadores a faltar nos casos de hospitalização domiciliária da criança</t>
+          <t>Artigo 38.º-A (Alteração ao Código do Trabalho)</t>
         </is>
       </c>
       <c r="O77" s="2" t="inlineStr">
@@ -8441,7 +8469,7 @@
       </c>
       <c r="Q77" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R77" s="2" t="inlineStr"/>
@@ -8468,7 +8496,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8570,7 +8598,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8672,7 +8700,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8722,12 +8750,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 63.º-C</t>
+        </is>
+      </c>
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr"/>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N80" s="2" t="inlineStr">
@@ -8774,7 +8806,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8824,17 +8856,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 22.º-A</t>
+        </is>
+      </c>
       <c r="K81" s="2" t="inlineStr"/>
       <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 22.º - A - Abertura de concursos em Medicina Geral e Familiar</t>
+          <t>Artigo 22.º-A (Abertura de concursos em Medicina Geral e Familiar)</t>
         </is>
       </c>
       <c r="O81" s="2" t="inlineStr">
@@ -8849,7 +8885,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R81" s="2" t="inlineStr"/>
@@ -8876,7 +8912,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8978,7 +9014,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9028,17 +9064,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 38.º-A</t>
+        </is>
+      </c>
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr"/>
       <c r="M83" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>NOVO] Artigo 38.º - A - Aditamento ao Decreto-Lei n.º 91/2009, de 9 de abril - Permite que ambos os pais acompanhem a criança com doença oncológica, sem perda financeira, sempre que medicamente recomendado</t>
+          <t>Artigo 38.º-A (Aditamento ao Decreto-Lei n.º 91/2009, de 9 de abril)</t>
         </is>
       </c>
       <c r="O83" s="2" t="inlineStr">
@@ -9053,7 +9093,7 @@
       </c>
       <c r="Q83" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R83" s="2" t="inlineStr"/>
@@ -9080,7 +9120,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9130,12 +9170,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 21.º-B</t>
+        </is>
+      </c>
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr"/>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N84" s="2" t="inlineStr">
@@ -9155,7 +9199,7 @@
       </c>
       <c r="Q84" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R84" s="2" t="inlineStr"/>
@@ -9182,7 +9226,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9284,7 +9328,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9386,7 +9430,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9436,17 +9480,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J87" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 62.º-A</t>
+        </is>
+      </c>
       <c r="K87" s="2" t="inlineStr"/>
       <c r="L87" s="2" t="inlineStr"/>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 62.º - A - Alteração ao Código do Imposto sobre o Valor Acrescentado (IVA Atos Veterinários)</t>
+          <t>Artigo 62.º-A (Alteração ao Código do Imposto sobre o Valor Acrescentado)</t>
         </is>
       </c>
       <c r="O87" s="2" t="inlineStr">
@@ -9461,7 +9509,7 @@
       </c>
       <c r="Q87" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R87" s="2" t="inlineStr"/>
@@ -9488,7 +9536,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9590,7 +9638,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9692,7 +9740,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9794,7 +9842,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9896,7 +9944,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -9946,17 +9994,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 62.º-A</t>
+        </is>
+      </c>
       <c r="K92" s="2" t="inlineStr"/>
       <c r="L92" s="2" t="inlineStr"/>
       <c r="M92" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 62.º-A Alteração ao Código do Imposto sobre o Rendimento das Pessoas Coletivas (Alarga a taxa reduzida de IRC das PME aos primeiros 100.000 € de lucro)</t>
+          <t>Artigo 62.º-A (Alteração ao Código do Imposto sobre o Rendimento das Pessoas Coletivas)</t>
         </is>
       </c>
       <c r="O92" s="2" t="inlineStr">
@@ -9971,7 +10023,7 @@
       </c>
       <c r="Q92" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R92" s="2" t="inlineStr"/>
@@ -9998,7 +10050,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10048,17 +10100,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J93" s="2" t="inlineStr"/>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 62.º-A</t>
+        </is>
+      </c>
       <c r="K93" s="2" t="inlineStr"/>
       <c r="L93" s="2" t="inlineStr"/>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 62.º-A Aditamento ao Código do Imposto sobre o Rendimento das Pessoas Coletivas (Condiciona a taxa reduzida de IRC à capitalização das empresas)</t>
+          <t>Artigo 62.º-A (Aditamento ao Código do Imposto sobre o Rendimento das Pessoas Coletivas)</t>
         </is>
       </c>
       <c r="O93" s="2" t="inlineStr">
@@ -10073,7 +10129,7 @@
       </c>
       <c r="Q93" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R93" s="2" t="inlineStr"/>
@@ -10100,7 +10156,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10202,7 +10258,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10304,7 +10360,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10406,7 +10462,7 @@
       </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE96" s="2" t="inlineStr">
@@ -10508,7 +10564,7 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05</t>
+          <t>2026-10-30 16:35</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
@@ -10518,8 +10574,416 @@
       </c>
       <c r="AF97" s="2" t="inlineStr"/>
     </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>97C</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>97C</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr"/>
+      <c r="D98" s="2" t="n">
+        <v>25504</v>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:10</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 127º-A Cadeias agroalimentares curtas</t>
+        </is>
+      </c>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>Agricultura e Pescas</t>
+        </is>
+      </c>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q98" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R98" s="2" t="inlineStr"/>
+      <c r="S98" s="2" t="inlineStr"/>
+      <c r="T98" s="2" t="inlineStr"/>
+      <c r="U98" s="2" t="inlineStr"/>
+      <c r="V98" s="2" t="inlineStr"/>
+      <c r="W98" s="2" t="inlineStr"/>
+      <c r="X98" s="2" t="inlineStr"/>
+      <c r="Y98" s="2" t="inlineStr"/>
+      <c r="Z98" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA98" s="2" t="inlineStr"/>
+      <c r="AB98" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338354e6d45305a6d4d344d69316c4e6a5a6b4c5451325a446774595755344e4331695a54686b596d45325a6a686b4e4745756347526d&amp;Fich=96a4fc82-e66d-46d8-ae84-be8dba6f8d4a.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:35</t>
+        </is>
+      </c>
+      <c r="AD98" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:35</t>
+        </is>
+      </c>
+      <c r="AE98" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>98C</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>98C</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr"/>
+      <c r="D99" s="2" t="n">
+        <v>25505</v>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:25</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr"/>
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr"/>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 38.º-A - Respostas de suporte habitacional (housing first) para pessoas em situação de sem-abrigo</t>
+        </is>
+      </c>
+      <c r="O99" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P99" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q99" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R99" s="2" t="inlineStr"/>
+      <c r="S99" s="2" t="inlineStr"/>
+      <c r="T99" s="2" t="inlineStr"/>
+      <c r="U99" s="2" t="inlineStr"/>
+      <c r="V99" s="2" t="inlineStr"/>
+      <c r="W99" s="2" t="inlineStr"/>
+      <c r="X99" s="2" t="inlineStr"/>
+      <c r="Y99" s="2" t="inlineStr"/>
+      <c r="Z99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA99" s="2" t="inlineStr"/>
+      <c r="AB99" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338355a6a6c6b5a4441304f5330794d5463774c545130597a4d744f444d324d4330784e4759314e6a517a5a5463775a4455756347526d&amp;Fich=9f9dd049-2170-44c3-8360-14f5643e70d5.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:35</t>
+        </is>
+      </c>
+      <c r="AD99" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:35</t>
+        </is>
+      </c>
+      <c r="AE99" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>99C</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>99C</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr"/>
+      <c r="D100" s="2" t="n">
+        <v>25506</v>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:28</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr"/>
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr"/>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 62.º - A Alteração ao Código do Imposto sobre o Valor Acrescentado</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P100" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q100" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R100" s="2" t="inlineStr"/>
+      <c r="S100" s="2" t="inlineStr"/>
+      <c r="T100" s="2" t="inlineStr"/>
+      <c r="U100" s="2" t="inlineStr"/>
+      <c r="V100" s="2" t="inlineStr"/>
+      <c r="W100" s="2" t="inlineStr"/>
+      <c r="X100" s="2" t="inlineStr"/>
+      <c r="Y100" s="2" t="inlineStr"/>
+      <c r="Z100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA100" s="2" t="inlineStr"/>
+      <c r="AB100" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4d445a695a6d4d774e7930334e7a5a694c5451354e6d55744f544e6c4f43316b4e6d59334d545931596d466a4d6a4d756347526d&amp;Fich=e06bfc07-776b-496e-93e8-d6f7165bac23.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:35</t>
+        </is>
+      </c>
+      <c r="AD100" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:35</t>
+        </is>
+      </c>
+      <c r="AE100" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>100C</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>100C</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr"/>
+      <c r="D101" s="2" t="n">
+        <v>25507</v>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:30</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr"/>
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 62.º-A (Alteração ao Código do IVA)</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P101" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q101" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R101" s="2" t="inlineStr"/>
+      <c r="S101" s="2" t="inlineStr"/>
+      <c r="T101" s="2" t="inlineStr"/>
+      <c r="U101" s="2" t="inlineStr"/>
+      <c r="V101" s="2" t="inlineStr"/>
+      <c r="W101" s="2" t="inlineStr"/>
+      <c r="X101" s="2" t="inlineStr"/>
+      <c r="Y101" s="2" t="inlineStr"/>
+      <c r="Z101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA101" s="2" t="inlineStr"/>
+      <c r="AB101" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338784f54526d5a544d345a4330345a4745314c5451304d7a6b74596a6c684d5330784d6a6b304d545a6d596a6c6c5a4445756347526d&amp;Fich=194fe38d-8da5-4439-b9a1-129416fb9ed1.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:35</t>
+        </is>
+      </c>
+      <c r="AD101" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:35</t>
+        </is>
+      </c>
+      <c r="AE101" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF101" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF97"/>
+  <autoFilter ref="A1:AF101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10577,7 +11041,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 14:05 UTC</t>
+          <t>2026-10-30 16:35 UTC</t>
         </is>
       </c>
     </row>
@@ -10589,7 +11053,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 14:06 UTC</t>
+          <t>2026-10-30 16:36 UTC</t>
         </is>
       </c>
     </row>
@@ -10600,7 +11064,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -10610,7 +11074,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-30 17:34 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF101"/>
+  <dimension ref="A1:AF111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,17 +690,25 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 91.º</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Fundo de Emergência Municipal</t>
+        </is>
+      </c>
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Números e Alíneas)</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Artigo 91.º (Fundo de Emergência Municipal)</t>
+          <t>N.º 5, Artigo 91.º</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -715,7 +723,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr"/>
@@ -742,7 +750,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -792,17 +800,25 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 80.º</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Montantes da participação das autarquias locais nos impostos do Estado</t>
+        </is>
+      </c>
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Substituição</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Alteração ao artigo 80.º</t>
+          <t>N.º 5, N.º10, Artigo 80.º</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -817,7 +833,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr"/>
@@ -844,7 +860,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -950,7 +966,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1056,7 +1072,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1158,7 +1174,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1260,7 +1276,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1362,7 +1378,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1412,17 +1428,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 89.º-A</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 89.º-A Garantia de apoio psicológico nas escolas</t>
+          <t>Artigo 89.º-A (Garantia de apoio psicológico nas escolas)</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1437,7 +1457,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr"/>
@@ -1464,7 +1484,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1566,7 +1586,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1668,7 +1688,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1718,17 +1738,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 115.º-A</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 115.º-A Criação do Plano Nacional para o Alojamento no Ensino Superior 2.0</t>
+          <t>Artigo 115.º-A (Criação do Plano Nacional para o Alojamento no Ensino Superior 2.0)</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1743,7 +1767,7 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr"/>
@@ -1770,7 +1794,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1820,17 +1844,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 120.º-A</t>
+        </is>
+      </c>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 120.º-A Rede Nacional de Bancos de Leite Materno</t>
+          <t>Artigo 120.º-A (Rede Nacional de Bancos de Leite Materno)</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -1845,7 +1873,7 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr"/>
@@ -1872,7 +1900,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -1978,7 +2006,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2084,7 +2112,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2186,7 +2214,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2288,7 +2316,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2338,12 +2366,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 104.º-C</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -2363,7 +2395,7 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R18" s="2" t="inlineStr"/>
@@ -2390,7 +2422,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2496,7 +2528,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2602,7 +2634,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2704,7 +2736,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2810,7 +2842,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2912,7 +2944,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3014,7 +3046,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3116,7 +3148,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3218,7 +3250,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3320,7 +3352,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3422,7 +3454,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3528,7 +3560,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3630,7 +3662,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3736,7 +3768,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3838,7 +3870,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3888,17 +3920,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 115.º-A</t>
+        </is>
+      </c>
       <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="inlineStr"/>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>«Artigo 115.º-A Criação do Plano Nacional para o Alojamento no Ensino Superior 2.0</t>
+          <t>Artigo 115.º-A (Criação do Plano Nacional para o Alojamento no Ensino Superior 2.0)</t>
         </is>
       </c>
       <c r="O33" s="2" t="inlineStr">
@@ -3913,7 +3949,7 @@
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr"/>
@@ -3940,7 +3976,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4042,7 +4078,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4148,7 +4184,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4254,7 +4290,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4356,7 +4392,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4406,17 +4442,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 110.º-A</t>
+        </is>
+      </c>
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 110.º-A - Retoma e alarga o Projeto-piloto da semana de quatro dias de trabalho no setor privado</t>
+          <t>Artigo 110.º-A (Retoma e alarga o Projeto-piloto da semana de quatro dias de trabalho no setor privado)</t>
         </is>
       </c>
       <c r="O38" s="2" t="inlineStr">
@@ -4431,7 +4471,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr"/>
@@ -4458,7 +4498,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4508,17 +4548,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 64.º-A</t>
+        </is>
+      </c>
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>Alteração ao Código do Imposto sobre o Valor Acrescentado</t>
+          <t>Artigo 64.º-A (Alteração ao Código do Imposto sobre o Valor Acrescentado)</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
@@ -4533,7 +4577,7 @@
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R39" s="2" t="inlineStr"/>
@@ -4560,7 +4604,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4610,17 +4654,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 64.º-A</t>
+        </is>
+      </c>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 64.º-A - Redução faseada da taxa de IVA</t>
+          <t>Artigo 64.º-A (Redução faseada da taxa de IVA)</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
@@ -4635,7 +4683,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R40" s="2" t="inlineStr"/>
@@ -4662,7 +4710,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4768,7 +4816,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4874,7 +4922,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -4924,17 +4972,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 64.º-A</t>
+        </is>
+      </c>
       <c r="K43" s="2" t="inlineStr"/>
       <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>Acompanhamento e fiscalização do IVA</t>
+          <t>Artigo 64.º-A (Acompanhamento e fiscalização do IVA)</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
@@ -4949,7 +5001,7 @@
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R43" s="2" t="inlineStr"/>
@@ -4976,7 +5028,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5082,7 +5134,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5132,17 +5184,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 118.°-A</t>
+        </is>
+      </c>
       <c r="K45" s="2" t="inlineStr"/>
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 118.° - A Reposição do orçamento para a promoção da saúde e prevenção da doença</t>
+          <t>Artigo 118.°-A (Reposição do orçamento para a promoção da saúde e prevenção da doença)</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
@@ -5157,7 +5213,7 @@
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr"/>
@@ -5184,7 +5240,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5234,17 +5290,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 122.º-A</t>
+        </is>
+      </c>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 122.º-A - Passe de Mobilidade Nacional</t>
+          <t>Artigo 122.º-A (Passe de Mobilidade Nacional)</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
@@ -5259,7 +5319,7 @@
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R46" s="2" t="inlineStr"/>
@@ -5286,7 +5346,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5336,17 +5396,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 122.º-A</t>
+        </is>
+      </c>
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 122.º-A - Reforço do Fundo para a Mobilidade e Transportes</t>
+          <t>Artigo 122.º-A (Reforço do Fundo para a Mobilidade e Transportes)</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
@@ -5361,7 +5425,7 @@
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R47" s="2" t="inlineStr"/>
@@ -5388,7 +5452,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5438,17 +5502,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 122.º-A</t>
+        </is>
+      </c>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>Reforço do Programa Incentiva +TP</t>
+          <t>Artigo 122.º-A (Reforço do Programa Incentiva+TP)</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
@@ -5463,7 +5531,7 @@
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R48" s="2" t="inlineStr"/>
@@ -5490,7 +5558,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5540,17 +5608,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 117.º-A</t>
+        </is>
+      </c>
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 117.º-A - Estratégia Nacional para a Recuperação e Reciclagem de Minerais Críticos 2050</t>
+          <t>Artigo 117.º-A (Estratégia Nacional para a Recuperação e Reciclagem de Minerais Críticos 2050)</t>
         </is>
       </c>
       <c r="O49" s="2" t="inlineStr">
@@ -5565,7 +5637,7 @@
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R49" s="2" t="inlineStr"/>
@@ -5592,7 +5664,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5694,7 +5766,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5800,7 +5872,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5902,7 +5974,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -6004,7 +6076,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6106,7 +6178,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6156,17 +6228,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 110.º-A</t>
+        </is>
+      </c>
       <c r="K55" s="2" t="inlineStr"/>
       <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 110.º-A - Retoma e alargamento do Programa 3C - Casa, Conforto e Clima</t>
+          <t>Artigo 110.º-A (Retoma e alargamento do Programa 3C - Casa, Conforto e Clima)</t>
         </is>
       </c>
       <c r="O55" s="2" t="inlineStr">
@@ -6181,7 +6257,7 @@
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R55" s="2" t="inlineStr"/>
@@ -6208,7 +6284,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6314,7 +6390,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6420,7 +6496,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6526,7 +6602,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6628,7 +6704,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6742,7 +6818,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6844,7 +6920,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -6894,17 +6970,29 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr"/>
-      <c r="K62" s="2" t="inlineStr"/>
-      <c r="L62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 60.º</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Alteração ao Código do Imposto sobre o Rendimento das Pessoas Singulares</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>Aprova o Código do Imposto sobre o Rendimento das Pessoas Singulares (IRS)</t>
+        </is>
+      </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Números e Alíneas)</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>Tributa em sede de IRS o saldo líquido obtido em jogos e apostas online - Artigo 60.º</t>
+          <t>Alínea f), N.º 1, N.º 5, N.º 6, N.º 7, N.º 8, N.º 9, Artigo 9.º do Código do IRS</t>
         </is>
       </c>
       <c r="O62" s="2" t="inlineStr">
@@ -6919,7 +7007,7 @@
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr"/>
@@ -6946,7 +7034,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -7052,7 +7140,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7158,7 +7246,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7264,7 +7352,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7370,7 +7458,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7420,17 +7508,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 110.º-A</t>
+        </is>
+      </c>
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr"/>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 110.º-A - Aumenta o período de apoio do Porta 65 - jovem</t>
+          <t>Artigo 110.º-A (Aumenta o período de apoio do Porta 65 - jovem)</t>
         </is>
       </c>
       <c r="O67" s="2" t="inlineStr">
@@ -7445,7 +7537,7 @@
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr"/>
@@ -7472,7 +7564,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7522,17 +7614,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 19.º-A</t>
+        </is>
+      </c>
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr"/>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 19.º - A - Aditamento ao Decreto-Lei n.º 89/2009, de 9 de abril - Alarga os direitos parentais em caso de doença ou acidente da criança</t>
+          <t>Artigo 19.º-A (Aditamento ao Decreto-Lei n.º 89/2009, de 9 de abril)</t>
         </is>
       </c>
       <c r="O68" s="2" t="inlineStr">
@@ -7547,7 +7643,7 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>Substituído(a)</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R68" s="2" t="inlineStr"/>
@@ -7574,7 +7670,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7676,7 +7772,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7778,7 +7874,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7880,7 +7976,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -7982,7 +8078,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8084,7 +8180,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8134,17 +8230,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 110.º-A</t>
+        </is>
+      </c>
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr"/>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>Programa Casas de Função - Artigo 110.º - A</t>
+          <t>Artigo 110.º-A (Programa Casas de Função)</t>
         </is>
       </c>
       <c r="O74" s="2" t="inlineStr">
@@ -8159,7 +8259,7 @@
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R74" s="2" t="inlineStr"/>
@@ -8186,7 +8286,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8236,12 +8336,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 104.º-B</t>
+        </is>
+      </c>
       <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr"/>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
@@ -8261,7 +8365,7 @@
       </c>
       <c r="Q75" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R75" s="2" t="inlineStr"/>
@@ -8288,7 +8392,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8338,17 +8442,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 115.º-A</t>
+        </is>
+      </c>
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 115.º-A - Língua Gestual Portuguesa nas Escolas</t>
+          <t>Artigo 115.º-A (Língua Gestual Portuguesa nas Escolas)</t>
         </is>
       </c>
       <c r="O76" s="2" t="inlineStr">
@@ -8363,7 +8471,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R76" s="2" t="inlineStr"/>
@@ -8390,7 +8498,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8496,7 +8604,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8546,12 +8654,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 63.º-D</t>
+        </is>
+      </c>
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N78" s="2" t="inlineStr">
@@ -8571,7 +8683,7 @@
       </c>
       <c r="Q78" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R78" s="2" t="inlineStr"/>
@@ -8598,7 +8710,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8648,12 +8760,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 65.º-A</t>
+        </is>
+      </c>
       <c r="K79" s="2" t="inlineStr"/>
       <c r="L79" s="2" t="inlineStr"/>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr">
@@ -8673,7 +8789,7 @@
       </c>
       <c r="Q79" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R79" s="2" t="inlineStr"/>
@@ -8700,7 +8816,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8779,7 +8895,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R80" s="2" t="inlineStr"/>
@@ -8806,7 +8922,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -8912,7 +9028,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -8962,12 +9078,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 127.º-A</t>
+        </is>
+      </c>
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr"/>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N82" s="2" t="inlineStr">
@@ -9014,7 +9134,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9120,7 +9240,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9226,7 +9346,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9328,7 +9448,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9378,12 +9498,16 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 116.º-A</t>
+        </is>
+      </c>
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr"/>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N86" s="2" t="inlineStr">
@@ -9403,7 +9527,7 @@
       </c>
       <c r="Q86" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R86" s="2" t="inlineStr"/>
@@ -9430,7 +9554,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9536,7 +9660,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9586,17 +9710,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 122.º-A</t>
+        </is>
+      </c>
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr"/>
       <c r="M88" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 122.º-A - Apoio para instalação de hangares de bicicletas em parques de estacionamento</t>
+          <t>Artigo 122.º-A (Apoio para instalação de hangares de bicicletas em parques de estacionamento)</t>
         </is>
       </c>
       <c r="O88" s="2" t="inlineStr">
@@ -9611,7 +9739,7 @@
       </c>
       <c r="Q88" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R88" s="2" t="inlineStr"/>
@@ -9638,7 +9766,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9688,17 +9816,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J89" s="2" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 64.º-A</t>
+        </is>
+      </c>
       <c r="K89" s="2" t="inlineStr"/>
       <c r="L89" s="2" t="inlineStr"/>
       <c r="M89" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N89" s="2" t="inlineStr">
         <is>
-          <t>PA - Aditamento - Redução da taxa normal do IVA de 23% para 22,5% - Artigo 64.º-A</t>
+          <t>Artigo 64.º-A (Alteração ao Código do Imposto sobre o Valor Acrescentado)</t>
         </is>
       </c>
       <c r="O89" s="2" t="inlineStr">
@@ -9713,7 +9845,7 @@
       </c>
       <c r="Q89" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R89" s="2" t="inlineStr"/>
@@ -9740,7 +9872,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9790,17 +9922,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 122.º-A</t>
+        </is>
+      </c>
       <c r="K90" s="2" t="inlineStr"/>
       <c r="L90" s="2" t="inlineStr"/>
       <c r="M90" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>[NOVO] Artigo 122.º-A - Projetos-piloto de logística urbana sustentável</t>
+          <t>Artigo 122.º-A (Projetos-piloto de logística urbana sustentável)</t>
         </is>
       </c>
       <c r="O90" s="2" t="inlineStr">
@@ -9815,7 +9951,7 @@
       </c>
       <c r="Q90" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R90" s="2" t="inlineStr"/>
@@ -9842,7 +9978,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -9892,17 +10028,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 85.º-A</t>
+        </is>
+      </c>
       <c r="K91" s="2" t="inlineStr"/>
       <c r="L91" s="2" t="inlineStr"/>
       <c r="M91" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>Valorização dos assistentes operacionais e assistentes técnicos nas escolas públicas - Artigo 85.º - A</t>
+          <t>Artigo 85.º-A (Valorização dos Assistentes Operacionais e Assistentes Técnicos nas escolas públicas)</t>
         </is>
       </c>
       <c r="O91" s="2" t="inlineStr">
@@ -9917,7 +10057,7 @@
       </c>
       <c r="Q91" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R91" s="2" t="inlineStr"/>
@@ -9944,7 +10084,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10050,7 +10190,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10156,7 +10296,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10206,17 +10346,21 @@
           <t>Articulado</t>
         </is>
       </c>
-      <c r="J94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 79.º-A</t>
+        </is>
+      </c>
       <c r="K94" s="2" t="inlineStr"/>
       <c r="L94" s="2" t="inlineStr"/>
       <c r="M94" s="2" t="inlineStr">
         <is>
-          <t>Por Definir</t>
+          <t>Aditamento (Artigo PPL)</t>
         </is>
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>NOVO] Artigo 79.º-A Revogação do regime de autorização de residência para atividade de investimento</t>
+          <t>Artigo 79.º-A (Revogação do regime de autorização de residência para atividade de investimento)</t>
         </is>
       </c>
       <c r="O94" s="2" t="inlineStr">
@@ -10231,7 +10375,7 @@
       </c>
       <c r="Q94" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R94" s="2" t="inlineStr"/>
@@ -10258,7 +10402,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10360,7 +10504,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10462,7 +10606,7 @@
       </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE96" s="2" t="inlineStr">
@@ -10564,7 +10708,7 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
@@ -10639,7 +10783,7 @@
       </c>
       <c r="Q98" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R98" s="2" t="inlineStr"/>
@@ -10666,7 +10810,7 @@
       </c>
       <c r="AD98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE98" s="2" t="inlineStr">
@@ -10741,7 +10885,7 @@
       </c>
       <c r="Q99" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R99" s="2" t="inlineStr"/>
@@ -10768,7 +10912,7 @@
       </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE99" s="2" t="inlineStr">
@@ -10843,7 +10987,7 @@
       </c>
       <c r="Q100" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R100" s="2" t="inlineStr"/>
@@ -10870,7 +11014,7 @@
       </c>
       <c r="AD100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE100" s="2" t="inlineStr">
@@ -10945,7 +11089,7 @@
       </c>
       <c r="Q101" s="2" t="inlineStr">
         <is>
-          <t>Entrada (via IPA)</t>
+          <t>Admitida</t>
         </is>
       </c>
       <c r="R101" s="2" t="inlineStr"/>
@@ -10972,7 +11116,7 @@
       </c>
       <c r="AD101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35</t>
+          <t>2026-10-30 17:33</t>
         </is>
       </c>
       <c r="AE101" s="2" t="inlineStr">
@@ -10982,8 +11126,1028 @@
       </c>
       <c r="AF101" s="2" t="inlineStr"/>
     </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>101C</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>101C</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr"/>
+      <c r="D102" s="2" t="n">
+        <v>25508</v>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:32</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr"/>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr"/>
+      <c r="M102" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 134.º-A (Plano Nacional de Combate à Violência Sexual Baseada em Imagens)</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P102" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q102" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R102" s="2" t="inlineStr"/>
+      <c r="S102" s="2" t="inlineStr"/>
+      <c r="T102" s="2" t="inlineStr"/>
+      <c r="U102" s="2" t="inlineStr"/>
+      <c r="V102" s="2" t="inlineStr"/>
+      <c r="W102" s="2" t="inlineStr"/>
+      <c r="X102" s="2" t="inlineStr"/>
+      <c r="Y102" s="2" t="inlineStr"/>
+      <c r="Z102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA102" s="2" t="inlineStr"/>
+      <c r="AB102" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338315a6a51784d6a63314d5330314e4455304c5452694d6a67744f44566d4d4330335a444d315a6a426a4f44646b4f546b756347526d&amp;Fich=5f412751-5454-4b28-85f0-7d35f0c87d99.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE102" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF102" s="2" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>102C</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>102C</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr"/>
+      <c r="D103" s="2" t="n">
+        <v>25509</v>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:33</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr"/>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr"/>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 134.º-A Atualização do Cartão Social Eletrônico</t>
+        </is>
+      </c>
+      <c r="O103" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P103" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q103" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R103" s="2" t="inlineStr"/>
+      <c r="S103" s="2" t="inlineStr"/>
+      <c r="T103" s="2" t="inlineStr"/>
+      <c r="U103" s="2" t="inlineStr"/>
+      <c r="V103" s="2" t="inlineStr"/>
+      <c r="W103" s="2" t="inlineStr"/>
+      <c r="X103" s="2" t="inlineStr"/>
+      <c r="Y103" s="2" t="inlineStr"/>
+      <c r="Z103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA103" s="2" t="inlineStr"/>
+      <c r="AB103" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324e6a466a4e6a4668596930795a57566a4c5451784e575974596a4d354e43316a4d6a67794f5455315a475934596d55756347526d&amp;Fich=661c61ab-2eec-415f-b394-c282955df8be.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD103" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE103" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF103" s="2" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>103C</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>103C</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr"/>
+      <c r="D104" s="2" t="n">
+        <v>25510</v>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:33</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr"/>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 38.º-A (Atualização do Programa Cartões Sociais)</t>
+        </is>
+      </c>
+      <c r="O104" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P104" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q104" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R104" s="2" t="inlineStr"/>
+      <c r="S104" s="2" t="inlineStr"/>
+      <c r="T104" s="2" t="inlineStr"/>
+      <c r="U104" s="2" t="inlineStr"/>
+      <c r="V104" s="2" t="inlineStr"/>
+      <c r="W104" s="2" t="inlineStr"/>
+      <c r="X104" s="2" t="inlineStr"/>
+      <c r="Y104" s="2" t="inlineStr"/>
+      <c r="Z104" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA104" s="2" t="inlineStr"/>
+      <c r="AB104" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338334e5755324d44497a4d5331694e54646b4c54526d597a4d744f54517a4e7930344f4459345a5463794d7a517a4f5451756347526d&amp;Fich=75e60231-b57d-4fc3-9437-8868e7234394.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD104" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE104" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>104C</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>104C</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr"/>
+      <c r="D105" s="2" t="n">
+        <v>25511</v>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:35</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>Mapas</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr"/>
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr"/>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 38.º-B (Financiamento das cantinas sociais)</t>
+        </is>
+      </c>
+      <c r="O105" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P105" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q105" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R105" s="2" t="inlineStr"/>
+      <c r="S105" s="2" t="inlineStr"/>
+      <c r="T105" s="2" t="inlineStr"/>
+      <c r="U105" s="2" t="inlineStr"/>
+      <c r="V105" s="2" t="inlineStr"/>
+      <c r="W105" s="2" t="inlineStr"/>
+      <c r="X105" s="2" t="inlineStr"/>
+      <c r="Y105" s="2" t="inlineStr"/>
+      <c r="Z105" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA105" s="2" t="inlineStr"/>
+      <c r="AB105" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4e6d4e6d597a6b775953316b4d7a686c4c5451334d7a5574596a6c694e43316a597a4d354d6d4d355a6d51354f5755756347526d&amp;Fich=e6cfc90a-d38e-4735-b9b4-cc392c9fd99e.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE105" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF105" s="2" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>105C</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>105C</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr"/>
+      <c r="D106" s="2" t="n">
+        <v>25512</v>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:36</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr"/>
+      <c r="K106" s="2" t="inlineStr"/>
+      <c r="L106" s="2" t="inlineStr"/>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 38.º-C (Reforço extraordinário dos apoios para crianças e famílias em situação de vulnerabilidade)</t>
+        </is>
+      </c>
+      <c r="O106" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P106" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q106" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R106" s="2" t="inlineStr"/>
+      <c r="S106" s="2" t="inlineStr"/>
+      <c r="T106" s="2" t="inlineStr"/>
+      <c r="U106" s="2" t="inlineStr"/>
+      <c r="V106" s="2" t="inlineStr"/>
+      <c r="W106" s="2" t="inlineStr"/>
+      <c r="X106" s="2" t="inlineStr"/>
+      <c r="Y106" s="2" t="inlineStr"/>
+      <c r="Z106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA106" s="2" t="inlineStr"/>
+      <c r="AB106" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4d32566b596a566c4d79316b597a5a694c5451354d5463744f47566b4f5330774e7a63774d7a646b4d7a59314e6d59756347526d&amp;Fich=f3edb5e3-dc6b-4917-8ed9-077037d3656f.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE106" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>106C</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>106C</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr"/>
+      <c r="D107" s="2" t="n">
+        <v>25513</v>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:37</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>PAN</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Inês de Sousa Real</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr"/>
+      <c r="K107" s="2" t="inlineStr"/>
+      <c r="L107" s="2" t="inlineStr"/>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>Artigo.º 116</t>
+        </is>
+      </c>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t>Educação e Ciência</t>
+        </is>
+      </c>
+      <c r="P107" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q107" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R107" s="2" t="inlineStr"/>
+      <c r="S107" s="2" t="inlineStr"/>
+      <c r="T107" s="2" t="inlineStr"/>
+      <c r="U107" s="2" t="inlineStr"/>
+      <c r="V107" s="2" t="inlineStr"/>
+      <c r="W107" s="2" t="inlineStr"/>
+      <c r="X107" s="2" t="inlineStr"/>
+      <c r="Y107" s="2" t="inlineStr"/>
+      <c r="Z107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA107" s="2" t="inlineStr"/>
+      <c r="AB107" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338325a6d566a4e4455334e79307a595459324c54526c4e574d745954526b5a4330775a475a684d474577597a566b4d4445756347526d&amp;Fich=6fec4577-3a66-4e5c-a4dd-0dfa0a0c5d01.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE107" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF107" s="2" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>107C</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>107C</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr"/>
+      <c r="D108" s="2" t="n">
+        <v>25514</v>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:40</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr"/>
+      <c r="K108" s="2" t="inlineStr"/>
+      <c r="L108" s="2" t="inlineStr"/>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 134.º-A Fiscalização da informação de preços ao consumidor</t>
+        </is>
+      </c>
+      <c r="O108" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P108" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q108" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R108" s="2" t="inlineStr"/>
+      <c r="S108" s="2" t="inlineStr"/>
+      <c r="T108" s="2" t="inlineStr"/>
+      <c r="U108" s="2" t="inlineStr"/>
+      <c r="V108" s="2" t="inlineStr"/>
+      <c r="W108" s="2" t="inlineStr"/>
+      <c r="X108" s="2" t="inlineStr"/>
+      <c r="Y108" s="2" t="inlineStr"/>
+      <c r="Z108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA108" s="2" t="inlineStr"/>
+      <c r="AB108" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338795a4467354e44686a4f53307a4f5449344c5451795a5449744f545530596930354d6a5134597a6b774e4746684e4451756347526d&amp;Fich=2d8948c9-3928-42e2-954b-9248c904aa44.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE108" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>108C</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>108C</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr"/>
+      <c r="D109" s="2" t="n">
+        <v>25515</v>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:51</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr"/>
+      <c r="K109" s="2" t="inlineStr"/>
+      <c r="L109" s="2" t="inlineStr"/>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 135.º-A Aditamento ao Decreto-Lei n.º 138/90, de 26 de abril</t>
+        </is>
+      </c>
+      <c r="O109" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P109" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q109" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R109" s="2" t="inlineStr"/>
+      <c r="S109" s="2" t="inlineStr"/>
+      <c r="T109" s="2" t="inlineStr"/>
+      <c r="U109" s="2" t="inlineStr"/>
+      <c r="V109" s="2" t="inlineStr"/>
+      <c r="W109" s="2" t="inlineStr"/>
+      <c r="X109" s="2" t="inlineStr"/>
+      <c r="Y109" s="2" t="inlineStr"/>
+      <c r="Z109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA109" s="2" t="inlineStr"/>
+      <c r="AB109" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a4d3245774e7a5178595331684d5442684c54517a4d6a6b744f575177597930354f5746694f4463774f4464694d6a45756347526d&amp;Fich=33a0741a-a10a-4329-9d0c-99ab87087b21.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE109" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF109" s="2" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>109C</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>109C</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr"/>
+      <c r="D110" s="2" t="n">
+        <v>25516</v>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:56</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr"/>
+      <c r="K110" s="2" t="inlineStr"/>
+      <c r="L110" s="2" t="inlineStr"/>
+      <c r="M110" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 22.º - A Contabilização da experiência no ingresso nas carreiras especiais do Serviço Nacional de Saúde</t>
+        </is>
+      </c>
+      <c r="O110" s="2" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="P110" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q110" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R110" s="2" t="inlineStr"/>
+      <c r="S110" s="2" t="inlineStr"/>
+      <c r="T110" s="2" t="inlineStr"/>
+      <c r="U110" s="2" t="inlineStr"/>
+      <c r="V110" s="2" t="inlineStr"/>
+      <c r="W110" s="2" t="inlineStr"/>
+      <c r="X110" s="2" t="inlineStr"/>
+      <c r="Y110" s="2" t="inlineStr"/>
+      <c r="Z110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA110" s="2" t="inlineStr"/>
+      <c r="AB110" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d324d7a4f4463305979316c5a6a5a684c5451795a444174595442695a4331694e6a51304f446b795a546b32597a55756347526d&amp;Fich=83c3874c-ef6a-42d0-a0bd-b644892e96c5.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD110" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE110" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>110C</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>110C</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr"/>
+      <c r="D111" s="2" t="n">
+        <v>25517</v>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 16:59</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr"/>
+      <c r="K111" s="2" t="inlineStr"/>
+      <c r="L111" s="2" t="inlineStr"/>
+      <c r="M111" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N111" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 45.º-A Cria a Rede Pública de Residências para as Pessoas Mais Velhas</t>
+        </is>
+      </c>
+      <c r="O111" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P111" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q111" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R111" s="2" t="inlineStr"/>
+      <c r="S111" s="2" t="inlineStr"/>
+      <c r="T111" s="2" t="inlineStr"/>
+      <c r="U111" s="2" t="inlineStr"/>
+      <c r="V111" s="2" t="inlineStr"/>
+      <c r="W111" s="2" t="inlineStr"/>
+      <c r="X111" s="2" t="inlineStr"/>
+      <c r="Y111" s="2" t="inlineStr"/>
+      <c r="Z111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA111" s="2" t="inlineStr"/>
+      <c r="AB111" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324f5745784d7a55784e69316a4d444a6d4c54526c597a55744f5468694d69307a596a41774d575977596a4268596a67756347526d&amp;Fich=69a13516-c02f-4ec5-98b2-3b001f0b0ab8.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AD111" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:33</t>
+        </is>
+      </c>
+      <c r="AE111" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF111" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF101"/>
+  <autoFilter ref="A1:AF111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11041,7 +12205,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 16:35 UTC</t>
+          <t>2026-10-30 17:33 UTC</t>
         </is>
       </c>
     </row>
@@ -11053,7 +12217,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 16:36 UTC</t>
+          <t>2026-10-30 17:33 UTC</t>
         </is>
       </c>
     </row>
@@ -11064,7 +12228,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7">
@@ -11074,7 +12238,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-30 18:52 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF111"/>
+  <dimension ref="A1:AF121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr"/>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="Q82" s="2" t="inlineStr">
         <is>
-          <t>Admitida</t>
+          <t>Aguarda Voto em Comissão</t>
         </is>
       </c>
       <c r="R82" s="2" t="inlineStr"/>
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10504,7 +10504,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE96" s="2" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
@@ -10810,7 +10810,7 @@
       </c>
       <c r="AD98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE98" s="2" t="inlineStr">
@@ -10912,7 +10912,7 @@
       </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE99" s="2" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="AD100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE100" s="2" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="AD101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE101" s="2" t="inlineStr">
@@ -11218,7 +11218,7 @@
       </c>
       <c r="AD102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE102" s="2" t="inlineStr">
@@ -11320,7 +11320,7 @@
       </c>
       <c r="AD103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE103" s="2" t="inlineStr">
@@ -11422,7 +11422,7 @@
       </c>
       <c r="AD104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE104" s="2" t="inlineStr">
@@ -11524,7 +11524,7 @@
       </c>
       <c r="AD105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE105" s="2" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="AD106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE106" s="2" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="AD107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE107" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="AD108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE108" s="2" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="AD109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE109" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="AD110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE110" s="2" t="inlineStr">
@@ -12136,7 +12136,7 @@
       </c>
       <c r="AD111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33</t>
+          <t>2026-10-30 18:51</t>
         </is>
       </c>
       <c r="AE111" s="2" t="inlineStr">
@@ -12146,8 +12146,988 @@
       </c>
       <c r="AF111" s="2" t="inlineStr"/>
     </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>111C</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>111C</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr"/>
+      <c r="D112" s="2" t="n">
+        <v>25518</v>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:36</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr"/>
+      <c r="K112" s="2" t="inlineStr"/>
+      <c r="L112" s="2" t="inlineStr"/>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N112" s="2" t="inlineStr"/>
+      <c r="O112" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P112" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q112" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R112" s="2" t="inlineStr"/>
+      <c r="S112" s="2" t="inlineStr"/>
+      <c r="T112" s="2" t="inlineStr"/>
+      <c r="U112" s="2" t="inlineStr"/>
+      <c r="V112" s="2" t="inlineStr"/>
+      <c r="W112" s="2" t="inlineStr"/>
+      <c r="X112" s="2" t="inlineStr"/>
+      <c r="Y112" s="2" t="inlineStr"/>
+      <c r="Z112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA112" s="2" t="inlineStr"/>
+      <c r="AB112" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338354f5449334e7a6c6d597930785932466c4c5451314e544d744f54417a4e6930345a6a63304d32466c4e545668597a59756347526d&amp;Fich=992779fc-1cae-4553-9036-8f743ae55ac6.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE112" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>112C</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>112C</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr"/>
+      <c r="D113" s="2" t="n">
+        <v>25519</v>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:37</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr"/>
+      <c r="K113" s="2" t="inlineStr"/>
+      <c r="L113" s="2" t="inlineStr"/>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N113" s="2" t="inlineStr"/>
+      <c r="O113" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação; Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P113" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q113" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R113" s="2" t="inlineStr"/>
+      <c r="S113" s="2" t="inlineStr"/>
+      <c r="T113" s="2" t="inlineStr"/>
+      <c r="U113" s="2" t="inlineStr"/>
+      <c r="V113" s="2" t="inlineStr"/>
+      <c r="W113" s="2" t="inlineStr"/>
+      <c r="X113" s="2" t="inlineStr"/>
+      <c r="Y113" s="2" t="inlineStr"/>
+      <c r="Z113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA113" s="2" t="inlineStr"/>
+      <c r="AB113" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4e6a41775a6a5a6b4f5330345a6a637a4c5451794e6a417459546b795969316b4e6a5a6d596d55324d6a426d4e6d59756347526d&amp;Fich=e600f6d9-8f73-4260-a92b-d66fbe620f6f.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE113" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF113" s="2" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>113C</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>113C</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr"/>
+      <c r="D114" s="2" t="n">
+        <v>25520</v>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:38</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr"/>
+      <c r="K114" s="2" t="inlineStr"/>
+      <c r="L114" s="2" t="inlineStr"/>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N114" s="2" t="inlineStr"/>
+      <c r="O114" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P114" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q114" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R114" s="2" t="inlineStr"/>
+      <c r="S114" s="2" t="inlineStr"/>
+      <c r="T114" s="2" t="inlineStr"/>
+      <c r="U114" s="2" t="inlineStr"/>
+      <c r="V114" s="2" t="inlineStr"/>
+      <c r="W114" s="2" t="inlineStr"/>
+      <c r="X114" s="2" t="inlineStr"/>
+      <c r="Y114" s="2" t="inlineStr"/>
+      <c r="Z114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA114" s="2" t="inlineStr"/>
+      <c r="AB114" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a5a6a4d77595467304f43303359546c6c4c54526d4d4755744f444d355a69316a4e474d334f5749304d54526c4f4463756347526d&amp;Fich=cf30a848-7a9e-4f0e-839f-c4c79b414e87.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD114" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE114" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>114C</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>114C</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr"/>
+      <c r="D115" s="2" t="n">
+        <v>25521</v>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:39</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="inlineStr"/>
+      <c r="K115" s="2" t="inlineStr"/>
+      <c r="L115" s="2" t="inlineStr"/>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N115" s="2" t="inlineStr"/>
+      <c r="O115" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P115" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q115" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R115" s="2" t="inlineStr"/>
+      <c r="S115" s="2" t="inlineStr"/>
+      <c r="T115" s="2" t="inlineStr"/>
+      <c r="U115" s="2" t="inlineStr"/>
+      <c r="V115" s="2" t="inlineStr"/>
+      <c r="W115" s="2" t="inlineStr"/>
+      <c r="X115" s="2" t="inlineStr"/>
+      <c r="Y115" s="2" t="inlineStr"/>
+      <c r="Z115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA115" s="2" t="inlineStr"/>
+      <c r="AB115" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d4451325a4467314d5330344e7a4d334c5452684e57517459545934596931694d5745355a446c695a4751314d5455756347526d&amp;Fich=8046d851-8737-4a5d-a68b-b1a9d9bdd515.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD115" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE115" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF115" s="2" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>115C</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>115C</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr"/>
+      <c r="D116" s="2" t="n">
+        <v>25522</v>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:40</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="inlineStr"/>
+      <c r="K116" s="2" t="inlineStr"/>
+      <c r="L116" s="2" t="inlineStr"/>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N116" s="2" t="inlineStr"/>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P116" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q116" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R116" s="2" t="inlineStr"/>
+      <c r="S116" s="2" t="inlineStr"/>
+      <c r="T116" s="2" t="inlineStr"/>
+      <c r="U116" s="2" t="inlineStr"/>
+      <c r="V116" s="2" t="inlineStr"/>
+      <c r="W116" s="2" t="inlineStr"/>
+      <c r="X116" s="2" t="inlineStr"/>
+      <c r="Y116" s="2" t="inlineStr"/>
+      <c r="Z116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA116" s="2" t="inlineStr"/>
+      <c r="AB116" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533878596a466a5a6a55325a6931685a44646c4c5451354d6a4574595449334e53316d4e7a4d794f5745324f4755304f5445756347526d&amp;Fich=1b1cf56f-ad7e-4921-a275-f7329a68e491.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE116" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF116" s="2" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>116C</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>116C</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr"/>
+      <c r="D117" s="2" t="n">
+        <v>25523</v>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:41</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr"/>
+      <c r="K117" s="2" t="inlineStr"/>
+      <c r="L117" s="2" t="inlineStr"/>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N117" s="2" t="inlineStr"/>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>Economia e Coesão Territorial</t>
+        </is>
+      </c>
+      <c r="P117" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q117" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R117" s="2" t="inlineStr"/>
+      <c r="S117" s="2" t="inlineStr"/>
+      <c r="T117" s="2" t="inlineStr"/>
+      <c r="U117" s="2" t="inlineStr"/>
+      <c r="V117" s="2" t="inlineStr"/>
+      <c r="W117" s="2" t="inlineStr"/>
+      <c r="X117" s="2" t="inlineStr"/>
+      <c r="Y117" s="2" t="inlineStr"/>
+      <c r="Z117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA117" s="2" t="inlineStr"/>
+      <c r="AB117" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324e445a6b4e445178597930334e5759794c54526b4f544d74596d4d7a4d5330304e6d4a694d6d45304d446b32595463756347526d&amp;Fich=646d441c-75f2-4d93-bc31-46bb2a4096a7.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD117" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE117" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF117" s="2" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>117C</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>117C</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr"/>
+      <c r="D118" s="2" t="n">
+        <v>25524</v>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:43</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr"/>
+      <c r="K118" s="2" t="inlineStr"/>
+      <c r="L118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N118" s="2" t="inlineStr"/>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>Ambiente e Energia</t>
+        </is>
+      </c>
+      <c r="P118" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q118" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R118" s="2" t="inlineStr"/>
+      <c r="S118" s="2" t="inlineStr"/>
+      <c r="T118" s="2" t="inlineStr"/>
+      <c r="U118" s="2" t="inlineStr"/>
+      <c r="V118" s="2" t="inlineStr"/>
+      <c r="W118" s="2" t="inlineStr"/>
+      <c r="X118" s="2" t="inlineStr"/>
+      <c r="Y118" s="2" t="inlineStr"/>
+      <c r="Z118" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA118" s="2" t="inlineStr"/>
+      <c r="AB118" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4e574934597a526b4f4331684f444a684c5451774d575174595749334d7931694e474a6b596a466b5a446b774d446b756347526d&amp;Fich=f5b8c4d8-a82a-401d-ab73-b4bdb1dd9009.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD118" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE118" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF118" s="2" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>118C</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>118C</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr"/>
+      <c r="D119" s="2" t="n">
+        <v>25525</v>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:43</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr"/>
+      <c r="K119" s="2" t="inlineStr"/>
+      <c r="L119" s="2" t="inlineStr"/>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N119" s="2" t="inlineStr"/>
+      <c r="O119" s="2" t="inlineStr">
+        <is>
+          <t>Ambiente e Energia</t>
+        </is>
+      </c>
+      <c r="P119" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q119" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R119" s="2" t="inlineStr"/>
+      <c r="S119" s="2" t="inlineStr"/>
+      <c r="T119" s="2" t="inlineStr"/>
+      <c r="U119" s="2" t="inlineStr"/>
+      <c r="V119" s="2" t="inlineStr"/>
+      <c r="W119" s="2" t="inlineStr"/>
+      <c r="X119" s="2" t="inlineStr"/>
+      <c r="Y119" s="2" t="inlineStr"/>
+      <c r="Z119" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA119" s="2" t="inlineStr"/>
+      <c r="AB119" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153387a596a67304f44426859533034596a64684c5451334e6a5574595445795a69307759546c6959574a6c4f4459324e7a63756347526d&amp;Fich=3b8480aa-8b7a-4765-a12f-0a9babe86677.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE119" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF119" s="2" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>119C</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>119C</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr"/>
+      <c r="D120" s="2" t="n">
+        <v>25526</v>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:45</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr"/>
+      <c r="K120" s="2" t="inlineStr"/>
+      <c r="L120" s="2" t="inlineStr"/>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N120" s="2" t="inlineStr"/>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P120" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q120" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R120" s="2" t="inlineStr"/>
+      <c r="S120" s="2" t="inlineStr"/>
+      <c r="T120" s="2" t="inlineStr"/>
+      <c r="U120" s="2" t="inlineStr"/>
+      <c r="V120" s="2" t="inlineStr"/>
+      <c r="W120" s="2" t="inlineStr"/>
+      <c r="X120" s="2" t="inlineStr"/>
+      <c r="Y120" s="2" t="inlineStr"/>
+      <c r="Z120" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA120" s="2" t="inlineStr"/>
+      <c r="AB120" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d3245794e5756684f5330304e3259304c5451354e6d4d7459546b3459533034596a646a596a6334597a55334d7a41756347526d&amp;Fich=83a25ea9-47f4-496c-a98a-8b7cb78c5730.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD120" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE120" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF120" s="2" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>120C</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>120C</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr"/>
+      <c r="D121" s="2" t="n">
+        <v>25527</v>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 17:46</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr"/>
+      <c r="K121" s="2" t="inlineStr"/>
+      <c r="L121" s="2" t="inlineStr"/>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N121" s="2" t="inlineStr"/>
+      <c r="O121" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P121" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q121" s="2" t="inlineStr">
+        <is>
+          <t>Admitida</t>
+        </is>
+      </c>
+      <c r="R121" s="2" t="inlineStr"/>
+      <c r="S121" s="2" t="inlineStr"/>
+      <c r="T121" s="2" t="inlineStr"/>
+      <c r="U121" s="2" t="inlineStr"/>
+      <c r="V121" s="2" t="inlineStr"/>
+      <c r="W121" s="2" t="inlineStr"/>
+      <c r="X121" s="2" t="inlineStr"/>
+      <c r="Y121" s="2" t="inlineStr"/>
+      <c r="Z121" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA121" s="2" t="inlineStr"/>
+      <c r="AB121" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338784f5467324d6d4a694f5331694f4446694c5451334e4751744f44426a596931694e7a55794d6a46694f445132597a49756347526d&amp;Fich=19862bb9-b81b-474d-80cb-b75221b846c2.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AD121" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:51</t>
+        </is>
+      </c>
+      <c r="AE121" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF121" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF111"/>
+  <autoFilter ref="A1:AF121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12205,7 +13185,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33 UTC</t>
+          <t>2026-10-30 18:51 UTC</t>
         </is>
       </c>
     </row>
@@ -12217,7 +13197,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 17:33 UTC</t>
+          <t>2026-10-30 18:52 UTC</t>
         </is>
       </c>
     </row>
@@ -12228,7 +13208,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7">
@@ -12238,7 +13218,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-30 19:31 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF121"/>
+  <dimension ref="A1:AF127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10504,7 +10504,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE96" s="2" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
@@ -10810,7 +10810,7 @@
       </c>
       <c r="AD98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE98" s="2" t="inlineStr">
@@ -10912,7 +10912,7 @@
       </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE99" s="2" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="AD100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE100" s="2" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="AD101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE101" s="2" t="inlineStr">
@@ -11218,7 +11218,7 @@
       </c>
       <c r="AD102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE102" s="2" t="inlineStr">
@@ -11320,7 +11320,7 @@
       </c>
       <c r="AD103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE103" s="2" t="inlineStr">
@@ -11422,7 +11422,7 @@
       </c>
       <c r="AD104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE104" s="2" t="inlineStr">
@@ -11524,7 +11524,7 @@
       </c>
       <c r="AD105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE105" s="2" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="AD106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE106" s="2" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="AD107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE107" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="AD108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE108" s="2" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="AD109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE109" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="AD110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE110" s="2" t="inlineStr">
@@ -12136,7 +12136,7 @@
       </c>
       <c r="AD111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE111" s="2" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="AD112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE112" s="2" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="AD113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE113" s="2" t="inlineStr">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="AD114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE114" s="2" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="AD115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE115" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="AD116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE116" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
       </c>
       <c r="AD117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE117" s="2" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="AD118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE118" s="2" t="inlineStr">
@@ -12920,7 +12920,7 @@
       </c>
       <c r="AD119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE119" s="2" t="inlineStr">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="AD120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE120" s="2" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="AD121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51</t>
+          <t>2026-10-30 19:30</t>
         </is>
       </c>
       <c r="AE121" s="2" t="inlineStr">
@@ -13126,8 +13126,616 @@
       </c>
       <c r="AF121" s="2" t="inlineStr"/>
     </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>121C</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>121C</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr"/>
+      <c r="D122" s="2" t="n">
+        <v>25528</v>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:00</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr"/>
+      <c r="K122" s="2" t="inlineStr"/>
+      <c r="L122" s="2" t="inlineStr"/>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N122" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 45-º-A Regulamentação e alargamento da resposta integrada de serviço de apoio domiciliário - SAD+Saúde</t>
+        </is>
+      </c>
+      <c r="O122" s="2" t="inlineStr">
+        <is>
+          <t>Trabalho, Segurança Social e Inclusão</t>
+        </is>
+      </c>
+      <c r="P122" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q122" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R122" s="2" t="inlineStr"/>
+      <c r="S122" s="2" t="inlineStr"/>
+      <c r="T122" s="2" t="inlineStr"/>
+      <c r="U122" s="2" t="inlineStr"/>
+      <c r="V122" s="2" t="inlineStr"/>
+      <c r="W122" s="2" t="inlineStr"/>
+      <c r="X122" s="2" t="inlineStr"/>
+      <c r="Y122" s="2" t="inlineStr"/>
+      <c r="Z122" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA122" s="2" t="inlineStr"/>
+      <c r="AB122" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338305a4749774f4467334d6930315a6a4d7a4c545179597a55744f445a6d4e7930324d4456684e445a6a5a6d45354d574d756347526d&amp;Fich=4db08872-5f33-42c5-86f7-605a46cfa91c.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AD122" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AE122" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF122" s="2" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>122C</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>122C</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr"/>
+      <c r="D123" s="2" t="n">
+        <v>25529</v>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:11</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr"/>
+      <c r="K123" s="2" t="inlineStr"/>
+      <c r="L123" s="2" t="inlineStr"/>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N123" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 25º-A Recrutamento de inspetores das pescas pela Direção-Geral de Recursos Naturais, Segurança e Serviços Marítimos</t>
+        </is>
+      </c>
+      <c r="O123" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P123" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q123" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R123" s="2" t="inlineStr"/>
+      <c r="S123" s="2" t="inlineStr"/>
+      <c r="T123" s="2" t="inlineStr"/>
+      <c r="U123" s="2" t="inlineStr"/>
+      <c r="V123" s="2" t="inlineStr"/>
+      <c r="W123" s="2" t="inlineStr"/>
+      <c r="X123" s="2" t="inlineStr"/>
+      <c r="Y123" s="2" t="inlineStr"/>
+      <c r="Z123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA123" s="2" t="inlineStr"/>
+      <c r="AB123" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4d574d324d44686c5953316b4d3249354c545130596d51744f544d305a6930784e574d314f574534595455774f546b756347526d&amp;Fich=e1c608ea-d3b9-44bd-934f-15c59a8a5099.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AD123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AE123" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF123" s="2" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>123C</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>123C</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr"/>
+      <c r="D124" s="2" t="n">
+        <v>25530</v>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:16</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr"/>
+      <c r="K124" s="2" t="inlineStr"/>
+      <c r="L124" s="2" t="inlineStr"/>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N124" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 28.º-A Promoção da saúde mental e prevenção do suicídio nas forças e serviços de segurança</t>
+        </is>
+      </c>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P124" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q124" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R124" s="2" t="inlineStr"/>
+      <c r="S124" s="2" t="inlineStr"/>
+      <c r="T124" s="2" t="inlineStr"/>
+      <c r="U124" s="2" t="inlineStr"/>
+      <c r="V124" s="2" t="inlineStr"/>
+      <c r="W124" s="2" t="inlineStr"/>
+      <c r="X124" s="2" t="inlineStr"/>
+      <c r="Y124" s="2" t="inlineStr"/>
+      <c r="Z124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA124" s="2" t="inlineStr"/>
+      <c r="AB124" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d4d4745344f5467344d43316b4f4446694c5451354e4749744f5463354d6930344d5463795a4459794d446c6c4d446b756347526d&amp;Fich=f0a89880-d81b-494b-9792-8172d6209e09.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AD124" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AE124" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF124" s="2" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>124C</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>124C</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr"/>
+      <c r="D125" s="2" t="n">
+        <v>25531</v>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:20</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="inlineStr"/>
+      <c r="K125" s="2" t="inlineStr"/>
+      <c r="L125" s="2" t="inlineStr"/>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N125" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 28.º-A Reforço do investimentos em infraestruturas e equipamentos das forças e serviços de segurança</t>
+        </is>
+      </c>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P125" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q125" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R125" s="2" t="inlineStr"/>
+      <c r="S125" s="2" t="inlineStr"/>
+      <c r="T125" s="2" t="inlineStr"/>
+      <c r="U125" s="2" t="inlineStr"/>
+      <c r="V125" s="2" t="inlineStr"/>
+      <c r="W125" s="2" t="inlineStr"/>
+      <c r="X125" s="2" t="inlineStr"/>
+      <c r="Y125" s="2" t="inlineStr"/>
+      <c r="Z125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA125" s="2" t="inlineStr"/>
+      <c r="AB125" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338785a6a426b4d324d794d6930314f4467314c54517a5a474d744f5455795a5331684f4745784d6a5a6d4e6a41784d6d55756347526d&amp;Fich=1f0d3c22-5885-43dc-952e-a8a126f6012e.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AD125" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AE125" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF125" s="2" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>125C</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>125C</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr"/>
+      <c r="D126" s="2" t="n">
+        <v>25532</v>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:25</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr"/>
+      <c r="K126" s="2" t="inlineStr"/>
+      <c r="L126" s="2" t="inlineStr"/>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N126" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 7.º-A Reforço das escolas e dos profissionais de referência para a Língua Gestual Portuguesa</t>
+        </is>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>Educação e Ciência</t>
+        </is>
+      </c>
+      <c r="P126" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q126" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R126" s="2" t="inlineStr"/>
+      <c r="S126" s="2" t="inlineStr"/>
+      <c r="T126" s="2" t="inlineStr"/>
+      <c r="U126" s="2" t="inlineStr"/>
+      <c r="V126" s="2" t="inlineStr"/>
+      <c r="W126" s="2" t="inlineStr"/>
+      <c r="X126" s="2" t="inlineStr"/>
+      <c r="Y126" s="2" t="inlineStr"/>
+      <c r="Z126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA126" s="2" t="inlineStr"/>
+      <c r="AB126" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338325954597a595752685979316b4d6a51774c5451794e574574596a67794e69316d4e544e6a5954637a593251344e5445756347526d&amp;Fich=6a63adac-d240-425a-b826-f53ca73cd851.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AD126" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AE126" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF126" s="2" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>126C</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>126C</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr"/>
+      <c r="D127" s="2" t="n">
+        <v>25533</v>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:27</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr"/>
+      <c r="K127" s="2" t="inlineStr"/>
+      <c r="L127" s="2" t="inlineStr"/>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N127" s="2" t="inlineStr"/>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P127" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q127" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R127" s="2" t="inlineStr"/>
+      <c r="S127" s="2" t="inlineStr"/>
+      <c r="T127" s="2" t="inlineStr"/>
+      <c r="U127" s="2" t="inlineStr"/>
+      <c r="V127" s="2" t="inlineStr"/>
+      <c r="W127" s="2" t="inlineStr"/>
+      <c r="X127" s="2" t="inlineStr"/>
+      <c r="Y127" s="2" t="inlineStr"/>
+      <c r="Z127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA127" s="2" t="inlineStr"/>
+      <c r="AB127" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684e7a67304e6d55774e7930304d5459314c54526c4e544574595751314f43316b5a4456694e325179597a417a596d4d756347526d&amp;Fich=a7846e07-4165-4e51-ad58-dd5b7d2c03bc.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AD127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:30</t>
+        </is>
+      </c>
+      <c r="AE127" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF127" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF121"/>
+  <autoFilter ref="A1:AF127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13185,7 +13793,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 18:51 UTC</t>
+          <t>2026-10-30 19:30 UTC</t>
         </is>
       </c>
     </row>
@@ -13197,7 +13805,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 18:52 UTC</t>
+          <t>2026-10-30 19:31 UTC</t>
         </is>
       </c>
     </row>
@@ -13208,7 +13816,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7">
@@ -13218,7 +13826,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-30 19:48 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$138</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF127"/>
+  <dimension ref="A1:AF138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10504,7 +10504,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE96" s="2" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
@@ -10810,7 +10810,7 @@
       </c>
       <c r="AD98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE98" s="2" t="inlineStr">
@@ -10912,7 +10912,7 @@
       </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE99" s="2" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="AD100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE100" s="2" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="AD101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE101" s="2" t="inlineStr">
@@ -11218,7 +11218,7 @@
       </c>
       <c r="AD102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE102" s="2" t="inlineStr">
@@ -11320,7 +11320,7 @@
       </c>
       <c r="AD103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE103" s="2" t="inlineStr">
@@ -11422,7 +11422,7 @@
       </c>
       <c r="AD104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE104" s="2" t="inlineStr">
@@ -11524,7 +11524,7 @@
       </c>
       <c r="AD105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE105" s="2" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="AD106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE106" s="2" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="AD107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE107" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="AD108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE108" s="2" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="AD109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE109" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="AD110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE110" s="2" t="inlineStr">
@@ -12136,7 +12136,7 @@
       </c>
       <c r="AD111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE111" s="2" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="AD112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE112" s="2" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="AD113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE113" s="2" t="inlineStr">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="AD114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE114" s="2" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="AD115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE115" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="AD116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE116" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
       </c>
       <c r="AD117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE117" s="2" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="AD118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE118" s="2" t="inlineStr">
@@ -12920,7 +12920,7 @@
       </c>
       <c r="AD119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE119" s="2" t="inlineStr">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="AD120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE120" s="2" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="AD121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE121" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="AD122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE122" s="2" t="inlineStr">
@@ -13320,7 +13320,7 @@
       </c>
       <c r="AD123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE123" s="2" t="inlineStr">
@@ -13422,7 +13422,7 @@
       </c>
       <c r="AD124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE124" s="2" t="inlineStr">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="AD125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE125" s="2" t="inlineStr">
@@ -13626,7 +13626,7 @@
       </c>
       <c r="AD126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE126" s="2" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="AD127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30</t>
+          <t>2026-10-30 19:48</t>
         </is>
       </c>
       <c r="AE127" s="2" t="inlineStr">
@@ -13734,8 +13734,1106 @@
       </c>
       <c r="AF127" s="2" t="inlineStr"/>
     </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>127C</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>127C</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr"/>
+      <c r="D128" s="2" t="n">
+        <v>25534</v>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:31</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr"/>
+      <c r="K128" s="2" t="inlineStr"/>
+      <c r="L128" s="2" t="inlineStr"/>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N128" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 60.º Alteração ao Código do Imposto sobre o Rendimento das Pessoas Singulares</t>
+        </is>
+      </c>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P128" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q128" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R128" s="2" t="inlineStr"/>
+      <c r="S128" s="2" t="inlineStr"/>
+      <c r="T128" s="2" t="inlineStr"/>
+      <c r="U128" s="2" t="inlineStr"/>
+      <c r="V128" s="2" t="inlineStr"/>
+      <c r="W128" s="2" t="inlineStr"/>
+      <c r="X128" s="2" t="inlineStr"/>
+      <c r="Y128" s="2" t="inlineStr"/>
+      <c r="Z128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA128" s="2" t="inlineStr"/>
+      <c r="AB128" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396b4e7a466b4d7a526a596930355a5749324c545131597a6b74596d56694e6930344f544d774e4459325a44526c5a6a51756347526d&amp;Fich=d71d34cb-9eb6-45c9-beb6-8930466d4ef4.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD128" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE128" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF128" s="2" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>128C</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>128C</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr"/>
+      <c r="D129" s="2" t="n">
+        <v>25535</v>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:31</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr"/>
+      <c r="K129" s="2" t="inlineStr"/>
+      <c r="L129" s="2" t="inlineStr"/>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N129" s="2" t="inlineStr"/>
+      <c r="O129" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P129" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q129" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R129" s="2" t="inlineStr"/>
+      <c r="S129" s="2" t="inlineStr"/>
+      <c r="T129" s="2" t="inlineStr"/>
+      <c r="U129" s="2" t="inlineStr"/>
+      <c r="V129" s="2" t="inlineStr"/>
+      <c r="W129" s="2" t="inlineStr"/>
+      <c r="X129" s="2" t="inlineStr"/>
+      <c r="Y129" s="2" t="inlineStr"/>
+      <c r="Z129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA129" s="2" t="inlineStr"/>
+      <c r="AB129" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338795a5755344f5455354e6931684f5464684c5451344d6a45744f5755314f5330334d57466c4d5463344d475a6a597a4d756347526d&amp;Fich=2ee89596-a97a-4821-9e59-71ae1780fcc3.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD129" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE129" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF129" s="2" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>129C</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>129C</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr"/>
+      <c r="D130" s="2" t="n">
+        <v>25536</v>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:33</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr"/>
+      <c r="K130" s="2" t="inlineStr"/>
+      <c r="L130" s="2" t="inlineStr"/>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N130" s="2" t="inlineStr"/>
+      <c r="O130" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P130" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q130" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R130" s="2" t="inlineStr"/>
+      <c r="S130" s="2" t="inlineStr"/>
+      <c r="T130" s="2" t="inlineStr"/>
+      <c r="U130" s="2" t="inlineStr"/>
+      <c r="V130" s="2" t="inlineStr"/>
+      <c r="W130" s="2" t="inlineStr"/>
+      <c r="X130" s="2" t="inlineStr"/>
+      <c r="Y130" s="2" t="inlineStr"/>
+      <c r="Z130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA130" s="2" t="inlineStr"/>
+      <c r="AB130" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396959545a694e32457759693077596a646b4c5451344e6a49744f5451324d5330774f544577597a45324e324977595759756347526d&amp;Fich=ba6b7a0b-0b7d-4862-9461-0910c167b0af.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD130" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE130" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF130" s="2" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>130C</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>130C</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr"/>
+      <c r="D131" s="2" t="n">
+        <v>25537</v>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:33</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr"/>
+      <c r="K131" s="2" t="inlineStr"/>
+      <c r="L131" s="2" t="inlineStr"/>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N131" s="2" t="inlineStr"/>
+      <c r="O131" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P131" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q131" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R131" s="2" t="inlineStr"/>
+      <c r="S131" s="2" t="inlineStr"/>
+      <c r="T131" s="2" t="inlineStr"/>
+      <c r="U131" s="2" t="inlineStr"/>
+      <c r="V131" s="2" t="inlineStr"/>
+      <c r="W131" s="2" t="inlineStr"/>
+      <c r="X131" s="2" t="inlineStr"/>
+      <c r="Y131" s="2" t="inlineStr"/>
+      <c r="Z131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA131" s="2" t="inlineStr"/>
+      <c r="AB131" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339684f574a694e7a466c5a6930315a4449354c5451314d544174595751355a5330785a44686d596a51354f546b32593251756347526d&amp;Fich=a9bb71ef-5d29-4510-ad9e-1d8fb49996cd.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE131" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF131" s="2" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>131C</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>131C</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr"/>
+      <c r="D132" s="2" t="n">
+        <v>25538</v>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:34</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr"/>
+      <c r="K132" s="2" t="inlineStr"/>
+      <c r="L132" s="2" t="inlineStr"/>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N132" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 119 - A Comparticipação dos tratamentos de imunoterapia específica com alergénios</t>
+        </is>
+      </c>
+      <c r="O132" s="2" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="P132" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q132" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R132" s="2" t="inlineStr"/>
+      <c r="S132" s="2" t="inlineStr"/>
+      <c r="T132" s="2" t="inlineStr"/>
+      <c r="U132" s="2" t="inlineStr"/>
+      <c r="V132" s="2" t="inlineStr"/>
+      <c r="W132" s="2" t="inlineStr"/>
+      <c r="X132" s="2" t="inlineStr"/>
+      <c r="Y132" s="2" t="inlineStr"/>
+      <c r="Z132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA132" s="2" t="inlineStr"/>
+      <c r="AB132" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396a596a4d79596a6b7a4e43307a4e6a56694c54513559325574596a42694e53307a4e5755784d6d466d4d6a6c6d4e4441756347526d&amp;Fich=cb32b934-365b-49ce-b0b5-35e12af29f40.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE132" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF132" s="2" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>132C</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>132C</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr"/>
+      <c r="D133" s="2" t="n">
+        <v>25539</v>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:34</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr"/>
+      <c r="K133" s="2" t="inlineStr"/>
+      <c r="L133" s="2" t="inlineStr"/>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N133" s="2" t="inlineStr"/>
+      <c r="O133" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P133" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q133" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R133" s="2" t="inlineStr"/>
+      <c r="S133" s="2" t="inlineStr"/>
+      <c r="T133" s="2" t="inlineStr"/>
+      <c r="U133" s="2" t="inlineStr"/>
+      <c r="V133" s="2" t="inlineStr"/>
+      <c r="W133" s="2" t="inlineStr"/>
+      <c r="X133" s="2" t="inlineStr"/>
+      <c r="Y133" s="2" t="inlineStr"/>
+      <c r="Z133" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA133" s="2" t="inlineStr"/>
+      <c r="AB133" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338784f474d78595455354d6930304e7a67794c5451795a6a5974596a4d345a53316c4e7a51325954686c4f545579596a59756347526d&amp;Fich=18c1a592-4782-42f6-b38e-e746a8e952b6.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE133" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF133" s="2" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>133C</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>133C</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr"/>
+      <c r="D134" s="2" t="n">
+        <v>25540</v>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:36</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr"/>
+      <c r="K134" s="2" t="inlineStr"/>
+      <c r="L134" s="2" t="inlineStr"/>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N134" s="2" t="inlineStr"/>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação</t>
+        </is>
+      </c>
+      <c r="P134" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q134" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R134" s="2" t="inlineStr"/>
+      <c r="S134" s="2" t="inlineStr"/>
+      <c r="T134" s="2" t="inlineStr"/>
+      <c r="U134" s="2" t="inlineStr"/>
+      <c r="V134" s="2" t="inlineStr"/>
+      <c r="W134" s="2" t="inlineStr"/>
+      <c r="X134" s="2" t="inlineStr"/>
+      <c r="Y134" s="2" t="inlineStr"/>
+      <c r="Z134" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA134" s="2" t="inlineStr"/>
+      <c r="AB134" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4d445130596d566c4e5330794d574d354c5452684f574974596d466b4f5330774e4445354f5451315a444e6a4d4749756347526d&amp;Fich=e044bee5-21c9-4a9b-bad9-0419945d3c0b.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE134" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF134" s="2" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>134C</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>134C</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr"/>
+      <c r="D135" s="2" t="n">
+        <v>25541</v>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:36</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr"/>
+      <c r="K135" s="2" t="inlineStr"/>
+      <c r="L135" s="2" t="inlineStr"/>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N135" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 119 - A Acessibilidade da população à prevenção contra a Zona (Herpes Zoster)</t>
+        </is>
+      </c>
+      <c r="O135" s="2" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="P135" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q135" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R135" s="2" t="inlineStr"/>
+      <c r="S135" s="2" t="inlineStr"/>
+      <c r="T135" s="2" t="inlineStr"/>
+      <c r="U135" s="2" t="inlineStr"/>
+      <c r="V135" s="2" t="inlineStr"/>
+      <c r="W135" s="2" t="inlineStr"/>
+      <c r="X135" s="2" t="inlineStr"/>
+      <c r="Y135" s="2" t="inlineStr"/>
+      <c r="Z135" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA135" s="2" t="inlineStr"/>
+      <c r="AB135" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338304f5464695a6a51324d69303259324e6c4c54526a4e546774596d49794f5331684e7a45314e6a6b334d4451325a6d59756347526d&amp;Fich=497bf462-6cce-4c58-bb29-a715697046ff.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE135" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF135" s="2" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>135C</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>135C</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr"/>
+      <c r="D136" s="2" t="n">
+        <v>25542</v>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:37</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr"/>
+      <c r="K136" s="2" t="inlineStr"/>
+      <c r="L136" s="2" t="inlineStr"/>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N136" s="2" t="inlineStr"/>
+      <c r="O136" s="2" t="inlineStr">
+        <is>
+          <t>Infraestruturas, Mobilidade e Habitação; Orçamento, Finanças e Administração Pública</t>
+        </is>
+      </c>
+      <c r="P136" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q136" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R136" s="2" t="inlineStr"/>
+      <c r="S136" s="2" t="inlineStr"/>
+      <c r="T136" s="2" t="inlineStr"/>
+      <c r="U136" s="2" t="inlineStr"/>
+      <c r="V136" s="2" t="inlineStr"/>
+      <c r="W136" s="2" t="inlineStr"/>
+      <c r="X136" s="2" t="inlineStr"/>
+      <c r="Y136" s="2" t="inlineStr"/>
+      <c r="Z136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA136" s="2" t="inlineStr"/>
+      <c r="AB136" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338304d44466a59574d324d533033596a686a4c5452694d7a45744f5459355a69316d5932566a4d7a63335954566c5a6d55756347526d&amp;Fich=401cac61-7b8c-4b31-969f-fcec377a5efe.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE136" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF136" s="2" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>136C</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>136C</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr"/>
+      <c r="D137" s="2" t="n">
+        <v>25543</v>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:40</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr"/>
+      <c r="K137" s="2" t="inlineStr"/>
+      <c r="L137" s="2" t="inlineStr"/>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N137" s="2" t="inlineStr">
+        <is>
+          <t>Artigo 118 [...] Reforço da transparência na contratação do Estado com prestadores de cuidados de saúde do setor privado e social</t>
+        </is>
+      </c>
+      <c r="O137" s="2" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="P137" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q137" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R137" s="2" t="inlineStr"/>
+      <c r="S137" s="2" t="inlineStr"/>
+      <c r="T137" s="2" t="inlineStr"/>
+      <c r="U137" s="2" t="inlineStr"/>
+      <c r="V137" s="2" t="inlineStr"/>
+      <c r="W137" s="2" t="inlineStr"/>
+      <c r="X137" s="2" t="inlineStr"/>
+      <c r="Y137" s="2" t="inlineStr"/>
+      <c r="Z137" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA137" s="2" t="inlineStr"/>
+      <c r="AB137" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338775a444d314d324d30595330315a444d354c5451324e6a6374596d51774e7930784f44637a4d6a4a6d4e4759324f5459756347526d&amp;Fich=0d353c4a-5d39-4667-bd07-187322f4f696.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE137" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF137" s="2" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>137C</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>137C</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr"/>
+      <c r="D138" s="2" t="n">
+        <v>25544</v>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:43</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr"/>
+      <c r="K138" s="2" t="inlineStr"/>
+      <c r="L138" s="2" t="inlineStr"/>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N138" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 118 - A Observatório da Literacia em Saúde</t>
+        </is>
+      </c>
+      <c r="O138" s="2" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="P138" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q138" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R138" s="2" t="inlineStr"/>
+      <c r="S138" s="2" t="inlineStr"/>
+      <c r="T138" s="2" t="inlineStr"/>
+      <c r="U138" s="2" t="inlineStr"/>
+      <c r="V138" s="2" t="inlineStr"/>
+      <c r="W138" s="2" t="inlineStr"/>
+      <c r="X138" s="2" t="inlineStr"/>
+      <c r="Y138" s="2" t="inlineStr"/>
+      <c r="Z138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA138" s="2" t="inlineStr"/>
+      <c r="AB138" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c4d44686a595751314e6930354d3255794c5451314d6a4d744f474a6d5a6931684d5755345a6a55795a5449785a4445756347526d&amp;Fich=e08cad56-93e2-4523-8bff-a1e8f52e21d1.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AD138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:48</t>
+        </is>
+      </c>
+      <c r="AE138" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF138" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF127"/>
+  <autoFilter ref="A1:AF138"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13793,7 +14891,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 19:30 UTC</t>
+          <t>2026-10-30 19:48 UTC</t>
         </is>
       </c>
     </row>
@@ -13805,7 +14903,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 19:31 UTC</t>
+          <t>2026-10-30 19:48 UTC</t>
         </is>
       </c>
     </row>
@@ -13816,7 +14914,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>126</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7">
@@ -13826,7 +14924,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>126</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-30 22:57 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$155</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF138"/>
+  <dimension ref="A1:AF155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10504,7 +10504,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE96" s="2" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
@@ -10810,7 +10810,7 @@
       </c>
       <c r="AD98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE98" s="2" t="inlineStr">
@@ -10912,7 +10912,7 @@
       </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE99" s="2" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="AD100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE100" s="2" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="AD101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE101" s="2" t="inlineStr">
@@ -11218,7 +11218,7 @@
       </c>
       <c r="AD102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE102" s="2" t="inlineStr">
@@ -11320,7 +11320,7 @@
       </c>
       <c r="AD103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE103" s="2" t="inlineStr">
@@ -11422,7 +11422,7 @@
       </c>
       <c r="AD104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE104" s="2" t="inlineStr">
@@ -11524,7 +11524,7 @@
       </c>
       <c r="AD105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE105" s="2" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="AD106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE106" s="2" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="AD107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE107" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="AD108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE108" s="2" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="AD109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE109" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="AD110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE110" s="2" t="inlineStr">
@@ -12136,7 +12136,7 @@
       </c>
       <c r="AD111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE111" s="2" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="AD112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE112" s="2" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="AD113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE113" s="2" t="inlineStr">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="AD114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE114" s="2" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="AD115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE115" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="AD116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE116" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
       </c>
       <c r="AD117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE117" s="2" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="AD118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE118" s="2" t="inlineStr">
@@ -12920,7 +12920,7 @@
       </c>
       <c r="AD119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE119" s="2" t="inlineStr">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="AD120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE120" s="2" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="AD121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE121" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="AD122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE122" s="2" t="inlineStr">
@@ -13320,7 +13320,7 @@
       </c>
       <c r="AD123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE123" s="2" t="inlineStr">
@@ -13422,7 +13422,7 @@
       </c>
       <c r="AD124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE124" s="2" t="inlineStr">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="AD125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE125" s="2" t="inlineStr">
@@ -13626,7 +13626,7 @@
       </c>
       <c r="AD126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE126" s="2" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="AD127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE127" s="2" t="inlineStr">
@@ -13826,7 +13826,7 @@
       </c>
       <c r="AD128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE128" s="2" t="inlineStr">
@@ -13924,7 +13924,7 @@
       </c>
       <c r="AD129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE129" s="2" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="AD130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE130" s="2" t="inlineStr">
@@ -14120,7 +14120,7 @@
       </c>
       <c r="AD131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE131" s="2" t="inlineStr">
@@ -14222,7 +14222,7 @@
       </c>
       <c r="AD132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE132" s="2" t="inlineStr">
@@ -14320,7 +14320,7 @@
       </c>
       <c r="AD133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE133" s="2" t="inlineStr">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="AD134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE134" s="2" t="inlineStr">
@@ -14520,7 +14520,7 @@
       </c>
       <c r="AD135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE135" s="2" t="inlineStr">
@@ -14618,7 +14618,7 @@
       </c>
       <c r="AD136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE136" s="2" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="AD137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE137" s="2" t="inlineStr">
@@ -14822,7 +14822,7 @@
       </c>
       <c r="AD138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48</t>
+          <t>2026-10-30 22:57</t>
         </is>
       </c>
       <c r="AE138" s="2" t="inlineStr">
@@ -14832,8 +14832,1678 @@
       </c>
       <c r="AF138" s="2" t="inlineStr"/>
     </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>138C</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>138C</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr"/>
+      <c r="D139" s="2" t="n">
+        <v>25545</v>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 19:46</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>Filipa Pinto; Isabel Mendes Lopes; Jorge Pinto; Patrícia Gonçalves; Paulo Muacho; Rui Tavares</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr"/>
+      <c r="K139" s="2" t="inlineStr"/>
+      <c r="L139" s="2" t="inlineStr"/>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N139" s="2" t="inlineStr">
+        <is>
+          <t>[NOVO] Artigo 118 - A Alteração ao Regime Jurídico dos Jogos e Apostas Online aprovado pelo Decreto-Lei n.º 66/2015, de 29 de abril</t>
+        </is>
+      </c>
+      <c r="O139" s="2" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="P139" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q139" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R139" s="2" t="inlineStr"/>
+      <c r="S139" s="2" t="inlineStr"/>
+      <c r="T139" s="2" t="inlineStr"/>
+      <c r="U139" s="2" t="inlineStr"/>
+      <c r="V139" s="2" t="inlineStr"/>
+      <c r="W139" s="2" t="inlineStr"/>
+      <c r="X139" s="2" t="inlineStr"/>
+      <c r="Y139" s="2" t="inlineStr"/>
+      <c r="Z139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA139" s="2" t="inlineStr"/>
+      <c r="AB139" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533834597a51795a57526d5a69316b596d4d774c54517959575974596d55314e7930335a4445315a5467774d7a646a5a546b756347526d&amp;Fich=8c42edff-dbc0-42af-be57-7d15e8037ce9.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC139" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD139" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE139" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF139" s="2" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>139C</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>139C</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr"/>
+      <c r="D140" s="2" t="n">
+        <v>25546</v>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:16</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr"/>
+      <c r="K140" s="2" t="inlineStr"/>
+      <c r="L140" s="2" t="inlineStr"/>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N140" s="2" t="inlineStr"/>
+      <c r="O140" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P140" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q140" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R140" s="2" t="inlineStr"/>
+      <c r="S140" s="2" t="inlineStr"/>
+      <c r="T140" s="2" t="inlineStr"/>
+      <c r="U140" s="2" t="inlineStr"/>
+      <c r="V140" s="2" t="inlineStr"/>
+      <c r="W140" s="2" t="inlineStr"/>
+      <c r="X140" s="2" t="inlineStr"/>
+      <c r="Y140" s="2" t="inlineStr"/>
+      <c r="Z140" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA140" s="2" t="inlineStr"/>
+      <c r="AB140" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324d324d344e54426d4e7930794d5745304c54513059574974596a49794d79316c4f5455334d7a6c694d6d52694e6d4d756347526d&amp;Fich=63c850f7-21a4-44ab-b223-e95739b2db6c.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE140" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF140" s="2" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>140C</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>140C</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr"/>
+      <c r="D141" s="2" t="n">
+        <v>25547</v>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:21</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr"/>
+      <c r="K141" s="2" t="inlineStr"/>
+      <c r="L141" s="2" t="inlineStr"/>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N141" s="2" t="inlineStr"/>
+      <c r="O141" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P141" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q141" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R141" s="2" t="inlineStr"/>
+      <c r="S141" s="2" t="inlineStr"/>
+      <c r="T141" s="2" t="inlineStr"/>
+      <c r="U141" s="2" t="inlineStr"/>
+      <c r="V141" s="2" t="inlineStr"/>
+      <c r="W141" s="2" t="inlineStr"/>
+      <c r="X141" s="2" t="inlineStr"/>
+      <c r="Y141" s="2" t="inlineStr"/>
+      <c r="Z141" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA141" s="2" t="inlineStr"/>
+      <c r="AB141" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314e5449344e7a59774d79316a4d5759334c54526a4f446b74596a5977596930344e4445304e7a5578597a426a5a6d4d756347526d&amp;Fich=55287603-c1f7-4c89-b60b-8414751c0cfc.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC141" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD141" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE141" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF141" s="2" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>141C</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>141C</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr"/>
+      <c r="D142" s="2" t="n">
+        <v>25548</v>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:22</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr"/>
+      <c r="K142" s="2" t="inlineStr"/>
+      <c r="L142" s="2" t="inlineStr"/>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N142" s="2" t="inlineStr"/>
+      <c r="O142" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P142" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q142" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R142" s="2" t="inlineStr"/>
+      <c r="S142" s="2" t="inlineStr"/>
+      <c r="T142" s="2" t="inlineStr"/>
+      <c r="U142" s="2" t="inlineStr"/>
+      <c r="V142" s="2" t="inlineStr"/>
+      <c r="W142" s="2" t="inlineStr"/>
+      <c r="X142" s="2" t="inlineStr"/>
+      <c r="Y142" s="2" t="inlineStr"/>
+      <c r="Z142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA142" s="2" t="inlineStr"/>
+      <c r="AB142" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314e5449344e7a59774d79316a4d5759334c54526a4f446b74596a5977596930344e4445304e7a5578597a426a5a6d4d756347526d&amp;Fich=55287603-c1f7-4c89-b60b-8414751c0cfc.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE142" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF142" s="2" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>142C</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>142C</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr"/>
+      <c r="D143" s="2" t="n">
+        <v>25549</v>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:25</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr"/>
+      <c r="K143" s="2" t="inlineStr"/>
+      <c r="L143" s="2" t="inlineStr"/>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N143" s="2" t="inlineStr"/>
+      <c r="O143" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P143" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q143" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R143" s="2" t="inlineStr"/>
+      <c r="S143" s="2" t="inlineStr"/>
+      <c r="T143" s="2" t="inlineStr"/>
+      <c r="U143" s="2" t="inlineStr"/>
+      <c r="V143" s="2" t="inlineStr"/>
+      <c r="W143" s="2" t="inlineStr"/>
+      <c r="X143" s="2" t="inlineStr"/>
+      <c r="Y143" s="2" t="inlineStr"/>
+      <c r="Z143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA143" s="2" t="inlineStr"/>
+      <c r="AB143" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338794f5455334d4463334d6930334e4745314c5451794f5451744f47526d4e43316b4d546c6b5a6d4a6d5a6a55324d7a55756347526d&amp;Fich=29570772-74a5-4294-8df4-d19dfbff5635.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE143" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF143" s="2" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>143C</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>143C</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr"/>
+      <c r="D144" s="2" t="n">
+        <v>25550</v>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:26</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr"/>
+      <c r="K144" s="2" t="inlineStr"/>
+      <c r="L144" s="2" t="inlineStr"/>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N144" s="2" t="inlineStr"/>
+      <c r="O144" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P144" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q144" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R144" s="2" t="inlineStr"/>
+      <c r="S144" s="2" t="inlineStr"/>
+      <c r="T144" s="2" t="inlineStr"/>
+      <c r="U144" s="2" t="inlineStr"/>
+      <c r="V144" s="2" t="inlineStr"/>
+      <c r="W144" s="2" t="inlineStr"/>
+      <c r="X144" s="2" t="inlineStr"/>
+      <c r="Y144" s="2" t="inlineStr"/>
+      <c r="Z144" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA144" s="2" t="inlineStr"/>
+      <c r="AB144" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338334f4463794e6a63324e43316b4f5456684c545131595455745957566d4e7930314e47466b4d5445335a445a6a5a546b756347526d&amp;Fich=78726764-d95a-45a5-aef7-54ad117d6ce9.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE144" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF144" s="2" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>144C</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>144C</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr"/>
+      <c r="D145" s="2" t="n">
+        <v>25551</v>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:34</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr"/>
+      <c r="K145" s="2" t="inlineStr"/>
+      <c r="L145" s="2" t="inlineStr"/>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N145" s="2" t="inlineStr"/>
+      <c r="O145" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P145" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q145" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R145" s="2" t="inlineStr"/>
+      <c r="S145" s="2" t="inlineStr"/>
+      <c r="T145" s="2" t="inlineStr"/>
+      <c r="U145" s="2" t="inlineStr"/>
+      <c r="V145" s="2" t="inlineStr"/>
+      <c r="W145" s="2" t="inlineStr"/>
+      <c r="X145" s="2" t="inlineStr"/>
+      <c r="Y145" s="2" t="inlineStr"/>
+      <c r="Z145" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA145" s="2" t="inlineStr"/>
+      <c r="AB145" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d5464685a47557a5a43316a4f4751304c545268596a55744f545a6a4d5330354f5463784d6a4130596a67794d6a51756347526d&amp;Fich=817ade3d-c8d4-4ab5-96c1-9971204b8224.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE145" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF145" s="2" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>145C</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>145C</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr"/>
+      <c r="D146" s="2" t="n">
+        <v>25552</v>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:35</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr"/>
+      <c r="K146" s="2" t="inlineStr"/>
+      <c r="L146" s="2" t="inlineStr"/>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N146" s="2" t="inlineStr"/>
+      <c r="O146" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P146" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q146" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R146" s="2" t="inlineStr"/>
+      <c r="S146" s="2" t="inlineStr"/>
+      <c r="T146" s="2" t="inlineStr"/>
+      <c r="U146" s="2" t="inlineStr"/>
+      <c r="V146" s="2" t="inlineStr"/>
+      <c r="W146" s="2" t="inlineStr"/>
+      <c r="X146" s="2" t="inlineStr"/>
+      <c r="Y146" s="2" t="inlineStr"/>
+      <c r="Z146" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA146" s="2" t="inlineStr"/>
+      <c r="AB146" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314d7a6b325957566c4d53316c4d47566d4c5451324e575574596d49355a53307a4e5463344d7a49774d544132595749756347526d&amp;Fich=5396aee1-e0ef-465e-bb9e-3578320106ab.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE146" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF146" s="2" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>146C</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>146C</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr"/>
+      <c r="D147" s="2" t="n">
+        <v>25553</v>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:36</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr"/>
+      <c r="K147" s="2" t="inlineStr"/>
+      <c r="L147" s="2" t="inlineStr"/>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N147" s="2" t="inlineStr"/>
+      <c r="O147" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P147" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q147" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R147" s="2" t="inlineStr"/>
+      <c r="S147" s="2" t="inlineStr"/>
+      <c r="T147" s="2" t="inlineStr"/>
+      <c r="U147" s="2" t="inlineStr"/>
+      <c r="V147" s="2" t="inlineStr"/>
+      <c r="W147" s="2" t="inlineStr"/>
+      <c r="X147" s="2" t="inlineStr"/>
+      <c r="Y147" s="2" t="inlineStr"/>
+      <c r="Z147" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA147" s="2" t="inlineStr"/>
+      <c r="AB147" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533879596a59304e6a526c5969316a4d5455324c54517a597a45744f4446684d69316c5a6a59784f5751325a6d45794e474d756347526d&amp;Fich=2b6464eb-c156-43c1-81a2-ef619d6fa24c.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC147" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD147" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE147" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF147" s="2" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>147C</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>147C</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr"/>
+      <c r="D148" s="2" t="n">
+        <v>25554</v>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:37</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr"/>
+      <c r="K148" s="2" t="inlineStr"/>
+      <c r="L148" s="2" t="inlineStr"/>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N148" s="2" t="inlineStr"/>
+      <c r="O148" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P148" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q148" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R148" s="2" t="inlineStr"/>
+      <c r="S148" s="2" t="inlineStr"/>
+      <c r="T148" s="2" t="inlineStr"/>
+      <c r="U148" s="2" t="inlineStr"/>
+      <c r="V148" s="2" t="inlineStr"/>
+      <c r="W148" s="2" t="inlineStr"/>
+      <c r="X148" s="2" t="inlineStr"/>
+      <c r="Y148" s="2" t="inlineStr"/>
+      <c r="Z148" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA148" s="2" t="inlineStr"/>
+      <c r="AB148" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d54637a596a51324d7930305a57457a4c5451354d5459744f5451344e4330344e44513459325978597a466c596d45756347526d&amp;Fich=8173b463-4ea3-4916-9484-8448cf1c1eba.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE148" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF148" s="2" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>148C</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>148C</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr"/>
+      <c r="D149" s="2" t="n">
+        <v>25555</v>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:38</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr"/>
+      <c r="K149" s="2" t="inlineStr"/>
+      <c r="L149" s="2" t="inlineStr"/>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N149" s="2" t="inlineStr"/>
+      <c r="O149" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P149" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q149" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R149" s="2" t="inlineStr"/>
+      <c r="S149" s="2" t="inlineStr"/>
+      <c r="T149" s="2" t="inlineStr"/>
+      <c r="U149" s="2" t="inlineStr"/>
+      <c r="V149" s="2" t="inlineStr"/>
+      <c r="W149" s="2" t="inlineStr"/>
+      <c r="X149" s="2" t="inlineStr"/>
+      <c r="Y149" s="2" t="inlineStr"/>
+      <c r="Z149" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA149" s="2" t="inlineStr"/>
+      <c r="AB149" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338314d6a4d315a4464684d6930784d5459334c5451304e4755744f574a6c5969316b5a44566b5a6a67795a444d314f546b756347526d&amp;Fich=5235d7a2-1167-444e-9beb-dd5df82d3599.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC149" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD149" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE149" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF149" s="2" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>149C</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>149C</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr"/>
+      <c r="D150" s="2" t="n">
+        <v>25556</v>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:39</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr"/>
+      <c r="K150" s="2" t="inlineStr"/>
+      <c r="L150" s="2" t="inlineStr"/>
+      <c r="M150" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N150" s="2" t="inlineStr"/>
+      <c r="O150" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P150" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q150" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R150" s="2" t="inlineStr"/>
+      <c r="S150" s="2" t="inlineStr"/>
+      <c r="T150" s="2" t="inlineStr"/>
+      <c r="U150" s="2" t="inlineStr"/>
+      <c r="V150" s="2" t="inlineStr"/>
+      <c r="W150" s="2" t="inlineStr"/>
+      <c r="X150" s="2" t="inlineStr"/>
+      <c r="Y150" s="2" t="inlineStr"/>
+      <c r="Z150" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA150" s="2" t="inlineStr"/>
+      <c r="AB150" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c5a4455344e7a6868597930785a6d526d4c54526b4d446774595446694f433035597a637a595749324d575268597a41756347526d&amp;Fich=ed5878ac-1fdf-4d08-a1b8-9c73ab61dac0.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC150" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD150" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE150" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF150" s="2" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>150C</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>150C</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr"/>
+      <c r="D151" s="2" t="n">
+        <v>25557</v>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:41</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr"/>
+      <c r="K151" s="2" t="inlineStr"/>
+      <c r="L151" s="2" t="inlineStr"/>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N151" s="2" t="inlineStr"/>
+      <c r="O151" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P151" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q151" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R151" s="2" t="inlineStr"/>
+      <c r="S151" s="2" t="inlineStr"/>
+      <c r="T151" s="2" t="inlineStr"/>
+      <c r="U151" s="2" t="inlineStr"/>
+      <c r="V151" s="2" t="inlineStr"/>
+      <c r="W151" s="2" t="inlineStr"/>
+      <c r="X151" s="2" t="inlineStr"/>
+      <c r="Y151" s="2" t="inlineStr"/>
+      <c r="Z151" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA151" s="2" t="inlineStr"/>
+      <c r="AB151" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533833597a497a596a566b4d6930794d5463324c5451354f544d744f546b314e6930795a6a5a6b4d7a5931596d56695a6d51756347526d&amp;Fich=7c23b5d2-2176-4993-9956-2f6d365bebfd.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC151" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD151" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE151" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF151" s="2" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>151C</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>151C</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr"/>
+      <c r="D152" s="2" t="n">
+        <v>25558</v>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:41</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr"/>
+      <c r="K152" s="2" t="inlineStr"/>
+      <c r="L152" s="2" t="inlineStr"/>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N152" s="2" t="inlineStr"/>
+      <c r="O152" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P152" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q152" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R152" s="2" t="inlineStr"/>
+      <c r="S152" s="2" t="inlineStr"/>
+      <c r="T152" s="2" t="inlineStr"/>
+      <c r="U152" s="2" t="inlineStr"/>
+      <c r="V152" s="2" t="inlineStr"/>
+      <c r="W152" s="2" t="inlineStr"/>
+      <c r="X152" s="2" t="inlineStr"/>
+      <c r="Y152" s="2" t="inlineStr"/>
+      <c r="Z152" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA152" s="2" t="inlineStr"/>
+      <c r="AB152" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338344d44457a4d54526d597930794f57526b4c54526a4e7a4974595455354f43316c4f47557a4e7a5668596a5178597a67756347526d&amp;Fich=801314fc-29dd-4c72-a598-e8e375ab41c8.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC152" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD152" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE152" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF152" s="2" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>152C</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>152C</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr"/>
+      <c r="D153" s="2" t="n">
+        <v>25559</v>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:43</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr"/>
+      <c r="K153" s="2" t="inlineStr"/>
+      <c r="L153" s="2" t="inlineStr"/>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N153" s="2" t="inlineStr"/>
+      <c r="O153" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P153" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q153" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R153" s="2" t="inlineStr"/>
+      <c r="S153" s="2" t="inlineStr"/>
+      <c r="T153" s="2" t="inlineStr"/>
+      <c r="U153" s="2" t="inlineStr"/>
+      <c r="V153" s="2" t="inlineStr"/>
+      <c r="W153" s="2" t="inlineStr"/>
+      <c r="X153" s="2" t="inlineStr"/>
+      <c r="Y153" s="2" t="inlineStr"/>
+      <c r="Z153" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA153" s="2" t="inlineStr"/>
+      <c r="AB153" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533830595455795a4449334e7930794e4455774c54526d5a446b744f5446695a6930775a5756695954686c4d44646a4d4441756347526d&amp;Fich=4a52d277-2450-4fd9-91bf-0eeba8e07c00.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC153" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD153" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE153" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF153" s="2" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>153C</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>153C</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr"/>
+      <c r="D154" s="2" t="n">
+        <v>25560</v>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:43</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr"/>
+      <c r="K154" s="2" t="inlineStr"/>
+      <c r="L154" s="2" t="inlineStr"/>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="inlineStr"/>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P154" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q154" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R154" s="2" t="inlineStr"/>
+      <c r="S154" s="2" t="inlineStr"/>
+      <c r="T154" s="2" t="inlineStr"/>
+      <c r="U154" s="2" t="inlineStr"/>
+      <c r="V154" s="2" t="inlineStr"/>
+      <c r="W154" s="2" t="inlineStr"/>
+      <c r="X154" s="2" t="inlineStr"/>
+      <c r="Y154" s="2" t="inlineStr"/>
+      <c r="Z154" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA154" s="2" t="inlineStr"/>
+      <c r="AB154" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324d6d5a6d4f5756684f43303259544d784c545135596d4d744f5759314f4330774e575a6b4d32557a4d6a417a4e7a45756347526d&amp;Fich=62ff9ea8-6a31-49bc-9f58-05fd3e320371.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC154" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD154" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE154" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF154" s="2" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>154C</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>154C</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr"/>
+      <c r="D155" s="2" t="n">
+        <v>25561</v>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:44</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr"/>
+      <c r="K155" s="2" t="inlineStr"/>
+      <c r="L155" s="2" t="inlineStr"/>
+      <c r="M155" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N155" s="2" t="inlineStr"/>
+      <c r="O155" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P155" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q155" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R155" s="2" t="inlineStr"/>
+      <c r="S155" s="2" t="inlineStr"/>
+      <c r="T155" s="2" t="inlineStr"/>
+      <c r="U155" s="2" t="inlineStr"/>
+      <c r="V155" s="2" t="inlineStr"/>
+      <c r="W155" s="2" t="inlineStr"/>
+      <c r="X155" s="2" t="inlineStr"/>
+      <c r="Y155" s="2" t="inlineStr"/>
+      <c r="Z155" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA155" s="2" t="inlineStr"/>
+      <c r="AB155" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338304e7a426c4f574d324e5330314d7a41794c54526d5a4449744f545a685a693077596a67315a4463315a4759794d6d49756347526d&amp;Fich=470e9c65-5302-4fd2-96af-0b85d75df22b.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC155" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AD155" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:57</t>
+        </is>
+      </c>
+      <c r="AE155" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF155" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF138"/>
+  <autoFilter ref="A1:AF155"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14891,7 +16561,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48 UTC</t>
+          <t>2026-10-30 22:57 UTC</t>
         </is>
       </c>
     </row>
@@ -14903,7 +16573,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 19:48 UTC</t>
+          <t>2026-10-30 22:57 UTC</t>
         </is>
       </c>
     </row>
@@ -14914,7 +16584,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>137</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7">
@@ -14924,7 +16594,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>137</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-31 07:31 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Sobre este ficheiro" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Propostas'!$A$1:$AF$164</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF155"/>
+  <dimension ref="A1:AF164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10504,7 +10504,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE96" s="2" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
@@ -10810,7 +10810,7 @@
       </c>
       <c r="AD98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE98" s="2" t="inlineStr">
@@ -10912,7 +10912,7 @@
       </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE99" s="2" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="AD100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE100" s="2" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="AD101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE101" s="2" t="inlineStr">
@@ -11218,7 +11218,7 @@
       </c>
       <c r="AD102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE102" s="2" t="inlineStr">
@@ -11320,7 +11320,7 @@
       </c>
       <c r="AD103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE103" s="2" t="inlineStr">
@@ -11422,7 +11422,7 @@
       </c>
       <c r="AD104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE104" s="2" t="inlineStr">
@@ -11524,7 +11524,7 @@
       </c>
       <c r="AD105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE105" s="2" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="AD106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE106" s="2" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="AD107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE107" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="AD108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE108" s="2" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="AD109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE109" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="AD110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE110" s="2" t="inlineStr">
@@ -12136,7 +12136,7 @@
       </c>
       <c r="AD111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE111" s="2" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="AD112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE112" s="2" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="AD113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE113" s="2" t="inlineStr">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="AD114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE114" s="2" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="AD115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE115" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="AD116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE116" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
       </c>
       <c r="AD117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE117" s="2" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="AD118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE118" s="2" t="inlineStr">
@@ -12920,7 +12920,7 @@
       </c>
       <c r="AD119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE119" s="2" t="inlineStr">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="AD120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE120" s="2" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="AD121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE121" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="AD122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE122" s="2" t="inlineStr">
@@ -13320,7 +13320,7 @@
       </c>
       <c r="AD123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE123" s="2" t="inlineStr">
@@ -13422,7 +13422,7 @@
       </c>
       <c r="AD124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE124" s="2" t="inlineStr">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="AD125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE125" s="2" t="inlineStr">
@@ -13626,7 +13626,7 @@
       </c>
       <c r="AD126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE126" s="2" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="AD127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE127" s="2" t="inlineStr">
@@ -13826,7 +13826,7 @@
       </c>
       <c r="AD128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE128" s="2" t="inlineStr">
@@ -13924,7 +13924,7 @@
       </c>
       <c r="AD129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE129" s="2" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="AD130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE130" s="2" t="inlineStr">
@@ -14120,7 +14120,7 @@
       </c>
       <c r="AD131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE131" s="2" t="inlineStr">
@@ -14222,7 +14222,7 @@
       </c>
       <c r="AD132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE132" s="2" t="inlineStr">
@@ -14320,7 +14320,7 @@
       </c>
       <c r="AD133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE133" s="2" t="inlineStr">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="AD134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE134" s="2" t="inlineStr">
@@ -14520,7 +14520,7 @@
       </c>
       <c r="AD135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE135" s="2" t="inlineStr">
@@ -14618,7 +14618,7 @@
       </c>
       <c r="AD136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE136" s="2" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="AD137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE137" s="2" t="inlineStr">
@@ -14822,7 +14822,7 @@
       </c>
       <c r="AD138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE138" s="2" t="inlineStr">
@@ -14924,7 +14924,7 @@
       </c>
       <c r="AD139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE139" s="2" t="inlineStr">
@@ -15022,7 +15022,7 @@
       </c>
       <c r="AD140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE140" s="2" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="AD141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE141" s="2" t="inlineStr">
@@ -15218,7 +15218,7 @@
       </c>
       <c r="AD142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE142" s="2" t="inlineStr">
@@ -15316,7 +15316,7 @@
       </c>
       <c r="AD143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE143" s="2" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="AD144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE144" s="2" t="inlineStr">
@@ -15512,7 +15512,7 @@
       </c>
       <c r="AD145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE145" s="2" t="inlineStr">
@@ -15610,7 +15610,7 @@
       </c>
       <c r="AD146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE146" s="2" t="inlineStr">
@@ -15708,7 +15708,7 @@
       </c>
       <c r="AD147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE147" s="2" t="inlineStr">
@@ -15806,7 +15806,7 @@
       </c>
       <c r="AD148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE148" s="2" t="inlineStr">
@@ -15904,7 +15904,7 @@
       </c>
       <c r="AD149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE149" s="2" t="inlineStr">
@@ -16002,7 +16002,7 @@
       </c>
       <c r="AD150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE150" s="2" t="inlineStr">
@@ -16100,7 +16100,7 @@
       </c>
       <c r="AD151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE151" s="2" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="AD152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE152" s="2" t="inlineStr">
@@ -16296,7 +16296,7 @@
       </c>
       <c r="AD153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE153" s="2" t="inlineStr">
@@ -16394,7 +16394,7 @@
       </c>
       <c r="AD154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE154" s="2" t="inlineStr">
@@ -16492,7 +16492,7 @@
       </c>
       <c r="AD155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57</t>
+          <t>2026-10-31 07:31</t>
         </is>
       </c>
       <c r="AE155" s="2" t="inlineStr">
@@ -16502,8 +16502,890 @@
       </c>
       <c r="AF155" s="2" t="inlineStr"/>
     </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>155C</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>155C</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr"/>
+      <c r="D156" s="2" t="n">
+        <v>25562</v>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 22:59</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr"/>
+      <c r="K156" s="2" t="inlineStr"/>
+      <c r="L156" s="2" t="inlineStr"/>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N156" s="2" t="inlineStr"/>
+      <c r="O156" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P156" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q156" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R156" s="2" t="inlineStr"/>
+      <c r="S156" s="2" t="inlineStr"/>
+      <c r="T156" s="2" t="inlineStr"/>
+      <c r="U156" s="2" t="inlineStr"/>
+      <c r="V156" s="2" t="inlineStr"/>
+      <c r="W156" s="2" t="inlineStr"/>
+      <c r="X156" s="2" t="inlineStr"/>
+      <c r="Y156" s="2" t="inlineStr"/>
+      <c r="Z156" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA156" s="2" t="inlineStr"/>
+      <c r="AB156" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153383259545a6b5a6d4a694d6930304e44686b4c5451324e545174596a45305a5330344d7a49354e4759784d7a4d334d7a41756347526d&amp;Fich=6a6dfbb2-448d-4654-b14e-83294f133730.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC156" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AD156" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AE156" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF156" s="2" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>156C</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>156C</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr"/>
+      <c r="D157" s="2" t="n">
+        <v>25563</v>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:00</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J157" s="2" t="inlineStr"/>
+      <c r="K157" s="2" t="inlineStr"/>
+      <c r="L157" s="2" t="inlineStr"/>
+      <c r="M157" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N157" s="2" t="inlineStr"/>
+      <c r="O157" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P157" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q157" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R157" s="2" t="inlineStr"/>
+      <c r="S157" s="2" t="inlineStr"/>
+      <c r="T157" s="2" t="inlineStr"/>
+      <c r="U157" s="2" t="inlineStr"/>
+      <c r="V157" s="2" t="inlineStr"/>
+      <c r="W157" s="2" t="inlineStr"/>
+      <c r="X157" s="2" t="inlineStr"/>
+      <c r="Y157" s="2" t="inlineStr"/>
+      <c r="Z157" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA157" s="2" t="inlineStr"/>
+      <c r="AB157" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396c5a54526b4e546b775a69303359574e6c4c5451354d544d74596a4e6a4e4330354d4459335a4451335a47557a596a41756347526d&amp;Fich=ee4d590f-7ace-4913-b3c4-9067d47de3b0.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC157" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AD157" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AE157" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF157" s="2" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>157C</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>157C</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr"/>
+      <c r="D158" s="2" t="n">
+        <v>25564</v>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:01</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J158" s="2" t="inlineStr"/>
+      <c r="K158" s="2" t="inlineStr"/>
+      <c r="L158" s="2" t="inlineStr"/>
+      <c r="M158" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N158" s="2" t="inlineStr"/>
+      <c r="O158" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P158" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q158" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R158" s="2" t="inlineStr"/>
+      <c r="S158" s="2" t="inlineStr"/>
+      <c r="T158" s="2" t="inlineStr"/>
+      <c r="U158" s="2" t="inlineStr"/>
+      <c r="V158" s="2" t="inlineStr"/>
+      <c r="W158" s="2" t="inlineStr"/>
+      <c r="X158" s="2" t="inlineStr"/>
+      <c r="Y158" s="2" t="inlineStr"/>
+      <c r="Z158" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA158" s="2" t="inlineStr"/>
+      <c r="AB158" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324e474e685a44566a4d53316b4d54566d4c5451794d545974596a646c4e4330784d7a56685a574979595745345a6a51756347526d&amp;Fich=64cad5c1-d15f-4216-b7e4-135aeb2aa8f4.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC158" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AD158" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AE158" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF158" s="2" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>158C</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>158C</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr"/>
+      <c r="D159" s="2" t="n">
+        <v>25565</v>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:02</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="inlineStr"/>
+      <c r="K159" s="2" t="inlineStr"/>
+      <c r="L159" s="2" t="inlineStr"/>
+      <c r="M159" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N159" s="2" t="inlineStr"/>
+      <c r="O159" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P159" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q159" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R159" s="2" t="inlineStr"/>
+      <c r="S159" s="2" t="inlineStr"/>
+      <c r="T159" s="2" t="inlineStr"/>
+      <c r="U159" s="2" t="inlineStr"/>
+      <c r="V159" s="2" t="inlineStr"/>
+      <c r="W159" s="2" t="inlineStr"/>
+      <c r="X159" s="2" t="inlineStr"/>
+      <c r="Y159" s="2" t="inlineStr"/>
+      <c r="Z159" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA159" s="2" t="inlineStr"/>
+      <c r="AB159" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338345a6a63354f546378596930794e6a56694c5451355a6a5174596d49304d43316d5a6a51794d324a6c596a526b5a6d4d756347526d&amp;Fich=8f79971b-265b-49f4-bb40-ff423beb4dfc.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC159" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AD159" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AE159" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF159" s="2" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>159C</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>159C</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr"/>
+      <c r="D160" s="2" t="n">
+        <v>25566</v>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:03</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J160" s="2" t="inlineStr"/>
+      <c r="K160" s="2" t="inlineStr"/>
+      <c r="L160" s="2" t="inlineStr"/>
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N160" s="2" t="inlineStr"/>
+      <c r="O160" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P160" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q160" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R160" s="2" t="inlineStr"/>
+      <c r="S160" s="2" t="inlineStr"/>
+      <c r="T160" s="2" t="inlineStr"/>
+      <c r="U160" s="2" t="inlineStr"/>
+      <c r="V160" s="2" t="inlineStr"/>
+      <c r="W160" s="2" t="inlineStr"/>
+      <c r="X160" s="2" t="inlineStr"/>
+      <c r="Y160" s="2" t="inlineStr"/>
+      <c r="Z160" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA160" s="2" t="inlineStr"/>
+      <c r="AB160" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515339694d4759794e574d785a6930315a444e6b4c54526a4e6a6b745954686d4d4330775a47466b5932566c4e6d466d596a55756347526d&amp;Fich=b0f25c1f-5d3d-4c69-a8f0-0dadcee6afb5.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC160" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AD160" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AE160" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF160" s="2" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>160C</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>160C</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr"/>
+      <c r="D161" s="2" t="n">
+        <v>25567</v>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:05</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I161" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J161" s="2" t="inlineStr"/>
+      <c r="K161" s="2" t="inlineStr"/>
+      <c r="L161" s="2" t="inlineStr"/>
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N161" s="2" t="inlineStr"/>
+      <c r="O161" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P161" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q161" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R161" s="2" t="inlineStr"/>
+      <c r="S161" s="2" t="inlineStr"/>
+      <c r="T161" s="2" t="inlineStr"/>
+      <c r="U161" s="2" t="inlineStr"/>
+      <c r="V161" s="2" t="inlineStr"/>
+      <c r="W161" s="2" t="inlineStr"/>
+      <c r="X161" s="2" t="inlineStr"/>
+      <c r="Y161" s="2" t="inlineStr"/>
+      <c r="Z161" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA161" s="2" t="inlineStr"/>
+      <c r="AB161" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338324e6a55784d7a6c6c4e69316c4d4459344c5451784d57517459544a694e693033597a566b4d6a677a4d6a56694d4445756347526d&amp;Fich=665139e6-e068-411d-a2b6-7c5d28325b01.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC161" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AD161" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AE161" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF161" s="2" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>161C</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>161C</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr"/>
+      <c r="D162" s="2" t="n">
+        <v>25568</v>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:06</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J162" s="2" t="inlineStr"/>
+      <c r="K162" s="2" t="inlineStr"/>
+      <c r="L162" s="2" t="inlineStr"/>
+      <c r="M162" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N162" s="2" t="inlineStr"/>
+      <c r="O162" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P162" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q162" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R162" s="2" t="inlineStr"/>
+      <c r="S162" s="2" t="inlineStr"/>
+      <c r="T162" s="2" t="inlineStr"/>
+      <c r="U162" s="2" t="inlineStr"/>
+      <c r="V162" s="2" t="inlineStr"/>
+      <c r="W162" s="2" t="inlineStr"/>
+      <c r="X162" s="2" t="inlineStr"/>
+      <c r="Y162" s="2" t="inlineStr"/>
+      <c r="Z162" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA162" s="2" t="inlineStr"/>
+      <c r="AB162" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f4339515153396d59574a6d4f4749344e69316d4d5455354c54517a5a5459744f4459325a5330314d5467305954526a4e44646d5a4749756347526d&amp;Fich=fabf8b86-f159-43e6-866e-5184a4c47fdb.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC162" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AD162" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AE162" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF162" s="2" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>162C</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>162C</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr"/>
+      <c r="D163" s="2" t="n">
+        <v>25569</v>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:07</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr"/>
+      <c r="K163" s="2" t="inlineStr"/>
+      <c r="L163" s="2" t="inlineStr"/>
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N163" s="2" t="inlineStr"/>
+      <c r="O163" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P163" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q163" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R163" s="2" t="inlineStr"/>
+      <c r="S163" s="2" t="inlineStr"/>
+      <c r="T163" s="2" t="inlineStr"/>
+      <c r="U163" s="2" t="inlineStr"/>
+      <c r="V163" s="2" t="inlineStr"/>
+      <c r="W163" s="2" t="inlineStr"/>
+      <c r="X163" s="2" t="inlineStr"/>
+      <c r="Y163" s="2" t="inlineStr"/>
+      <c r="Z163" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA163" s="2" t="inlineStr"/>
+      <c r="AB163" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f433951515338784d4456684e6d4d324f53316c597a6c6b4c5452684d7a4174596a5a6b596931684e4752694e544a68597a45314d4459756347526d&amp;Fich=105a6c69-ec9d-4a30-b6db-a4db52ac1506.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC163" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AD163" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AE163" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF163" s="2" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>163C</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>163C</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr"/>
+      <c r="D164" s="2" t="n">
+        <v>25570</v>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:08</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr">
+        <is>
+          <t>PCP</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>Alfredo Maia; Paula Santos; Paulo Raimundo</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>Comissão</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t>Articulado</t>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr"/>
+      <c r="K164" s="2" t="inlineStr"/>
+      <c r="L164" s="2" t="inlineStr"/>
+      <c r="M164" s="2" t="inlineStr">
+        <is>
+          <t>Por Definir</t>
+        </is>
+      </c>
+      <c r="N164" s="2" t="inlineStr"/>
+      <c r="O164" s="2" t="inlineStr">
+        <is>
+          <t>Assuntos Constitucionais, Direitos, Liberdades e Garantias</t>
+        </is>
+      </c>
+      <c r="P164" s="2" t="inlineStr">
+        <is>
+          <t>em apreciação</t>
+        </is>
+      </c>
+      <c r="Q164" s="2" t="inlineStr">
+        <is>
+          <t>Entrada (via IPA)</t>
+        </is>
+      </c>
+      <c r="R164" s="2" t="inlineStr"/>
+      <c r="S164" s="2" t="inlineStr"/>
+      <c r="T164" s="2" t="inlineStr"/>
+      <c r="U164" s="2" t="inlineStr"/>
+      <c r="V164" s="2" t="inlineStr"/>
+      <c r="W164" s="2" t="inlineStr"/>
+      <c r="X164" s="2" t="inlineStr"/>
+      <c r="Y164" s="2" t="inlineStr"/>
+      <c r="Z164" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA164" s="2" t="inlineStr"/>
+      <c r="AB164" s="2" t="inlineStr">
+        <is>
+          <t>https://app.parlamento.pt/webutils/docs/doc.pdf?path=6148523063484d364c793942556b356c6443397a6158526c63793959566b6c4a544556484c3039464c7a49774d6a63794d4449324d5441774f43395151533878593245314e7a64684e5331684e44457a4c5451314e546774595449344d43316c4e57557a5a574a6b4f446b354e6a59756347526d&amp;Fich=1ca577a5-a413-4558-a280-e5e3ebd89966.pdf&amp;Inline=true</t>
+        </is>
+      </c>
+      <c r="AC164" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AD164" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:31</t>
+        </is>
+      </c>
+      <c r="AE164" s="2" t="inlineStr">
+        <is>
+          <t>opendata</t>
+        </is>
+      </c>
+      <c r="AF164" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AF155"/>
+  <autoFilter ref="A1:AF164"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16561,7 +17443,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57 UTC</t>
+          <t>2026-10-31 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -16573,7 +17455,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30 22:57 UTC</t>
+          <t>2026-10-31 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -16584,7 +17466,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>154</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7">
@@ -16594,7 +17476,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>154</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
captura 2026-10-31 13:37 UTC
</commit_message>
<xml_diff>
--- a/docs/PA_OE2027_dados_AR.xlsx
+++ b/docs/PA_OE2027_dados_AR.xlsx
@@ -750,7 +750,7 @@
       </c>
       <c r="AD2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE2" s="2" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="AD8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE8" s="2" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="AD9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE9" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="AD10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE10" s="2" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="AD11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE11" s="2" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="AD12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE12" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="AD13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE13" s="2" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AD14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE14" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="AD15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE15" s="2" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="AD16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE16" s="2" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="AD17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE17" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="AD18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE18" s="2" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="AD19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE19" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       </c>
       <c r="AD20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE20" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="AD21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE21" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="AD22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE22" s="2" t="inlineStr">
@@ -2944,7 +2944,7 @@
       </c>
       <c r="AD23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE23" s="2" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="AD24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE24" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="AD25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE25" s="2" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="AD26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE26" s="2" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="AD27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE27" s="2" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="AD28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE28" s="2" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="AD29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE29" s="2" t="inlineStr">
@@ -3662,7 +3662,7 @@
       </c>
       <c r="AD30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE30" s="2" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="AD31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE31" s="2" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="AD32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE32" s="2" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="AD33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE33" s="2" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="AD34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE34" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="AD35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE35" s="2" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="AD36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE36" s="2" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="AD38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE38" s="2" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="AD39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE39" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="AD40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE40" s="2" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="AD41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE41" s="2" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="AD42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE42" s="2" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="AD43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE43" s="2" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -5240,7 +5240,7 @@
       </c>
       <c r="AD45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE45" s="2" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="AD46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE46" s="2" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="AD47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE47" s="2" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="AD48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE48" s="2" t="inlineStr">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="AD49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE49" s="2" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="AD50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE50" s="2" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="AD52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE52" s="2" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="AD53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE53" s="2" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="AD54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE54" s="2" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="AD55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE55" s="2" t="inlineStr">
@@ -6390,7 +6390,7 @@
       </c>
       <c r="AD56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE56" s="2" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="AD57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE57" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="AD58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE58" s="2" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="AD59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE59" s="2" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="AD60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE60" s="2" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="AD61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE61" s="2" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="AD62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE62" s="2" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="AD63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE63" s="2" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="AD64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE64" s="2" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="AD65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE65" s="2" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="AD66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE66" s="2" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="AD67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE67" s="2" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="AD68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE68" s="2" t="inlineStr">
@@ -7772,7 +7772,7 @@
       </c>
       <c r="AD69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE69" s="2" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="AD70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE70" s="2" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="AD71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE71" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AD72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE72" s="2" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="AD73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE73" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="AD74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE74" s="2" t="inlineStr">
@@ -8392,7 +8392,7 @@
       </c>
       <c r="AD75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE75" s="2" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="AD76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE76" s="2" t="inlineStr">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="AD77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE77" s="2" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="AD78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE78" s="2" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="AD79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE79" s="2" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="AD80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE80" s="2" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="AD81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE81" s="2" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AD82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE82" s="2" t="inlineStr">
@@ -9240,7 +9240,7 @@
       </c>
       <c r="AD83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE83" s="2" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="AD84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE84" s="2" t="inlineStr">
@@ -9448,7 +9448,7 @@
       </c>
       <c r="AD85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE85" s="2" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="AD86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE86" s="2" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="AD87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE87" s="2" t="inlineStr">
@@ -9766,7 +9766,7 @@
       </c>
       <c r="AD88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE88" s="2" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="AD89" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE89" s="2" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="AD90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE90" s="2" t="inlineStr">
@@ -10084,7 +10084,7 @@
       </c>
       <c r="AD91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE91" s="2" t="inlineStr">
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AD92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE92" s="2" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="AD93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE93" s="2" t="inlineStr">
@@ -10402,7 +10402,7 @@
       </c>
       <c r="AD94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE94" s="2" t="inlineStr">
@@ -10504,7 +10504,7 @@
       </c>
       <c r="AD95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE95" s="2" t="inlineStr">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="AD96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE96" s="2" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="AD97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE97" s="2" t="inlineStr">
@@ -10810,7 +10810,7 @@
       </c>
       <c r="AD98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE98" s="2" t="inlineStr">
@@ -10912,7 +10912,7 @@
       </c>
       <c r="AD99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE99" s="2" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="AD100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE100" s="2" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="AD101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE101" s="2" t="inlineStr">
@@ -11218,7 +11218,7 @@
       </c>
       <c r="AD102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE102" s="2" t="inlineStr">
@@ -11320,7 +11320,7 @@
       </c>
       <c r="AD103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE103" s="2" t="inlineStr">
@@ -11422,7 +11422,7 @@
       </c>
       <c r="AD104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE104" s="2" t="inlineStr">
@@ -11524,7 +11524,7 @@
       </c>
       <c r="AD105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE105" s="2" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="AD106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE106" s="2" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="AD107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE107" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="AD108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE108" s="2" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="AD109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE109" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="AD110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE110" s="2" t="inlineStr">
@@ -12136,7 +12136,7 @@
       </c>
       <c r="AD111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE111" s="2" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="AD112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE112" s="2" t="inlineStr">
@@ -12332,7 +12332,7 @@
       </c>
       <c r="AD113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE113" s="2" t="inlineStr">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="AD114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE114" s="2" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="AD115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE115" s="2" t="inlineStr">
@@ -12626,7 +12626,7 @@
       </c>
       <c r="AD116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE116" s="2" t="inlineStr">
@@ -12724,7 +12724,7 @@
       </c>
       <c r="AD117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE117" s="2" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="AD118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE118" s="2" t="inlineStr">
@@ -12920,7 +12920,7 @@
       </c>
       <c r="AD119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE119" s="2" t="inlineStr">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="AD120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE120" s="2" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="AD121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE121" s="2" t="inlineStr">
@@ -13218,7 +13218,7 @@
       </c>
       <c r="AD122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE122" s="2" t="inlineStr">
@@ -13320,7 +13320,7 @@
       </c>
       <c r="AD123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE123" s="2" t="inlineStr">
@@ -13422,7 +13422,7 @@
       </c>
       <c r="AD124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE124" s="2" t="inlineStr">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="AD125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE125" s="2" t="inlineStr">
@@ -13626,7 +13626,7 @@
       </c>
       <c r="AD126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE126" s="2" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="AD127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE127" s="2" t="inlineStr">
@@ -13826,7 +13826,7 @@
       </c>
       <c r="AD128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE128" s="2" t="inlineStr">
@@ -13924,7 +13924,7 @@
       </c>
       <c r="AD129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE129" s="2" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="AD130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE130" s="2" t="inlineStr">
@@ -14120,7 +14120,7 @@
       </c>
       <c r="AD131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE131" s="2" t="inlineStr">
@@ -14222,7 +14222,7 @@
       </c>
       <c r="AD132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE132" s="2" t="inlineStr">
@@ -14320,7 +14320,7 @@
       </c>
       <c r="AD133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE133" s="2" t="inlineStr">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="AD134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE134" s="2" t="inlineStr">
@@ -14520,7 +14520,7 @@
       </c>
       <c r="AD135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE135" s="2" t="inlineStr">
@@ -14618,7 +14618,7 @@
       </c>
       <c r="AD136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE136" s="2" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="AD137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE137" s="2" t="inlineStr">
@@ -14822,7 +14822,7 @@
       </c>
       <c r="AD138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE138" s="2" t="inlineStr">
@@ -14924,7 +14924,7 @@
       </c>
       <c r="AD139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE139" s="2" t="inlineStr">
@@ -15022,7 +15022,7 @@
       </c>
       <c r="AD140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE140" s="2" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="AD141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE141" s="2" t="inlineStr">
@@ -15218,7 +15218,7 @@
       </c>
       <c r="AD142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE142" s="2" t="inlineStr">
@@ -15316,7 +15316,7 @@
       </c>
       <c r="AD143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE143" s="2" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="AD144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE144" s="2" t="inlineStr">
@@ -15512,7 +15512,7 @@
       </c>
       <c r="AD145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE145" s="2" t="inlineStr">
@@ -15610,7 +15610,7 @@
       </c>
       <c r="AD146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE146" s="2" t="inlineStr">
@@ -15708,7 +15708,7 @@
       </c>
       <c r="AD147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE147" s="2" t="inlineStr">
@@ -15806,7 +15806,7 @@
       </c>
       <c r="AD148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE148" s="2" t="inlineStr">
@@ -15904,7 +15904,7 @@
       </c>
       <c r="AD149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE149" s="2" t="inlineStr">
@@ -16002,7 +16002,7 @@
       </c>
       <c r="AD150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE150" s="2" t="inlineStr">
@@ -16100,7 +16100,7 @@
       </c>
       <c r="AD151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE151" s="2" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="AD152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE152" s="2" t="inlineStr">
@@ -16296,7 +16296,7 @@
       </c>
       <c r="AD153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE153" s="2" t="inlineStr">
@@ -16394,7 +16394,7 @@
       </c>
       <c r="AD154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE154" s="2" t="inlineStr">
@@ -16492,7 +16492,7 @@
       </c>
       <c r="AD155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE155" s="2" t="inlineStr">
@@ -16590,7 +16590,7 @@
       </c>
       <c r="AD156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE156" s="2" t="inlineStr">
@@ -16688,7 +16688,7 @@
       </c>
       <c r="AD157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE157" s="2" t="inlineStr">
@@ -16786,7 +16786,7 @@
       </c>
       <c r="AD158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE158" s="2" t="inlineStr">
@@ -16884,7 +16884,7 @@
       </c>
       <c r="AD159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE159" s="2" t="inlineStr">
@@ -16982,7 +16982,7 @@
       </c>
       <c r="AD160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE160" s="2" t="inlineStr">
@@ -17080,7 +17080,7 @@
       </c>
       <c r="AD161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE161" s="2" t="inlineStr">
@@ -17178,7 +17178,7 @@
       </c>
       <c r="AD162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE162" s="2" t="inlineStr">
@@ -17276,7 +17276,7 @@
       </c>
       <c r="AD163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE163" s="2" t="inlineStr">
@@ -17374,7 +17374,7 @@
       </c>
       <c r="AD164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31</t>
+          <t>2026-10-31 13:37</t>
         </is>
       </c>
       <c r="AE164" s="2" t="inlineStr">
@@ -17443,7 +17443,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31 UTC</t>
+          <t>2026-10-31 13:37 UTC</t>
         </is>
       </c>
     </row>
@@ -17455,7 +17455,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-31 07:31 UTC</t>
+          <t>2026-10-31 13:37 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>